<commit_message>
Add YBBN flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E76D82D-9264-40C5-8B19-53311331E6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705A2FFF-2D4A-4F71-88ED-805567D24B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="8835" windowHeight="20985" firstSheet="3" activeTab="4" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
     <sheet name="YSSY" sheetId="10" r:id="rId2"/>
     <sheet name="YMHB" sheetId="11" r:id="rId3"/>
     <sheet name="YMLT" sheetId="12" r:id="rId4"/>
+    <sheet name="YBBN" sheetId="13" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
   <si>
     <t>-</t>
   </si>
@@ -294,6 +295,123 @@
   </si>
   <si>
     <t>LATUM MLTND</t>
+  </si>
+  <si>
+    <t>RWY 01L</t>
+  </si>
+  <si>
+    <t>RWY 01R</t>
+  </si>
+  <si>
+    <t>RWY 19L</t>
+  </si>
+  <si>
+    <t>RWY 19R</t>
+  </si>
+  <si>
+    <t>BLAKA A</t>
+  </si>
+  <si>
+    <t>BLAKA X</t>
+  </si>
+  <si>
+    <t>ENLIP A</t>
+  </si>
+  <si>
+    <t>ENLIP X</t>
+  </si>
+  <si>
+    <t>GOMOL A</t>
+  </si>
+  <si>
+    <t>GOMOL V</t>
+  </si>
+  <si>
+    <t>GOMOL X</t>
+  </si>
+  <si>
+    <t>MORBI A</t>
+  </si>
+  <si>
+    <t>MORBI V</t>
+  </si>
+  <si>
+    <t>SMOKA A</t>
+  </si>
+  <si>
+    <t>SMOKA M</t>
+  </si>
+  <si>
+    <t>SMOKA X</t>
+  </si>
+  <si>
+    <t>TEBOT A</t>
+  </si>
+  <si>
+    <t>TEBOT X</t>
+  </si>
+  <si>
+    <t>UGTUG A</t>
+  </si>
+  <si>
+    <t>UGTUG X</t>
+  </si>
+  <si>
+    <t>WOODY A</t>
+  </si>
+  <si>
+    <t>WOODY V</t>
+  </si>
+  <si>
+    <t>Runway 01L</t>
+  </si>
+  <si>
+    <t>Runway 01R</t>
+  </si>
+  <si>
+    <t>Runway 19L</t>
+  </si>
+  <si>
+    <t>Runway 19R</t>
+  </si>
+  <si>
+    <t>RNP X (RUSVA)</t>
+  </si>
+  <si>
+    <t>LOC (TANIK)</t>
+  </si>
+  <si>
+    <t>RNP X (SORVA)</t>
+  </si>
+  <si>
+    <t>LOC (GLENN)</t>
+  </si>
+  <si>
+    <t>RNP X (ATSEP)</t>
+  </si>
+  <si>
+    <t>LOC (BETSO)</t>
+  </si>
+  <si>
+    <t>RNP X (LUVNA)</t>
+  </si>
+  <si>
+    <t>LOC (OSOKO)</t>
+  </si>
+  <si>
+    <t>ISPON (ENLIP trans)</t>
+  </si>
+  <si>
+    <t>ISPON (BLAKA trans)</t>
+  </si>
+  <si>
+    <t>ISPON (GOMOL trans)</t>
+  </si>
+  <si>
+    <t>ISPON (UGTUG trans)</t>
+  </si>
+  <si>
+    <t>RNP M (BIPUD)</t>
   </si>
 </sst>
 </file>
@@ -317,7 +435,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -345,6 +463,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -413,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -453,6 +577,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1818,4 +1948,604 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
+  <dimension ref="A2:F40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="5">
+        <v>55.5</v>
+      </c>
+      <c r="D4" s="5">
+        <v>54.7</v>
+      </c>
+      <c r="E4" s="5">
+        <v>87.5</v>
+      </c>
+      <c r="F4" s="5">
+        <v>98.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5">
+        <v>50.5</v>
+      </c>
+      <c r="E5" s="5">
+        <v>68.8</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="5">
+        <v>44.5</v>
+      </c>
+      <c r="D6" s="5">
+        <v>44.7</v>
+      </c>
+      <c r="E6" s="5">
+        <v>91.5</v>
+      </c>
+      <c r="F6" s="5">
+        <v>81.400000000000006</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>72.8</v>
+      </c>
+      <c r="F7" s="5">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="5">
+        <v>58.5</v>
+      </c>
+      <c r="D8" s="5">
+        <v>57.7</v>
+      </c>
+      <c r="E8" s="5">
+        <v>83.5</v>
+      </c>
+      <c r="F8" s="5">
+        <v>93.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5">
+        <v>52.6</v>
+      </c>
+      <c r="E9" s="5">
+        <v>66.099999999999994</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>50.5</v>
+      </c>
+      <c r="E10" s="5">
+        <v>67.8</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>92.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>88.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>84.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>57.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="5">
+        <v>70.5</v>
+      </c>
+      <c r="D15" s="5">
+        <v>65.7</v>
+      </c>
+      <c r="E15" s="5">
+        <v>51.5</v>
+      </c>
+      <c r="F15" s="5">
+        <v>50.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="5">
+        <v>51.3</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>41.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="5">
+        <v>64.5</v>
+      </c>
+      <c r="D17" s="5">
+        <v>61.7</v>
+      </c>
+      <c r="E17" s="5">
+        <v>54.5</v>
+      </c>
+      <c r="F17" s="5">
+        <v>53.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
+        <v>47.6</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="5">
+        <v>51.5</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="5">
+        <v>81.5</v>
+      </c>
+      <c r="D20" s="5">
+        <v>82.7</v>
+      </c>
+      <c r="E20" s="5">
+        <v>43.5</v>
+      </c>
+      <c r="F20" s="5">
+        <v>45.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <v>67.5</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="5">
+        <v>65.5</v>
+      </c>
+      <c r="D22" s="5">
+        <v>66.7</v>
+      </c>
+      <c r="E22" s="5">
+        <v>56.5</v>
+      </c>
+      <c r="F22" s="5">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>51.5</v>
+      </c>
+      <c r="E23" s="5">
+        <v>46.8</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="5">
+        <v>59.5</v>
+      </c>
+      <c r="D24" s="5">
+        <v>56.7</v>
+      </c>
+      <c r="E24" s="5">
+        <v>63.5</v>
+      </c>
+      <c r="F24" s="5">
+        <v>62.4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="5">
+        <v>44.3</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <v>49.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="18"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="6">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C30" s="6">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32" s="7">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="12"/>
+      <c r="B33" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="7">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="12"/>
+      <c r="B34" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="7">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="8"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" s="22">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="19"/>
+      <c r="B37" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C37" s="22">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="8"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C39" s="5">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C40" s="5">
+        <v>11.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add YBCG flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705A2FFF-2D4A-4F71-88ED-805567D24B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A906D408-5C02-4358-B94D-489D4B3759B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="8835" windowHeight="20985" firstSheet="3" activeTab="4" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="9510" windowHeight="20985" activeTab="5" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="YMHB" sheetId="11" r:id="rId3"/>
     <sheet name="YMLT" sheetId="12" r:id="rId4"/>
     <sheet name="YBBN" sheetId="13" r:id="rId5"/>
+    <sheet name="YBCG" sheetId="14" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="142">
   <si>
     <t>-</t>
   </si>
@@ -412,6 +413,66 @@
   </si>
   <si>
     <t>RNP M (BIPUD)</t>
+  </si>
+  <si>
+    <t>Arrival</t>
+  </si>
+  <si>
+    <t>RWY 14</t>
+  </si>
+  <si>
+    <t>RWY 32</t>
+  </si>
+  <si>
+    <t>Runway 14</t>
+  </si>
+  <si>
+    <t>Runway 32</t>
+  </si>
+  <si>
+    <t>RNP Z (CG2NC)</t>
+  </si>
+  <si>
+    <t>RNP Z (KEGAN)</t>
+  </si>
+  <si>
+    <t>RNP Y (KERRI)</t>
+  </si>
+  <si>
+    <t>RNP W (VAPMU)</t>
+  </si>
+  <si>
+    <t>LOC (IRPOD)</t>
+  </si>
+  <si>
+    <t>RNP Z (FIKUL)</t>
+  </si>
+  <si>
+    <t>RNP Z (CG2SA)</t>
+  </si>
+  <si>
+    <t>LAMSI A STAR</t>
+  </si>
+  <si>
+    <t>BERNI Y STAR</t>
+  </si>
+  <si>
+    <t>BERNI V STAR</t>
+  </si>
+  <si>
+    <t>BERNI A STAR</t>
+  </si>
+  <si>
+    <t>LAMSI Y STAR</t>
+  </si>
+  <si>
+    <t>BN Y177 IDRIL CG2SA</t>
+  </si>
+  <si>
+    <t>BN Y177 IDRIL CG2NC</t>
+  </si>
+  <si>
+    <t>RNP Y (ATKEN)</t>
   </si>
 </sst>
 </file>
@@ -564,6 +625,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -577,12 +644,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -927,13 +988,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1172,11 +1233,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -1278,16 +1339,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1338,16 +1399,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -1374,14 +1435,14 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -1488,11 +1549,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -1580,12 +1641,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1700,11 +1761,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -1770,12 +1831,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1890,11 +1951,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -1963,14 +2024,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2431,11 +2492,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2497,22 +2558,22 @@
       <c r="C35" s="8"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="22">
+      <c r="C36" s="17">
         <v>12.8</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="19"/>
-      <c r="B37" s="20" t="s">
+      <c r="A37" s="14"/>
+      <c r="B37" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="C37" s="22">
+      <c r="C37" s="17">
         <v>14.5</v>
       </c>
     </row>
@@ -2522,7 +2583,7 @@
       <c r="C38" s="8"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
       <c r="B39" s="2" t="s">
@@ -2548,4 +2609,231 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
+  <dimension ref="A2:D37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="5">
+        <v>66.8</v>
+      </c>
+      <c r="D4" s="5">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="5">
+        <v>58.4</v>
+      </c>
+      <c r="D5" s="5">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="5">
+        <v>59.7</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="5">
+        <v>55.8</v>
+      </c>
+      <c r="D7" s="5">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" s="5">
+        <v>49.7</v>
+      </c>
+      <c r="D8" s="5">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5">
+        <v>68.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="5">
+        <v>47.4</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="6">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="6">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="6">
+        <v>14.7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C33" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="7">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="12"/>
+      <c r="B36" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" s="7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="12"/>
+      <c r="B37" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="7">
+        <v>10.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add YPDN flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A906D408-5C02-4358-B94D-489D4B3759B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1985BEB-30A2-4A83-813B-DEFEA65D3B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="9510" windowHeight="20985" activeTab="5" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="9180" windowHeight="20985" activeTab="6" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="YMLT" sheetId="12" r:id="rId4"/>
     <sheet name="YBBN" sheetId="13" r:id="rId5"/>
     <sheet name="YBCG" sheetId="14" r:id="rId6"/>
+    <sheet name="YPDN" sheetId="15" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="159">
   <si>
     <t>-</t>
   </si>
@@ -473,6 +474,57 @@
   </si>
   <si>
     <t>RNP Y (ATKEN)</t>
+  </si>
+  <si>
+    <t>Runway 11</t>
+  </si>
+  <si>
+    <t>Runway 29</t>
+  </si>
+  <si>
+    <t>RNP Z (All)</t>
+  </si>
+  <si>
+    <t>RNP X (NASUX)</t>
+  </si>
+  <si>
+    <t>RNP W (WOKKI)</t>
+  </si>
+  <si>
+    <t>RNP W (KITTY)</t>
+  </si>
+  <si>
+    <t>RNP W (UPSEN)</t>
+  </si>
+  <si>
+    <t>RNP Z (DRWEB)</t>
+  </si>
+  <si>
+    <t>LOC (LAPAR)</t>
+  </si>
+  <si>
+    <t>ANUPA A/X</t>
+  </si>
+  <si>
+    <t>GATOR A/X</t>
+  </si>
+  <si>
+    <t>RWY 11</t>
+  </si>
+  <si>
+    <t>RWY 29</t>
+  </si>
+  <si>
+    <t>VEGPU A/X</t>
+  </si>
+  <si>
+    <t>VEGPU W</t>
+  </si>
+  <si>
+    <t>WANGI W</t>
+  </si>
+  <si>
+    <t>WANGI A/X</t>
   </si>
 </sst>
 </file>
@@ -2836,4 +2888,226 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
+  <dimension ref="A2:D38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C4" s="5">
+        <v>48.4</v>
+      </c>
+      <c r="D4" s="5">
+        <v>82.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C5" s="5">
+        <v>75.400000000000006</v>
+      </c>
+      <c r="D5" s="5">
+        <v>52.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C6" s="5">
+        <v>55.4</v>
+      </c>
+      <c r="D6" s="5">
+        <v>26.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" s="5">
+        <v>45.4</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C8" s="5">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="D8" s="5">
+        <v>74.400000000000006</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="5">
+        <v>58.9</v>
+      </c>
+      <c r="D9" s="5">
+        <v>65.400000000000006</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C29" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="6">
+        <v>19.100000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" s="6">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="6">
+        <v>18.899999999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C35" s="7">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="12"/>
+      <c r="B36" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C36" s="7">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="12"/>
+      <c r="B37" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C37" s="7">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="12"/>
+      <c r="B38" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C38" s="7">
+        <v>20.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add YPPH flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1985BEB-30A2-4A83-813B-DEFEA65D3B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C42C46-C15D-43D1-B842-3D8F1233B84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="9180" windowHeight="20985" activeTab="6" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="YBBN" sheetId="13" r:id="rId5"/>
     <sheet name="YBCG" sheetId="14" r:id="rId6"/>
     <sheet name="YPDN" sheetId="15" r:id="rId7"/>
+    <sheet name="YPPH" sheetId="16" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="193">
   <si>
     <t>-</t>
   </si>
@@ -525,6 +526,108 @@
   </si>
   <si>
     <t>WANGI A/X</t>
+  </si>
+  <si>
+    <t>RWY 03</t>
+  </si>
+  <si>
+    <t>RWY 06</t>
+  </si>
+  <si>
+    <t>RWY 21</t>
+  </si>
+  <si>
+    <t>RWY 24</t>
+  </si>
+  <si>
+    <t>Runway 03</t>
+  </si>
+  <si>
+    <t>Runway 06</t>
+  </si>
+  <si>
+    <t>Runway 21</t>
+  </si>
+  <si>
+    <t>Runway 24</t>
+  </si>
+  <si>
+    <t>RNP X (KARGO)</t>
+  </si>
+  <si>
+    <t>LOC (BITUM)</t>
+  </si>
+  <si>
+    <t>RNP Z (LENNY)</t>
+  </si>
+  <si>
+    <t>LOC (HAIGH)</t>
+  </si>
+  <si>
+    <t>LOC (KOORI)</t>
+  </si>
+  <si>
+    <t>DAYLR A</t>
+  </si>
+  <si>
+    <t>DAYLR V</t>
+  </si>
+  <si>
+    <t>DAYLR X</t>
+  </si>
+  <si>
+    <t>IPMOR A</t>
+  </si>
+  <si>
+    <t>LOC (WOOFY arc)</t>
+  </si>
+  <si>
+    <t>LOC (KOORI arc)</t>
+  </si>
+  <si>
+    <t>JULIM A</t>
+  </si>
+  <si>
+    <t>JULIM V</t>
+  </si>
+  <si>
+    <t>JULIM X</t>
+  </si>
+  <si>
+    <t>KABLI A</t>
+  </si>
+  <si>
+    <t>KABLI V</t>
+  </si>
+  <si>
+    <t>KABLI X</t>
+  </si>
+  <si>
+    <t>LAVEX A</t>
+  </si>
+  <si>
+    <t>LAVEX V</t>
+  </si>
+  <si>
+    <t>LAVEX X</t>
+  </si>
+  <si>
+    <t>SAPKO A</t>
+  </si>
+  <si>
+    <t>SAPKO V</t>
+  </si>
+  <si>
+    <t>SAPKO X</t>
+  </si>
+  <si>
+    <t>SOLUS A</t>
+  </si>
+  <si>
+    <t>SOLUS V</t>
+  </si>
+  <si>
+    <t>SOLUS X</t>
   </si>
 </sst>
 </file>
@@ -2913,7 +3016,7 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
-        <v>122</v>
+        <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>153</v>
@@ -3110,4 +3213,526 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
+  <dimension ref="A2:F38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="6">
+        <v>47</v>
+      </c>
+      <c r="D4" s="6">
+        <v>55.2</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" s="6">
+        <v>40</v>
+      </c>
+      <c r="D5" s="6">
+        <v>44</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="6">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C7" s="5">
+        <v>74</v>
+      </c>
+      <c r="D7" s="5">
+        <v>58.2</v>
+      </c>
+      <c r="E7" s="5">
+        <v>64.3</v>
+      </c>
+      <c r="F7" s="5">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C8" s="7">
+        <v>78.599999999999994</v>
+      </c>
+      <c r="D8" s="7">
+        <v>86.8</v>
+      </c>
+      <c r="E8" s="7">
+        <v>37.1</v>
+      </c>
+      <c r="F8" s="7">
+        <v>37.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="7">
+        <v>66</v>
+      </c>
+      <c r="D9" s="7">
+        <v>70</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" s="7">
+        <v>64.3</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="7">
+        <v>65</v>
+      </c>
+      <c r="D11" s="7">
+        <v>73.2</v>
+      </c>
+      <c r="E11" s="7">
+        <v>63.1</v>
+      </c>
+      <c r="F11" s="7">
+        <v>57.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C12" s="7">
+        <v>55</v>
+      </c>
+      <c r="D12" s="7">
+        <v>59</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C13" s="7">
+        <v>53.3</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="6">
+        <v>70</v>
+      </c>
+      <c r="D14" s="6">
+        <v>78.2</v>
+      </c>
+      <c r="E14" s="6">
+        <v>59.1</v>
+      </c>
+      <c r="F14" s="6">
+        <v>53.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C15" s="6">
+        <v>58</v>
+      </c>
+      <c r="D15" s="6">
+        <v>62</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C16" s="6">
+        <v>56.3</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="6">
+        <v>79</v>
+      </c>
+      <c r="D17" s="6">
+        <v>87.2</v>
+      </c>
+      <c r="E17" s="6">
+        <v>37.1</v>
+      </c>
+      <c r="F17" s="6">
+        <v>35.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C18" s="6">
+        <v>66</v>
+      </c>
+      <c r="D18" s="6">
+        <v>70</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C19" s="6">
+        <v>64.3</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C20" s="5">
+        <v>43</v>
+      </c>
+      <c r="D20" s="5">
+        <v>51.2</v>
+      </c>
+      <c r="E20" s="5">
+        <v>61.1</v>
+      </c>
+      <c r="F20" s="5">
+        <v>49.1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C21" s="5">
+        <v>40</v>
+      </c>
+      <c r="D21" s="5">
+        <v>44</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C22" s="5">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C29" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="6">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C32" s="7">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="8"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="17">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="14"/>
+      <c r="B35" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="C35" s="17">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="14"/>
+      <c r="B36" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="17">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="8"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C38" s="5">
+        <v>8.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add last edit date for data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C42C46-C15D-43D1-B842-3D8F1233B84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF0AEF5-E870-4EF7-B69D-3DC7B2DFBBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="194">
   <si>
     <t>-</t>
   </si>
@@ -628,6 +628,9 @@
   </si>
   <si>
     <t>SOLUS X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last edit 8th May 2025 on DAP 182 </t>
   </si>
 </sst>
 </file>
@@ -1135,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
-  <dimension ref="A2:E28"/>
+  <dimension ref="A2:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1473,6 +1476,11 @@
       </c>
       <c r="C28" s="7">
         <v>14.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1486,7 +1494,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
-  <dimension ref="A2:Q25"/>
+  <dimension ref="A2:Q42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -1774,6 +1782,11 @@
       </c>
       <c r="C25" s="8">
         <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1788,7 +1801,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
-  <dimension ref="A2:Q24"/>
+  <dimension ref="A2:Q42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -1965,6 +1978,11 @@
       </c>
       <c r="C24" s="7">
         <v>11.7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1978,7 +1996,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
-  <dimension ref="A2:Q24"/>
+  <dimension ref="A2:Q42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -2155,6 +2173,11 @@
       </c>
       <c r="C24" s="7">
         <v>17.2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2168,7 +2191,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
-  <dimension ref="A2:F40"/>
+  <dimension ref="A2:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -2757,6 +2780,11 @@
         <v>11.4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -2768,7 +2796,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
-  <dimension ref="A2:D37"/>
+  <dimension ref="A2:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -2984,6 +3012,11 @@
         <v>10.5</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A28:C28"/>
@@ -2995,7 +3028,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
-  <dimension ref="A2:D38"/>
+  <dimension ref="A2:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -3206,6 +3239,11 @@
         <v>20.7</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:D2"/>
@@ -3217,7 +3255,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
-  <dimension ref="A2:F38"/>
+  <dimension ref="A2:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -3728,6 +3766,11 @@
         <v>8.4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A28:C28"/>

</xml_diff>

<commit_message>
Add YBCS flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF0AEF5-E870-4EF7-B69D-3DC7B2DFBBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58392CAD-3B7A-4311-93F8-8FC7D4363644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="YBCG" sheetId="14" r:id="rId6"/>
     <sheet name="YPDN" sheetId="15" r:id="rId7"/>
     <sheet name="YPPH" sheetId="16" r:id="rId8"/>
+    <sheet name="YBCS" sheetId="17" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="252">
   <si>
     <t>-</t>
   </si>
@@ -631,13 +632,187 @@
   </si>
   <si>
     <t xml:space="preserve">Last edit 8th May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>RWY 15</t>
+  </si>
+  <si>
+    <t>RWY 33</t>
+  </si>
+  <si>
+    <t>Runway 15</t>
+  </si>
+  <si>
+    <t>Runway 33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last edit 9th May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>LOC (HENDO)</t>
+  </si>
+  <si>
+    <t>RNP X (TODEG)</t>
+  </si>
+  <si>
+    <t>LOC (GUNRO)</t>
+  </si>
+  <si>
+    <t>RNP W (EPGAG)</t>
+  </si>
+  <si>
+    <t>LOC (RAINY arc)</t>
+  </si>
+  <si>
+    <t>LOC (KASPI arc)</t>
+  </si>
+  <si>
+    <t>RNP Y (LOTVA)</t>
+  </si>
+  <si>
+    <t>RNP X (LAVUP)</t>
+  </si>
+  <si>
+    <t>RNP W (LEBAD)</t>
+  </si>
+  <si>
+    <t>CODIE A (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>CODIE A (ANDOP trans)</t>
+  </si>
+  <si>
+    <t>CODIE A (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>CODIE A (PUNIT trans)</t>
+  </si>
+  <si>
+    <t>CODIE A (OVLET trans)</t>
+  </si>
+  <si>
+    <t>CODIE A (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (ANDOP trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (BARIA trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (ISNER trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (NORMA trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (OVLET trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (PUNIT trans)</t>
+  </si>
+  <si>
+    <t>HENDO A (VEKBI trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (ANDOP trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (OVLET trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (PUNIT trans)</t>
+  </si>
+  <si>
+    <t>KAPSI B/V (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>KEEWI A (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>KEEWI A (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>KEEWI A (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>KEEWI V (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>KEEWI V (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>KEEWI V (OVLET trans)</t>
+  </si>
+  <si>
+    <t>KEEWI V (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>KEEWI X (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>KEEWI X (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>KEEWI X (OVLET trans)</t>
+  </si>
+  <si>
+    <t>KEEWI X (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>KEEWI Y (AVDAN trans)</t>
+  </si>
+  <si>
+    <t>KEEWI Y (LOCKA trans)</t>
+  </si>
+  <si>
+    <t>KEEWI Y (ZANEY trans)</t>
+  </si>
+  <si>
+    <t>NONUM A</t>
+  </si>
+  <si>
+    <t>NONUM V</t>
+  </si>
+  <si>
+    <t>NONUM W</t>
+  </si>
+  <si>
+    <t>TOTTY W (ANDOP trans)</t>
+  </si>
+  <si>
+    <t>TOTTY W (ISNER trans)</t>
+  </si>
+  <si>
+    <t>TOTTY W (NORMA trans)</t>
+  </si>
+  <si>
+    <t>TOTTY W (PUNIT trans)</t>
+  </si>
+  <si>
+    <t>TOTTY W (VEKBI trans)</t>
+  </si>
+  <si>
+    <t>UPOLO A</t>
+  </si>
+  <si>
+    <t>UPOLO V</t>
+  </si>
+  <si>
+    <t>UPOLO W</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,6 +824,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3778,4 +3959,760 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
+  <dimension ref="A2:D64"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C4" s="5">
+        <v>58.1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5" s="5">
+        <v>51.1</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C6" s="5">
+        <v>52.1</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="5">
+        <v>61.1</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C8" s="5">
+        <v>52.1</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C9" s="5">
+        <v>57.1</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>97.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5">
+        <v>48.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <v>50.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>94.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <v>113.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C17" s="5">
+        <v>63</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C18" s="5">
+        <v>55</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C19" s="5">
+        <v>51</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="5">
+        <v>58</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C21" s="5">
+        <v>66</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C22" s="5">
+        <v>51</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>109.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <v>105.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <v>101.9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5">
+        <v>81.900000000000006</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5">
+        <v>77.900000000000006</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5">
+        <v>84.9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5">
+        <v>73.900000000000006</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5">
+        <v>105.1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5">
+        <v>101.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5">
+        <v>97.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C37" s="5">
+        <v>35</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C38" s="5">
+        <v>46</v>
+      </c>
+      <c r="D38" s="5"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C39" s="5">
+        <v>31.2</v>
+      </c>
+      <c r="D39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D40" s="5">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5">
+        <v>56.3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D42" s="5">
+        <v>54.3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="5">
+        <v>85.3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D44" s="5">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C45" s="5">
+        <v>32</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C46" s="5">
+        <v>28</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C47" s="5">
+        <v>28.4</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" s="21"/>
+      <c r="C50" s="22"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C51" s="6">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C52" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C53" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="3"/>
+      <c r="B54" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C54" s="6">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C55" s="6">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C57" s="7">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="12"/>
+      <c r="B58" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C58" s="7">
+        <v>18.899999999999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="12"/>
+      <c r="B59" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="C59" s="7">
+        <v>32.1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="12"/>
+      <c r="B60" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C60" s="7">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>198</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add YBTL flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46722658-E65C-44FA-B63B-B62E1B48B92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7979A651-0927-48EA-A53B-E829E29B42D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="8692" windowHeight="14794" activeTab="9" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="YPDN" sheetId="15" r:id="rId7"/>
     <sheet name="YPPH" sheetId="16" r:id="rId8"/>
     <sheet name="YBCS" sheetId="17" r:id="rId9"/>
+    <sheet name="YBTL" sheetId="18" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="276">
   <si>
     <t>-</t>
   </si>
@@ -815,6 +816,69 @@
   </si>
   <si>
     <t>IPMOR A (KAGMI FF)</t>
+  </si>
+  <si>
+    <t>RWY 01</t>
+  </si>
+  <si>
+    <t>RWY 19</t>
+  </si>
+  <si>
+    <t>Runway 01</t>
+  </si>
+  <si>
+    <t>Runway 19</t>
+  </si>
+  <si>
+    <t>LOC (SATCO)</t>
+  </si>
+  <si>
+    <t>LOC (KAKRO)</t>
+  </si>
+  <si>
+    <t>LOC (PARPO)</t>
+  </si>
+  <si>
+    <t>RNP P (GUGAN)</t>
+  </si>
+  <si>
+    <t>RNP P (VILUN)</t>
+  </si>
+  <si>
+    <t>VOR (TODOX)</t>
+  </si>
+  <si>
+    <t>IBUXI A</t>
+  </si>
+  <si>
+    <t>IBUXI Z</t>
+  </si>
+  <si>
+    <t>IGIKI A</t>
+  </si>
+  <si>
+    <t>POROB A</t>
+  </si>
+  <si>
+    <t>POROB Z</t>
+  </si>
+  <si>
+    <t>POROB B</t>
+  </si>
+  <si>
+    <t>POROB P</t>
+  </si>
+  <si>
+    <t>VOMPA A</t>
+  </si>
+  <si>
+    <t>VOMPA B</t>
+  </si>
+  <si>
+    <t>VOMPA P</t>
+  </si>
+  <si>
+    <t>VOMPA Z</t>
   </si>
 </sst>
 </file>
@@ -1329,13 +1393,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
   <dimension ref="A2:E42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -1344,7 +1408,7 @@
       <c r="D2" s="18"/>
       <c r="E2" s="18"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1359,7 +1423,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1376,7 +1440,7 @@
         <v>68.099999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1393,7 +1457,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1410,7 +1474,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1427,7 +1491,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1444,7 +1508,7 @@
         <v>57.5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -1461,7 +1525,7 @@
         <v>64.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -1478,7 +1542,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -1495,7 +1559,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1512,7 +1576,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1529,7 +1593,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1546,7 +1610,7 @@
         <v>43.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1563,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1580,14 +1644,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
@@ -1598,7 +1662,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1607,7 +1671,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -1616,7 +1680,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -1625,12 +1689,12 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="12" t="s">
         <v>26</v>
       </c>
@@ -1641,7 +1705,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>22</v>
@@ -1650,7 +1714,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>23</v>
@@ -1659,7 +1723,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>24</v>
@@ -1668,7 +1732,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -1682,16 +1746,295 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
+  <dimension ref="A2:D42"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="5">
+        <v>72.5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C6" s="5">
+        <v>101.3</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C7" s="5">
+        <v>51.5</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5">
+        <v>53.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C9" s="5">
+        <v>43.5</v>
+      </c>
+      <c r="D9" s="5">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>52.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" s="5">
+        <v>38.5</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C13" s="5">
+        <v>38.5</v>
+      </c>
+      <c r="D13" s="5">
+        <v>53.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A29" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" s="6">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C30" s="6">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C31" s="6">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C32" s="6">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A34" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="7">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A35" s="12"/>
+      <c r="B35" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="C35" s="7">
+        <v>19.899999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A36" s="12"/>
+      <c r="B36" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C36" s="7">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>244</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -1703,7 +2046,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1727,7 +2070,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1763,7 +2106,7 @@
       <c r="P4" s="19"/>
       <c r="Q4" s="19"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1797,7 +2140,7 @@
       <c r="P5" s="19"/>
       <c r="Q5" s="19"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1823,7 +2166,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -1849,7 +2192,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -1875,7 +2218,7 @@
         <v>79.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -1901,14 +2244,14 @@
         <v>81.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -1919,7 +2262,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="9" t="s">
         <v>36</v>
       </c>
@@ -1930,7 +2273,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9" t="s">
         <v>37</v>
       </c>
@@ -1941,7 +2284,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -1952,7 +2295,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="9" t="s">
         <v>39</v>
       </c>
@@ -1963,7 +2306,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
@@ -1974,7 +2317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -1992,13 +2335,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -2006,7 +2349,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2018,7 +2361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2040,7 +2383,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2062,7 +2405,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2076,7 +2419,7 @@
         <v>39.700000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2090,7 +2433,7 @@
         <v>67.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2104,7 +2447,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2118,14 +2461,14 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -2136,7 +2479,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>56</v>
@@ -2145,12 +2488,12 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>57</v>
       </c>
@@ -2161,7 +2504,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>59</v>
@@ -2170,7 +2513,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2187,13 +2530,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -2201,7 +2544,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>72</v>
@@ -2213,7 +2556,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2235,7 +2578,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2257,7 +2600,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2271,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2285,7 +2628,7 @@
         <v>88.6</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2299,7 +2642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2313,14 +2656,14 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>66</v>
       </c>
@@ -2331,7 +2674,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>69</v>
@@ -2340,12 +2683,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>67</v>
       </c>
@@ -2356,7 +2699,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>71</v>
@@ -2365,7 +2708,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2382,16 +2725,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -2401,7 +2744,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2419,7 +2762,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2439,7 +2782,7 @@
         <v>98.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2459,7 +2802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2479,7 +2822,7 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2499,7 +2842,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2519,7 +2862,7 @@
         <v>93.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2539,7 +2882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2559,7 +2902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2579,7 +2922,7 @@
         <v>92.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2599,7 +2942,7 @@
         <v>88.4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2619,7 +2962,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2639,7 +2982,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -2659,7 +3002,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -2679,7 +3022,7 @@
         <v>41.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -2699,7 +3042,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -2719,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -2739,7 +3082,7 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2759,7 +3102,7 @@
         <v>45.4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -2779,7 +3122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -2799,7 +3142,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -2819,7 +3162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2839,7 +3182,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -2859,14 +3202,14 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>103</v>
       </c>
@@ -2877,7 +3220,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>108</v>
@@ -2886,12 +3229,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>104</v>
       </c>
@@ -2902,7 +3245,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
         <v>119</v>
@@ -2911,7 +3254,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
         <v>110</v>
@@ -2920,12 +3263,12 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="9"/>
       <c r="B35" s="1"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14" t="s">
         <v>105</v>
       </c>
@@ -2936,7 +3279,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
         <v>112</v>
@@ -2945,12 +3288,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="9"/>
       <c r="B38" s="1"/>
       <c r="C38" s="8"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" s="16" t="s">
         <v>106</v>
       </c>
@@ -2961,7 +3304,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>114</v>
@@ -2970,7 +3313,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2987,16 +3330,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3004,7 +3347,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -3016,7 +3359,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3030,7 +3373,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3044,7 +3387,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3058,7 +3401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3072,7 +3415,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3086,7 +3429,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3100,7 +3443,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -3114,14 +3457,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>123</v>
       </c>
@@ -3132,7 +3475,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>126</v>
@@ -3141,7 +3484,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>127</v>
@@ -3150,7 +3493,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>128</v>
@@ -3159,7 +3502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>129</v>
@@ -3168,12 +3511,12 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>124</v>
       </c>
@@ -3184,7 +3527,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>131</v>
@@ -3193,7 +3536,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>139</v>
@@ -3202,7 +3545,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3219,16 +3562,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3236,7 +3579,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3248,7 +3591,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3262,7 +3605,7 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3276,7 +3619,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3290,7 +3633,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3304,7 +3647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3318,7 +3661,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3332,14 +3675,14 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>140</v>
       </c>
@@ -3350,7 +3693,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>143</v>
@@ -3359,7 +3702,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>144</v>
@@ -3368,7 +3711,7 @@
         <v>19.100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>145</v>
@@ -3377,7 +3720,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>146</v>
@@ -3386,12 +3729,12 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>141</v>
       </c>
@@ -3402,7 +3745,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>148</v>
@@ -3411,7 +3754,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>145</v>
@@ -3420,7 +3763,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>144</v>
@@ -3429,7 +3772,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3446,16 +3789,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -3465,7 +3808,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3483,7 +3826,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -3503,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3523,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -3543,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3563,7 +3906,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -3583,7 +3926,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -3603,7 +3946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -3623,7 +3966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -3643,7 +3986,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -3663,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>2</v>
       </c>
@@ -3683,7 +4026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -3703,7 +4046,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -3723,7 +4066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -3743,7 +4086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -3763,7 +4106,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -3783,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -3803,7 +4146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -3823,7 +4166,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3843,7 +4186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -3863,14 +4206,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>160</v>
       </c>
@@ -3881,7 +4224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>164</v>
@@ -3890,12 +4233,12 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>161</v>
       </c>
@@ -3906,12 +4249,12 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="9"/>
       <c r="B33" s="1"/>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="14" t="s">
         <v>162</v>
       </c>
@@ -3922,7 +4265,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>172</v>
@@ -3931,7 +4274,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>173</v>
@@ -3940,12 +4283,12 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="9"/>
       <c r="B37" s="1"/>
       <c r="C37" s="8"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="16" t="s">
         <v>163</v>
       </c>
@@ -3956,7 +4299,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3973,16 +4316,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
   <dimension ref="A2:D67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3990,7 +4333,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4002,7 +4345,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4016,7 +4359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4030,7 +4373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4044,7 +4387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4058,7 +4401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4072,7 +4415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4086,7 +4429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4100,7 +4443,7 @@
         <v>97.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -4114,7 +4457,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -4128,7 +4471,7 @@
         <v>50.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4142,7 +4485,7 @@
         <v>56.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4156,7 +4499,7 @@
         <v>104.9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -4170,7 +4513,7 @@
         <v>94.9</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -4184,7 +4527,7 @@
         <v>113.9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -4198,7 +4541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -4212,7 +4555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -4226,7 +4569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4240,7 +4583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -4254,7 +4597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4268,7 +4611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -4282,7 +4625,7 @@
         <v>109.9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -4296,7 +4639,7 @@
         <v>105.9</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -4310,7 +4653,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -4324,7 +4667,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -4338,7 +4681,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -4352,7 +4695,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -4366,7 +4709,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -4380,7 +4723,7 @@
         <v>81.900000000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -4394,7 +4737,7 @@
         <v>77.900000000000006</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -4408,7 +4751,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -4422,7 +4765,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -4436,7 +4779,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -4450,7 +4793,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -4464,7 +4807,7 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -4478,7 +4821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -4490,7 +4833,7 @@
       </c>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -4502,7 +4845,7 @@
       </c>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -4516,7 +4859,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -4530,7 +4873,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -4544,7 +4887,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -4558,7 +4901,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -4572,7 +4915,7 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -4586,7 +4929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -4600,7 +4943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -4614,7 +4957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
@@ -4628,7 +4971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -4642,7 +4985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -4656,14 +4999,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B53" s="21"/>
       <c r="C53" s="22"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="11" t="s">
         <v>192</v>
       </c>
@@ -4674,7 +5017,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>198</v>
@@ -4683,7 +5026,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="3"/>
       <c r="B56" s="3" t="s">
         <v>199</v>
@@ -4692,7 +5035,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A57" s="3"/>
       <c r="B57" s="3" t="s">
         <v>195</v>
@@ -4701,7 +5044,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>197</v>
@@ -4710,12 +5053,12 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="12" t="s">
         <v>193</v>
       </c>
@@ -4726,7 +5069,7 @@
         <v>22.9</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="12"/>
       <c r="B61" s="4" t="s">
         <v>201</v>
@@ -4735,7 +5078,7 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="12"/>
       <c r="B62" s="4" t="s">
         <v>200</v>
@@ -4744,7 +5087,7 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="12"/>
       <c r="B63" s="4" t="s">
         <v>202</v>
@@ -4753,7 +5096,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>244</v>
       </c>

</xml_diff>

<commit_message>
Update FF for YBTL STAR
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\GitHub\image-source-files\flow-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7979A651-0927-48EA-A53B-E829E29B42D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76E108A-2200-49E2-BC45-77C10FAF975B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="8692" windowHeight="14794" activeTab="9" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="7845" windowHeight="10545" activeTab="9" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -854,9 +854,6 @@
     <t>IBUXI Z</t>
   </si>
   <si>
-    <t>IGIKI A</t>
-  </si>
-  <si>
     <t>POROB A</t>
   </si>
   <si>
@@ -879,6 +876,9 @@
   </si>
   <si>
     <t>VOMPA Z</t>
+  </si>
+  <si>
+    <t>IGIKI A (36 DME TL FF)</t>
   </si>
 </sst>
 </file>
@@ -1393,13 +1393,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
   <dimension ref="A2:E42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -1408,7 +1408,7 @@
       <c r="D2" s="18"/>
       <c r="E2" s="18"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1423,7 +1423,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>68.099999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>57.5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>64.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1576,7 +1576,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>43.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1644,14 +1644,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1671,7 +1671,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -1680,7 +1680,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -1689,12 +1689,12 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>26</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>22</v>
@@ -1714,7 +1714,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>23</v>
@@ -1723,7 +1723,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>24</v>
@@ -1732,7 +1732,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -1749,16 +1749,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -1766,7 +1766,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1778,7 +1778,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1806,26 +1806,26 @@
         <v>41.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="5">
+        <v>58.2</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>267</v>
-      </c>
-      <c r="C6" s="5">
-        <v>101.3</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="C7" s="5">
         <v>51.5</v>
@@ -1834,12 +1834,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -1848,12 +1848,12 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C9" s="5">
         <v>43.5</v>
@@ -1862,12 +1862,12 @@
         <v>44.9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -1876,12 +1876,12 @@
         <v>52.5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C11" s="5">
         <v>38.5</v>
@@ -1890,12 +1890,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -1904,12 +1904,12 @@
         <v>63.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C13" s="5">
         <v>38.5</v>
@@ -1918,12 +1918,12 @@
         <v>53.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -1932,14 +1932,14 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>257</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>260</v>
@@ -1959,7 +1959,7 @@
         <v>19.3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>261</v>
@@ -1968,7 +1968,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>262</v>
@@ -1977,12 +1977,12 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>258</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
         <v>263</v>
@@ -2002,7 +2002,7 @@
         <v>19.899999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>264</v>
@@ -2011,7 +2011,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>244</v>
       </c>
@@ -2028,13 +2028,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -2046,7 +2046,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2070,7 +2070,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2106,7 +2106,7 @@
       <c r="P4" s="19"/>
       <c r="Q4" s="19"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2140,7 +2140,7 @@
       <c r="P5" s="19"/>
       <c r="Q5" s="19"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>79.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2244,14 +2244,14 @@
         <v>81.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>36</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>37</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>39</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
@@ -2317,7 +2317,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2335,13 +2335,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -2349,7 +2349,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2361,7 +2361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2383,7 +2383,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2405,7 +2405,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>39.700000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>67.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2461,14 +2461,14 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>56</v>
@@ -2488,12 +2488,12 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>57</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>59</v>
@@ -2513,7 +2513,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2530,13 +2530,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -2544,7 +2544,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>72</v>
@@ -2556,7 +2556,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2578,7 +2578,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2600,7 +2600,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>88.6</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2656,14 +2656,14 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>66</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>69</v>
@@ -2683,12 +2683,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>67</v>
       </c>
@@ -2699,7 +2699,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>71</v>
@@ -2708,7 +2708,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2725,16 +2725,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -2744,7 +2744,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2762,7 +2762,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>98.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2802,7 +2802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2822,7 +2822,7 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>93.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>92.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>88.4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>41.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>45.4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -3202,14 +3202,14 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>103</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>108</v>
@@ -3229,12 +3229,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>104</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
         <v>119</v>
@@ -3254,7 +3254,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
         <v>110</v>
@@ -3263,12 +3263,12 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="B35" s="1"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>105</v>
       </c>
@@ -3279,7 +3279,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
         <v>112</v>
@@ -3288,12 +3288,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
       <c r="B38" s="1"/>
       <c r="C38" s="8"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>106</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>114</v>
@@ -3313,7 +3313,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3330,16 +3330,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3347,7 +3347,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -3359,7 +3359,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3387,7 +3387,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3415,7 +3415,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -3457,14 +3457,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>123</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>126</v>
@@ -3484,7 +3484,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>127</v>
@@ -3493,7 +3493,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>128</v>
@@ -3502,7 +3502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>129</v>
@@ -3511,12 +3511,12 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>124</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>131</v>
@@ -3536,7 +3536,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>139</v>
@@ -3545,7 +3545,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3562,16 +3562,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3579,7 +3579,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3591,7 +3591,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3605,7 +3605,7 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3675,14 +3675,14 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>140</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>143</v>
@@ -3702,7 +3702,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>144</v>
@@ -3711,7 +3711,7 @@
         <v>19.100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>145</v>
@@ -3720,7 +3720,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>146</v>
@@ -3729,12 +3729,12 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>141</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>148</v>
@@ -3754,7 +3754,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>145</v>
@@ -3763,7 +3763,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>144</v>
@@ -3772,7 +3772,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3789,16 +3789,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -3808,7 +3808,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3826,7 +3826,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -3946,7 +3946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -3966,7 +3966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>2</v>
       </c>
@@ -4026,7 +4026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -4146,7 +4146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4166,7 +4166,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -4186,7 +4186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4206,14 +4206,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>160</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>164</v>
@@ -4233,12 +4233,12 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>161</v>
       </c>
@@ -4249,12 +4249,12 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="1"/>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>162</v>
       </c>
@@ -4265,7 +4265,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>172</v>
@@ -4274,7 +4274,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>173</v>
@@ -4283,12 +4283,12 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="1"/>
       <c r="C37" s="8"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>163</v>
       </c>
@@ -4299,7 +4299,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4316,16 +4316,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
   <dimension ref="A2:D67"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -4333,7 +4333,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4345,7 +4345,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4359,7 +4359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4401,7 +4401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4429,7 +4429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>97.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -4457,7 +4457,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>50.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4485,7 +4485,7 @@
         <v>56.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>104.9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -4513,7 +4513,7 @@
         <v>94.9</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>113.9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -4541,7 +4541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -4569,7 +4569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4583,7 +4583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4611,7 +4611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>109.9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -4639,7 +4639,7 @@
         <v>105.9</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -4667,7 +4667,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -4695,7 +4695,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -4709,7 +4709,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>81.900000000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>77.900000000000006</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -4751,7 +4751,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -4765,7 +4765,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -4821,7 +4821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -4859,7 +4859,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -4873,7 +4873,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -4943,7 +4943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -4957,7 +4957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -4999,14 +4999,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B53" s="21"/>
       <c r="C53" s="22"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
         <v>192</v>
       </c>
@@ -5017,7 +5017,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>198</v>
@@ -5026,7 +5026,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3" t="s">
         <v>199</v>
@@ -5035,7 +5035,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3" t="s">
         <v>195</v>
@@ -5044,7 +5044,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>197</v>
@@ -5053,12 +5053,12 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="12" t="s">
         <v>193</v>
       </c>
@@ -5069,7 +5069,7 @@
         <v>22.9</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="12"/>
       <c r="B61" s="4" t="s">
         <v>201</v>
@@ -5078,7 +5078,7 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="12"/>
       <c r="B62" s="4" t="s">
         <v>200</v>
@@ -5087,7 +5087,7 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="12"/>
       <c r="B63" s="4" t="s">
         <v>202</v>
@@ -5096,7 +5096,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>244</v>
       </c>

</xml_diff>

<commit_message>
Add YWLM flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76E108A-2200-49E2-BC45-77C10FAF975B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B002A2F4-11B8-4CD9-8322-C977127FE570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="7845" windowHeight="10545" activeTab="9" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="8220" windowHeight="20985" activeTab="10" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="YPPH" sheetId="16" r:id="rId8"/>
     <sheet name="YBCS" sheetId="17" r:id="rId9"/>
     <sheet name="YBTL" sheetId="18" r:id="rId10"/>
+    <sheet name="YWLM" sheetId="19" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="300">
   <si>
     <t>-</t>
   </si>
@@ -879,6 +880,78 @@
   </si>
   <si>
     <t>IGIKI A (36 DME TL FF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last edit 11th May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>LOC (IPMED)</t>
+  </si>
+  <si>
+    <t>LOC (OSATO)</t>
+  </si>
+  <si>
+    <t>LOC (OMLIR)</t>
+  </si>
+  <si>
+    <t>RNP Z (DOXAP)</t>
+  </si>
+  <si>
+    <t>RNP Z (AKLOL)</t>
+  </si>
+  <si>
+    <t>RNP X (IDSAX)</t>
+  </si>
+  <si>
+    <t>RNP W (UBGIM)</t>
+  </si>
+  <si>
+    <t>ASUVA</t>
+  </si>
+  <si>
+    <t>RNP Z (UPVIB)</t>
+  </si>
+  <si>
+    <t>EKIPU</t>
+  </si>
+  <si>
+    <t>IVTAG R (EKIPU trans)</t>
+  </si>
+  <si>
+    <t>IVTAG R (OVLUX trans)</t>
+  </si>
+  <si>
+    <t>IVTAG R (PUDUT trans)</t>
+  </si>
+  <si>
+    <t>IVTAG V (EKIPU trans)</t>
+  </si>
+  <si>
+    <t>IVTAG V (OVLUX trans)</t>
+  </si>
+  <si>
+    <t>IVTAG V (PUDUT trans)</t>
+  </si>
+  <si>
+    <t>LAXUM A</t>
+  </si>
+  <si>
+    <t>LAXUM B</t>
+  </si>
+  <si>
+    <t>LAXUM R</t>
+  </si>
+  <si>
+    <t>RNP X (IDSUS)</t>
+  </si>
+  <si>
+    <t>LAXUM V</t>
+  </si>
+  <si>
+    <t>OVLUX</t>
+  </si>
+  <si>
+    <t>PUDUT</t>
   </si>
 </sst>
 </file>
@@ -2025,6 +2098,345 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49864E6F-5D2D-438C-A891-0771B0E2C7F9}">
+  <dimension ref="A2:D42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C4" s="5">
+        <v>63.5</v>
+      </c>
+      <c r="D4" s="5">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C5" s="5">
+        <v>48.5</v>
+      </c>
+      <c r="D5" s="5">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="5">
+        <v>31.5</v>
+      </c>
+      <c r="D12" s="5">
+        <v>65.900000000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="5">
+        <v>41.7</v>
+      </c>
+      <c r="D13" s="5">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C14" s="5">
+        <v>28.6</v>
+      </c>
+      <c r="D14" s="5">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="5">
+        <v>28.5</v>
+      </c>
+      <c r="D15" s="5">
+        <v>45.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C16" s="5">
+        <v>44.5</v>
+      </c>
+      <c r="D16" s="5">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C17" s="5">
+        <v>34.5</v>
+      </c>
+      <c r="D17" s="5">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C29" s="6">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C30" s="6">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C31" s="6">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C32" s="6">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C34" s="7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="12"/>
+      <c r="B35" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="C35" s="7">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="12"/>
+      <c r="B36" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C36" s="7">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="12"/>
+      <c r="B37" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C37" s="7">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="12"/>
+      <c r="B38" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="C38" s="7">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>

</xml_diff>

<commit_message>
Add initial YPAD flow data structure
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E4CD0F-FE7D-4962-9146-36D9EB4BEBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082F0071-DB9D-48EA-800A-645F766C053D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15345" activeTab="10" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="YBCS" sheetId="17" r:id="rId9"/>
     <sheet name="YBTL" sheetId="18" r:id="rId10"/>
     <sheet name="YWLM" sheetId="19" r:id="rId11"/>
+    <sheet name="YPAD" sheetId="20" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="343">
   <si>
     <t>-</t>
   </si>
@@ -955,6 +956,132 @@
   </si>
   <si>
     <t>Both IVTAG STARs can be presented as a single option, for obvious reasons</t>
+  </si>
+  <si>
+    <t>Runway 05</t>
+  </si>
+  <si>
+    <t>Runway 23</t>
+  </si>
+  <si>
+    <t>RNP Z (PADSE)</t>
+  </si>
+  <si>
+    <t>RNP Z (ELGIS/PEGTU)</t>
+  </si>
+  <si>
+    <t>RNP Y (TUMDI)</t>
+  </si>
+  <si>
+    <t>RNP X (OGUGU)</t>
+  </si>
+  <si>
+    <t>RNP W (SADMI)</t>
+  </si>
+  <si>
+    <t>LOC (VIRAT)</t>
+  </si>
+  <si>
+    <t>RNP (PADNJ)</t>
+  </si>
+  <si>
+    <t>RWY 05</t>
+  </si>
+  <si>
+    <t>RWY 23</t>
+  </si>
+  <si>
+    <t>ATNAR V</t>
+  </si>
+  <si>
+    <t>ATNAR W</t>
+  </si>
+  <si>
+    <t>ATPIP</t>
+  </si>
+  <si>
+    <t>BEVSO</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z (MARGO trans)</t>
+  </si>
+  <si>
+    <t>ATNAR A/Z</t>
+  </si>
+  <si>
+    <t>BUGSO V (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSO V (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSO V (MARGO trans)</t>
+  </si>
+  <si>
+    <t>BUGSO W (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSO W (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSO W (MARGO trans)</t>
+  </si>
+  <si>
+    <t>DRINA A/Z</t>
+  </si>
+  <si>
+    <t>DRINA V</t>
+  </si>
+  <si>
+    <t>ELROX V</t>
+  </si>
+  <si>
+    <t>GULFS V (ATNAR FF)</t>
+  </si>
+  <si>
+    <t>INTOG V</t>
+  </si>
+  <si>
+    <t>INTOG X</t>
+  </si>
+  <si>
+    <t>INTOG Z</t>
+  </si>
+  <si>
+    <t>KAKLU A/Z</t>
+  </si>
+  <si>
+    <t>KAKLU V</t>
+  </si>
+  <si>
+    <t>KAKLU X</t>
+  </si>
+  <si>
+    <t>PAMMY V (AGROS trans)</t>
+  </si>
+  <si>
+    <t>PAMMY V (MARGO trans)</t>
+  </si>
+  <si>
+    <t>RAYNA A/Z (ERITH trans)</t>
+  </si>
+  <si>
+    <t>RAYNA A/Z (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>RAYNA V (ERITH trans)</t>
+  </si>
+  <si>
+    <t>RAYNA V (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>SURGN (KAKLU FF)</t>
   </si>
 </sst>
 </file>
@@ -2089,7 +2216,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>244</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -2491,6 +2618,645 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
+  <dimension ref="A2:F50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B38" s="21"/>
+      <c r="C38" s="22"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C39" s="6">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C40" s="6">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C41" s="6">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C42" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C43" s="6">
+        <v>9.8000000000000007</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C45" s="7">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="12"/>
+      <c r="B46" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="C46" s="7">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>

</xml_diff>

<commit_message>
More YPAD structural updates
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72ACD2FD-A6B2-497A-A031-00D622A437E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CCEE9F-EEEB-4D95-8DFF-75BF6460C26B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="344">
   <si>
     <t>-</t>
   </si>
@@ -997,9 +997,6 @@
     <t>ATNAR W</t>
   </si>
   <si>
-    <t>ATPIP</t>
-  </si>
-  <si>
     <t>BEVSO</t>
   </si>
   <si>
@@ -1015,24 +1012,6 @@
     <t>ATNAR A/Z</t>
   </si>
   <si>
-    <t>BUGSO V (AGROS trans)</t>
-  </si>
-  <si>
-    <t>BUGSO V (KLAVA trans)</t>
-  </si>
-  <si>
-    <t>BUGSO V (MARGO trans)</t>
-  </si>
-  <si>
-    <t>BUGSO W (AGROS trans)</t>
-  </si>
-  <si>
-    <t>BUGSO W (KLAVA trans)</t>
-  </si>
-  <si>
-    <t>BUGSO W (MARGO trans)</t>
-  </si>
-  <si>
     <t>DRINA A/Z</t>
   </si>
   <si>
@@ -1087,10 +1066,25 @@
     <t>ERITH DCT IAF</t>
   </si>
   <si>
-    <t>DRINA DCT IAF</t>
-  </si>
-  <si>
-    <t>INTOG DCT IAF</t>
+    <t>ATPIP (INTOG FF)</t>
+  </si>
+  <si>
+    <t>BUGSU V (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU V (MARGO trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W (MARGO trans)</t>
+  </si>
+  <si>
+    <t>BUGSU V (KLAVA trans)</t>
   </si>
 </sst>
 </file>
@@ -1605,13 +1599,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
   <dimension ref="A2:E42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -1620,7 +1614,7 @@
       <c r="D2" s="18"/>
       <c r="E2" s="18"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1635,7 +1629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1652,7 +1646,7 @@
         <v>68.099999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1669,7 +1663,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1686,7 +1680,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1703,7 +1697,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1720,7 +1714,7 @@
         <v>57.5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -1737,7 +1731,7 @@
         <v>64.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -1754,7 +1748,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -1771,7 +1765,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1788,7 +1782,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1805,7 +1799,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1822,7 +1816,7 @@
         <v>43.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1839,7 +1833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1856,14 +1850,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
@@ -1874,7 +1868,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1883,7 +1877,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -1892,7 +1886,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -1901,12 +1895,12 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="12" t="s">
         <v>26</v>
       </c>
@@ -1917,7 +1911,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>22</v>
@@ -1926,7 +1920,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>23</v>
@@ -1935,7 +1929,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>24</v>
@@ -1944,7 +1938,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -1961,16 +1955,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -1978,7 +1972,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1990,7 +1984,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2004,7 +1998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2018,7 +2012,7 @@
         <v>41.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2032,7 +2026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2046,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2060,7 +2054,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2074,7 +2068,7 @@
         <v>44.9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2088,7 +2082,7 @@
         <v>52.5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2102,7 +2096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2116,7 +2110,7 @@
         <v>63.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2130,7 +2124,7 @@
         <v>53.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2144,14 +2138,14 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>257</v>
       </c>
@@ -2162,7 +2156,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>260</v>
@@ -2171,7 +2165,7 @@
         <v>19.3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>261</v>
@@ -2180,7 +2174,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>262</v>
@@ -2189,12 +2183,12 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12" t="s">
         <v>258</v>
       </c>
@@ -2205,7 +2199,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
         <v>263</v>
@@ -2214,7 +2208,7 @@
         <v>19.899999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>264</v>
@@ -2223,7 +2217,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>276</v>
       </c>
@@ -2240,16 +2234,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49864E6F-5D2D-438C-A891-0771B0E2C7F9}">
   <dimension ref="A2:M42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -2257,7 +2251,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2269,7 +2263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2283,7 +2277,7 @@
         <v>24.1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2297,7 +2291,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2321,7 +2315,7 @@
       <c r="L6" s="19"/>
       <c r="M6" s="19"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2343,7 +2337,7 @@
       <c r="L7" s="19"/>
       <c r="M7" s="19"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2365,7 +2359,7 @@
       <c r="L8" s="19"/>
       <c r="M8" s="19"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2387,7 +2381,7 @@
       <c r="L9" s="19"/>
       <c r="M9" s="19"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2409,7 +2403,7 @@
       <c r="L10" s="19"/>
       <c r="M10" s="19"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2431,7 +2425,7 @@
       <c r="L11" s="19"/>
       <c r="M11" s="19"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2445,7 +2439,7 @@
         <v>65.900000000000006</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2459,7 +2453,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2473,7 +2467,7 @@
         <v>43.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -2487,7 +2481,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -2501,7 +2495,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -2515,14 +2509,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>54</v>
       </c>
@@ -2533,7 +2527,7 @@
         <v>12.7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>278</v>
@@ -2542,7 +2536,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>279</v>
@@ -2551,7 +2545,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>296</v>
@@ -2560,12 +2554,12 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12" t="s">
         <v>57</v>
       </c>
@@ -2576,7 +2570,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
         <v>281</v>
@@ -2585,7 +2579,7 @@
         <v>20.9</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>285</v>
@@ -2594,7 +2588,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>282</v>
@@ -2603,7 +2597,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>283</v>
@@ -2612,7 +2606,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>276</v>
       </c>
@@ -2630,16 +2624,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
   <dimension ref="A2:F51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="24.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -2649,7 +2643,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2667,12 +2661,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
@@ -2683,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2699,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2717,36 +2711,36 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>314</v>
+        <v>337</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
@@ -2757,12 +2751,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
@@ -2773,12 +2767,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
@@ -2789,12 +2783,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
@@ -2805,12 +2799,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>321</v>
+        <v>343</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
@@ -2821,12 +2815,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
@@ -2837,12 +2831,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>323</v>
+        <v>340</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
@@ -2855,12 +2849,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
@@ -2873,12 +2867,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>325</v>
+        <v>342</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
@@ -2891,12 +2885,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>0</v>
@@ -2909,12 +2903,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>0</v>
@@ -2927,26 +2921,26 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>344</v>
+        <v>321</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -2955,26 +2949,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
@@ -2987,12 +2985,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
@@ -3005,124 +3003,128 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E25" s="5"/>
       <c r="F25" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E27" s="5"/>
+      <c r="E27" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F27" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="2" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>339</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -3135,12 +3137,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>0</v>
@@ -3153,74 +3155,38 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A34" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+      <c r="B34" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A35" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B39" s="18"/>
       <c r="C39" s="18"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" s="11" t="s">
         <v>301</v>
       </c>
@@ -3231,7 +3197,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
       <c r="B41" s="3" t="s">
         <v>304</v>
@@ -3240,7 +3206,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
         <v>305</v>
@@ -3249,7 +3215,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
         <v>306</v>
@@ -3258,7 +3224,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" s="3"/>
       <c r="B44" s="3" t="s">
         <v>307</v>
@@ -3267,12 +3233,12 @@
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46" s="12" t="s">
         <v>302</v>
       </c>
@@ -3283,7 +3249,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47" s="12"/>
       <c r="B47" s="4" t="s">
         <v>309</v>
@@ -3292,7 +3258,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>276</v>
       </c>
@@ -3309,13 +3275,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -3327,7 +3293,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3351,7 +3317,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3387,7 +3353,7 @@
       <c r="P4" s="19"/>
       <c r="Q4" s="19"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3421,7 +3387,7 @@
       <c r="P5" s="19"/>
       <c r="Q5" s="19"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3447,7 +3413,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3473,7 +3439,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3499,7 +3465,7 @@
         <v>79.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3525,14 +3491,14 @@
         <v>81.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -3543,7 +3509,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="9" t="s">
         <v>36</v>
       </c>
@@ -3554,7 +3520,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9" t="s">
         <v>37</v>
       </c>
@@ -3565,7 +3531,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -3576,7 +3542,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="9" t="s">
         <v>39</v>
       </c>
@@ -3587,7 +3553,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
@@ -3598,7 +3564,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3616,13 +3582,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3630,7 +3596,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3642,7 +3608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3664,7 +3630,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3686,7 +3652,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3700,7 +3666,7 @@
         <v>39.700000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3714,7 +3680,7 @@
         <v>67.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3728,7 +3694,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3742,14 +3708,14 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -3760,7 +3726,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>56</v>
@@ -3769,12 +3735,12 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>57</v>
       </c>
@@ -3785,7 +3751,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>59</v>
@@ -3794,7 +3760,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -3811,13 +3777,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -3825,7 +3791,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>72</v>
@@ -3837,7 +3803,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3859,7 +3825,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3881,7 +3847,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3895,7 +3861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -3909,7 +3875,7 @@
         <v>88.6</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -3923,7 +3889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -3937,14 +3903,14 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>66</v>
       </c>
@@ -3955,7 +3921,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>69</v>
@@ -3964,12 +3930,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>67</v>
       </c>
@@ -3980,7 +3946,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>71</v>
@@ -3989,7 +3955,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4006,16 +3972,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -4025,7 +3991,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4043,7 +4009,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4063,7 +4029,7 @@
         <v>98.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4083,7 +4049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4103,7 +4069,7 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4123,7 +4089,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4143,7 +4109,7 @@
         <v>93.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4163,7 +4129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4183,7 +4149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -4203,7 +4169,7 @@
         <v>92.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -4223,7 +4189,7 @@
         <v>88.4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4243,7 +4209,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4263,7 +4229,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -4283,7 +4249,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -4303,7 +4269,7 @@
         <v>41.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -4323,7 +4289,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -4343,7 +4309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -4363,7 +4329,7 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4383,7 +4349,7 @@
         <v>45.4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -4403,7 +4369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4423,7 +4389,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -4443,7 +4409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -4463,7 +4429,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -4483,14 +4449,14 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>103</v>
       </c>
@@ -4501,7 +4467,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>108</v>
@@ -4510,12 +4476,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>104</v>
       </c>
@@ -4526,7 +4492,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
         <v>119</v>
@@ -4535,7 +4501,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
         <v>110</v>
@@ -4544,12 +4510,12 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="9"/>
       <c r="B35" s="1"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14" t="s">
         <v>105</v>
       </c>
@@ -4560,7 +4526,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
         <v>112</v>
@@ -4569,12 +4535,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="9"/>
       <c r="B38" s="1"/>
       <c r="C38" s="8"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" s="16" t="s">
         <v>106</v>
       </c>
@@ -4585,7 +4551,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>114</v>
@@ -4594,7 +4560,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4611,16 +4577,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -4628,7 +4594,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -4640,7 +4606,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4654,7 +4620,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4668,7 +4634,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4682,7 +4648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4696,7 +4662,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4710,7 +4676,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4724,7 +4690,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4738,14 +4704,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>123</v>
       </c>
@@ -4756,7 +4722,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>126</v>
@@ -4765,7 +4731,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>127</v>
@@ -4774,7 +4740,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>128</v>
@@ -4783,7 +4749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>129</v>
@@ -4792,12 +4758,12 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>124</v>
       </c>
@@ -4808,7 +4774,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>131</v>
@@ -4817,7 +4783,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>139</v>
@@ -4826,7 +4792,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4843,16 +4809,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -4860,7 +4826,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4872,7 +4838,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4886,7 +4852,7 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4900,7 +4866,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4914,7 +4880,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4928,7 +4894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4942,7 +4908,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4956,14 +4922,14 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>140</v>
       </c>
@@ -4974,7 +4940,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>143</v>
@@ -4983,7 +4949,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>144</v>
@@ -4992,7 +4958,7 @@
         <v>19.100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>145</v>
@@ -5001,7 +4967,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>146</v>
@@ -5010,12 +4976,12 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>141</v>
       </c>
@@ -5026,7 +4992,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>148</v>
@@ -5035,7 +5001,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>145</v>
@@ -5044,7 +5010,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>144</v>
@@ -5053,7 +5019,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5070,16 +5036,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="18" t="s">
         <v>27</v>
       </c>
@@ -5089,7 +5055,7 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5107,7 +5073,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -5127,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -5147,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -5167,7 +5133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5187,7 +5153,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -5207,7 +5173,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -5227,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -5247,7 +5213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -5267,7 +5233,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -5287,7 +5253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>2</v>
       </c>
@@ -5307,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -5327,7 +5293,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -5347,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -5367,7 +5333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -5387,7 +5353,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -5407,7 +5373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -5427,7 +5393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -5447,7 +5413,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -5467,7 +5433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -5487,14 +5453,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="21"/>
       <c r="C28" s="22"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>160</v>
       </c>
@@ -5505,7 +5471,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>164</v>
@@ -5514,12 +5480,12 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>161</v>
       </c>
@@ -5530,12 +5496,12 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="9"/>
       <c r="B33" s="1"/>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="14" t="s">
         <v>162</v>
       </c>
@@ -5546,7 +5512,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>172</v>
@@ -5555,7 +5521,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>173</v>
@@ -5564,12 +5530,12 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="9"/>
       <c r="B37" s="1"/>
       <c r="C37" s="8"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="16" t="s">
         <v>163</v>
       </c>
@@ -5580,7 +5546,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5597,16 +5563,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
   <dimension ref="A2:D67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
@@ -5614,7 +5580,7 @@
       <c r="C2" s="21"/>
       <c r="D2" s="22"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5626,7 +5592,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -5640,7 +5606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5654,7 +5620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -5668,7 +5634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5682,7 +5648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5696,7 +5662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -5710,7 +5676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -5724,7 +5690,7 @@
         <v>97.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -5738,7 +5704,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -5752,7 +5718,7 @@
         <v>50.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -5766,7 +5732,7 @@
         <v>56.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5780,7 +5746,7 @@
         <v>104.9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -5794,7 +5760,7 @@
         <v>94.9</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -5808,7 +5774,7 @@
         <v>113.9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -5822,7 +5788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -5836,7 +5802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -5850,7 +5816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -5864,7 +5830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -5878,7 +5844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -5892,7 +5858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -5906,7 +5872,7 @@
         <v>109.9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -5920,7 +5886,7 @@
         <v>105.9</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -5934,7 +5900,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -5948,7 +5914,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -5962,7 +5928,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -5976,7 +5942,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -5990,7 +5956,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -6004,7 +5970,7 @@
         <v>81.900000000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -6018,7 +5984,7 @@
         <v>77.900000000000006</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -6032,7 +5998,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -6046,7 +6012,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -6060,7 +6026,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -6074,7 +6040,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -6088,7 +6054,7 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -6102,7 +6068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -6114,7 +6080,7 @@
       </c>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -6126,7 +6092,7 @@
       </c>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -6140,7 +6106,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -6154,7 +6120,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -6168,7 +6134,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -6182,7 +6148,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -6196,7 +6162,7 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -6210,7 +6176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -6224,7 +6190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -6238,7 +6204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
@@ -6252,7 +6218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -6266,7 +6232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -6280,14 +6246,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B53" s="21"/>
       <c r="C53" s="22"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="11" t="s">
         <v>192</v>
       </c>
@@ -6298,7 +6264,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>198</v>
@@ -6307,7 +6273,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="3"/>
       <c r="B56" s="3" t="s">
         <v>199</v>
@@ -6316,7 +6282,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A57" s="3"/>
       <c r="B57" s="3" t="s">
         <v>195</v>
@@ -6325,7 +6291,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>197</v>
@@ -6334,12 +6300,12 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="12" t="s">
         <v>193</v>
       </c>
@@ -6350,7 +6316,7 @@
         <v>22.9</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="12"/>
       <c r="B61" s="4" t="s">
         <v>201</v>
@@ -6359,7 +6325,7 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="12"/>
       <c r="B62" s="4" t="s">
         <v>200</v>
@@ -6368,7 +6334,7 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="12"/>
       <c r="B63" s="4" t="s">
         <v>202</v>
@@ -6377,7 +6343,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>244</v>
       </c>

</xml_diff>

<commit_message>
Fix YBCS flow data error
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD493AEC-35C6-452A-9163-8F2153B91725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D662BA-FE08-45D4-96F9-D1809D66BD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10620" windowHeight="20805" firstSheet="5" activeTab="8" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="362">
   <si>
     <t>-</t>
   </si>
@@ -778,36 +778,6 @@
     <t>TOTTY W (VEKBI trans)</t>
   </si>
   <si>
-    <t>NONUM A (BARIA FF)</t>
-  </si>
-  <si>
-    <t>NONUM V (BARIA FF)</t>
-  </si>
-  <si>
-    <t>NONUM W (BARIA FF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last edit 10th May 2025 on DAP 182 </t>
-  </si>
-  <si>
-    <t>UPOLO A (MUSEY FF)</t>
-  </si>
-  <si>
-    <t>UPOLO V (MUSEY FF)</t>
-  </si>
-  <si>
-    <t>UPOLO W (MUSEY FF)</t>
-  </si>
-  <si>
-    <t>UPOLO V (NORMA FF)</t>
-  </si>
-  <si>
-    <t>UPOLO W (NORMA FF)</t>
-  </si>
-  <si>
-    <t>UPOLO A (NORMA FF)</t>
-  </si>
-  <si>
     <t>MEPIL (YAKKA FF)</t>
   </si>
   <si>
@@ -1130,6 +1100,45 @@
   </si>
   <si>
     <t>To Add:</t>
+  </si>
+  <si>
+    <t>UPOLO A (BARIA FF)</t>
+  </si>
+  <si>
+    <t>UPOLO V (BARIA FF)</t>
+  </si>
+  <si>
+    <t>UPOLO W (BARIA FF)</t>
+  </si>
+  <si>
+    <t>NONUM A (MUSEY FF)</t>
+  </si>
+  <si>
+    <t>NONUM V (MUSEY FF)</t>
+  </si>
+  <si>
+    <t>NONUM W (MUSEY FF)</t>
+  </si>
+  <si>
+    <t>NONUM W (NORMA FF)</t>
+  </si>
+  <si>
+    <t>NONUM V (NORMA FF)</t>
+  </si>
+  <si>
+    <t>NONUM A (NORMA FF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last edit 18th May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>NONUM A (NONUM FF)</t>
+  </si>
+  <si>
+    <t>NONUM V (NONUM FF)</t>
+  </si>
+  <si>
+    <t>NONUM W (NONUM FF)</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1168,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1193,6 +1202,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1261,7 +1276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1294,6 +1309,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1309,7 +1334,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1652,13 +1677,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1897,11 +1922,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -2011,12 +2036,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2024,10 +2049,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2035,7 +2060,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C4" s="5">
         <v>72.5</v>
@@ -2049,7 +2074,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>0</v>
@@ -2063,7 +2088,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="C6" s="5">
         <v>58.2</v>
@@ -2077,7 +2102,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="C7" s="5">
         <v>51.5</v>
@@ -2091,7 +2116,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -2105,7 +2130,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C9" s="5">
         <v>43.5</v>
@@ -2119,7 +2144,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -2133,7 +2158,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="C11" s="5">
         <v>38.5</v>
@@ -2147,7 +2172,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -2161,7 +2186,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="C13" s="5">
         <v>38.5</v>
@@ -2175,7 +2200,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -2185,18 +2210,18 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="C29" s="6">
         <v>13.5</v>
@@ -2205,7 +2230,7 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C30" s="6">
         <v>19.3</v>
@@ -2214,7 +2239,7 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C31" s="6">
         <v>21.5</v>
@@ -2223,7 +2248,7 @@
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C32" s="6">
         <v>19.5</v>
@@ -2236,7 +2261,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>142</v>
@@ -2248,7 +2273,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C35" s="7">
         <v>19.899999999999999</v>
@@ -2257,7 +2282,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="C36" s="7">
         <v>24.5</v>
@@ -2265,7 +2290,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -2290,12 +2315,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2314,7 +2339,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="C4" s="5">
         <v>63.5</v>
@@ -2328,7 +2353,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="C5" s="5">
         <v>48.5</v>
@@ -2342,7 +2367,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>0</v>
@@ -2350,23 +2375,23 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>300</v>
-      </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
+      <c r="F6" s="23" t="s">
+        <v>290</v>
+      </c>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>0</v>
@@ -2374,21 +2399,21 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -2396,21 +2421,21 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -2418,21 +2443,21 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -2440,21 +2465,21 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>0</v>
@@ -2462,21 +2487,21 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="C12" s="5">
         <v>31.5</v>
@@ -2490,7 +2515,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="C13" s="5">
         <v>41.7</v>
@@ -2504,7 +2529,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="C14" s="5">
         <v>28.6</v>
@@ -2518,7 +2543,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="C15" s="5">
         <v>28.5</v>
@@ -2532,7 +2557,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="C16" s="5">
         <v>44.5</v>
@@ -2546,7 +2571,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="C17" s="5">
         <v>34.5</v>
@@ -2556,18 +2581,18 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>54</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="C29" s="6">
         <v>12.7</v>
@@ -2576,7 +2601,7 @@
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="C30" s="6">
         <v>16.5</v>
@@ -2585,7 +2610,7 @@
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="C31" s="6">
         <v>16.5</v>
@@ -2594,7 +2619,7 @@
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="C32" s="6">
         <v>9.6</v>
@@ -2610,7 +2635,7 @@
         <v>57</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="C34" s="7">
         <v>21</v>
@@ -2619,7 +2644,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="C35" s="7">
         <v>20.9</v>
@@ -2628,7 +2653,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="C36" s="7">
         <v>14.1</v>
@@ -2637,7 +2662,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="C37" s="7">
         <v>14.8</v>
@@ -2646,7 +2671,7 @@
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="C38" s="7">
         <v>9.5</v>
@@ -2654,7 +2679,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -2680,14 +2705,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2695,13 +2720,13 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>53</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>5</v>
@@ -2712,7 +2737,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
@@ -2728,7 +2753,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
@@ -2744,7 +2769,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
@@ -2762,7 +2787,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
@@ -2774,7 +2799,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
@@ -2786,7 +2811,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
@@ -2796,8 +2821,8 @@
       <c r="F9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J9" s="23" t="s">
-        <v>343</v>
+      <c r="J9" s="21" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2805,7 +2830,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
@@ -2816,7 +2841,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2824,7 +2849,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
@@ -2835,7 +2860,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2843,7 +2868,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
@@ -2854,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2862,7 +2887,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
@@ -2873,7 +2898,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -2881,7 +2906,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
@@ -2892,7 +2917,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -2900,7 +2925,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
@@ -2913,7 +2938,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -2921,7 +2946,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
@@ -2939,7 +2964,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
@@ -2952,7 +2977,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -2960,7 +2985,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>0</v>
@@ -2973,10 +2998,10 @@
         <v>0</v>
       </c>
       <c r="J18" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="M18" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -2984,7 +3009,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>0</v>
@@ -2997,10 +3022,10 @@
         <v>0</v>
       </c>
       <c r="J19" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="M19" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -3008,7 +3033,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
@@ -3017,10 +3042,10 @@
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="M20" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -3028,7 +3053,7 @@
         <v>3</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -3037,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="M21" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -3045,7 +3070,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5" t="s">
@@ -3058,7 +3083,7 @@
         <v>0</v>
       </c>
       <c r="M22" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -3066,7 +3091,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
@@ -3084,7 +3109,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
@@ -3102,7 +3127,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
@@ -3118,7 +3143,7 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
@@ -3136,7 +3161,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
@@ -3154,7 +3179,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -3168,7 +3193,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -3182,7 +3207,7 @@
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>0</v>
@@ -3200,7 +3225,7 @@
         <v>20</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>0</v>
@@ -3218,7 +3243,7 @@
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -3236,7 +3261,7 @@
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>0</v>
@@ -3254,7 +3279,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
@@ -3262,18 +3287,18 @@
       <c r="F34" s="6"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="18" t="s">
+      <c r="A39" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="C40" s="6">
         <v>14.8</v>
@@ -3282,7 +3307,7 @@
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="C41" s="6">
         <v>15.8</v>
@@ -3291,7 +3316,7 @@
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="C42" s="6">
         <v>6.5</v>
@@ -3300,7 +3325,7 @@
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="C43" s="6">
         <v>9.4</v>
@@ -3309,7 +3334,7 @@
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="C44" s="6">
         <v>9.8000000000000007</v>
@@ -3322,10 +3347,10 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="C46" s="7">
         <v>14.2</v>
@@ -3334,7 +3359,7 @@
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12"/>
       <c r="B47" s="4" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="C47" s="7">
         <v>18.7</v>
@@ -3342,7 +3367,7 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3364,16 +3389,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3424,16 +3449,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3460,21 +3485,21 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="C6" s="5">
         <v>67.2</v>
@@ -3552,7 +3577,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="C9" s="5">
         <v>44</v>
@@ -3574,11 +3599,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -3671,12 +3696,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3791,11 +3816,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -3866,12 +3891,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3986,11 +4011,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4064,14 +4089,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4532,11 +4557,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4669,12 +4694,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4787,11 +4812,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4901,12 +4926,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4925,7 +4950,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C4" s="5">
         <v>48.4</v>
@@ -5005,11 +5030,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5128,14 +5153,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5220,7 +5245,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="C7" s="5">
         <v>74</v>
@@ -5536,11 +5561,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5644,7 +5669,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
-  <dimension ref="A2:D67"/>
+  <dimension ref="A2:E70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -5655,12 +5680,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -6080,7 +6105,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -6094,7 +6119,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -6108,7 +6133,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -6122,7 +6147,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -6136,45 +6161,48 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>241</v>
+        <v>349</v>
       </c>
       <c r="C37" s="5">
-        <v>35</v>
+        <v>71.2</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" s="27"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>242</v>
+        <v>350</v>
       </c>
       <c r="C38" s="5">
-        <v>46</v>
+        <v>67.2</v>
       </c>
       <c r="D38" s="5"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38" s="27"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>243</v>
+        <v>351</v>
       </c>
       <c r="C39" s="5">
-        <v>31.2</v>
+        <v>67.599999999999994</v>
       </c>
       <c r="D39" s="5"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" s="27"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -6188,7 +6216,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -6202,7 +6230,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -6216,7 +6244,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -6230,7 +6258,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -6244,195 +6272,245 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>245</v>
+        <v>352</v>
       </c>
       <c r="C45" s="5">
-        <v>102.5</v>
+        <v>65.8</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45" s="27"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>246</v>
+        <v>353</v>
       </c>
       <c r="C46" s="5">
-        <v>98.5</v>
+        <v>76.8</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46" s="27"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>247</v>
+        <v>354</v>
       </c>
       <c r="C47" s="5">
-        <v>98.9</v>
+        <v>62</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47" s="27"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>250</v>
+        <v>357</v>
       </c>
       <c r="C48" s="5">
-        <v>116.5</v>
+        <v>80.400000000000006</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E48" s="27"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>248</v>
+        <v>356</v>
       </c>
       <c r="C49" s="5">
-        <v>112.5</v>
+        <v>91.4</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" s="27"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>249</v>
+        <v>355</v>
       </c>
       <c r="C50" s="5">
-        <v>112.9</v>
+        <v>76.599999999999994</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="20" t="s">
+      <c r="E50" s="27"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C51" s="5">
+        <v>35</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E51" s="27"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E52" s="27"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C53" s="5">
+        <v>31.2</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E53" s="27"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B53" s="21"/>
-      <c r="C53" s="22"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="11" t="s">
+      <c r="B56" s="19"/>
+      <c r="C56" s="20"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B57" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="C54" s="6">
+      <c r="C57" s="6">
         <v>17.7</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C55" s="6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="C56" s="6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="C57" s="6">
-        <v>20.399999999999999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C58" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C59" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C60" s="6">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C58" s="6">
+      <c r="C61" s="6">
         <v>21.2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="12" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B63" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C60" s="7">
+      <c r="C63" s="7">
         <v>22.9</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="12"/>
-      <c r="B61" s="4" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="12"/>
+      <c r="B64" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C61" s="7">
+      <c r="C64" s="7">
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="12"/>
-      <c r="B62" s="4" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="12"/>
+      <c r="B65" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C62" s="7">
+      <c r="C65" s="7">
         <v>32.1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="12"/>
-      <c r="B63" s="4" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="12"/>
+      <c r="B66" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="C63" s="7">
+      <c r="C66" s="7">
         <v>25.3</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>244</v>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>358</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A53:C53"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Add YPAD Non-Jet Entries
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7FDEC2-8BF5-42F7-B691-31069975097A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207067C8-6C1E-499F-B6FB-16E4C58DA700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="8625" windowHeight="10545" firstSheet="5" activeTab="8" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="5" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="353">
   <si>
     <t>-</t>
   </si>
@@ -961,147 +961,6 @@
     <t>RWY 23</t>
   </si>
   <si>
-    <t>ATNAR V</t>
-  </si>
-  <si>
-    <t>ATNAR W</t>
-  </si>
-  <si>
-    <t>BEVSO</t>
-  </si>
-  <si>
-    <t>BUGSU A/Z (AGROS trans)</t>
-  </si>
-  <si>
-    <t>BUGSU A/Z (KLAVA trans)</t>
-  </si>
-  <si>
-    <t>BUGSU A/Z (MARGO trans)</t>
-  </si>
-  <si>
-    <t>ATNAR A/Z</t>
-  </si>
-  <si>
-    <t>DRINA A/Z</t>
-  </si>
-  <si>
-    <t>DRINA V</t>
-  </si>
-  <si>
-    <t>ELROX V</t>
-  </si>
-  <si>
-    <t>GULFS V (ATNAR FF)</t>
-  </si>
-  <si>
-    <t>INTOG V</t>
-  </si>
-  <si>
-    <t>INTOG X</t>
-  </si>
-  <si>
-    <t>INTOG Z</t>
-  </si>
-  <si>
-    <t>KAKLU A/Z</t>
-  </si>
-  <si>
-    <t>KAKLU V</t>
-  </si>
-  <si>
-    <t>KAKLU X</t>
-  </si>
-  <si>
-    <t>PAMMY V (AGROS trans)</t>
-  </si>
-  <si>
-    <t>PAMMY V (MARGO trans)</t>
-  </si>
-  <si>
-    <t>SURGN (KAKLU FF)</t>
-  </si>
-  <si>
-    <t>RAYNA A/Z (ERITH FF)</t>
-  </si>
-  <si>
-    <t>RAYNA A/Z (KLAVA FF)</t>
-  </si>
-  <si>
-    <t>RAYNA V (ERITH FF)</t>
-  </si>
-  <si>
-    <t>RAYNA V (KLAVA FF)</t>
-  </si>
-  <si>
-    <t>ATPIP (INTOG FF)</t>
-  </si>
-  <si>
-    <t>BUGSU V (AGROS trans)</t>
-  </si>
-  <si>
-    <t>BUGSU V (MARGO trans)</t>
-  </si>
-  <si>
-    <t>BUGSU W (AGROS trans)</t>
-  </si>
-  <si>
-    <t>BUGSU W (KLAVA trans)</t>
-  </si>
-  <si>
-    <t>BUGSU W (MARGO trans)</t>
-  </si>
-  <si>
-    <t>BUGSU V (KLAVA trans)</t>
-  </si>
-  <si>
-    <t>Non-Jets</t>
-  </si>
-  <si>
-    <t>INTOG to DRINA for 23I</t>
-  </si>
-  <si>
-    <t>MARGO has STARs to all applicable runways</t>
-  </si>
-  <si>
-    <t>ATNAR has STARs to all applicable runways</t>
-  </si>
-  <si>
-    <t>KLAVA has STARs to 05/23</t>
-  </si>
-  <si>
-    <t>KAKLU has STARs to 05/23</t>
-  </si>
-  <si>
-    <t>ELROX has STARs to all applicable runways</t>
-  </si>
-  <si>
-    <t>Visual Entries:</t>
-  </si>
-  <si>
-    <t>DRINA 23/05</t>
-  </si>
-  <si>
-    <t>KLAVA 23/05</t>
-  </si>
-  <si>
-    <t>Instrument Entries:</t>
-  </si>
-  <si>
-    <t>BEVSO 23/05</t>
-  </si>
-  <si>
-    <t>MARGO</t>
-  </si>
-  <si>
-    <t>ATNAR</t>
-  </si>
-  <si>
-    <t>ELROX</t>
-  </si>
-  <si>
-    <t>To Add:</t>
-  </si>
-  <si>
     <t>UPOLO A (BARIA FF)</t>
   </si>
   <si>
@@ -1139,13 +998,127 @@
   </si>
   <si>
     <t>NONUM W (NONUM FF)</t>
+  </si>
+  <si>
+    <t>ATNAR A/Z STAR</t>
+  </si>
+  <si>
+    <t>ATNAR V STAR</t>
+  </si>
+  <si>
+    <t>ATNAR W STAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATPIP STAR (INTOG FF) </t>
+  </si>
+  <si>
+    <t>BEVSO STAR</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z STAR (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z STAR (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSU A/Z STAR (MARGO trans)</t>
+  </si>
+  <si>
+    <t>BUGSU V STAR (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU V STAR (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSU V STAR (MARGO trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W STAR (AGROS trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W STAR (KLAVA trans)</t>
+  </si>
+  <si>
+    <t>BUGSU W STAR (MARGO trans)</t>
+  </si>
+  <si>
+    <t>DRINA A/Z STAR</t>
+  </si>
+  <si>
+    <t>DRINA V STAR</t>
+  </si>
+  <si>
+    <t>ELROX V STAR</t>
+  </si>
+  <si>
+    <t>GULFS V STAR (ATNAR FF)</t>
+  </si>
+  <si>
+    <t>INTOG V STAR</t>
+  </si>
+  <si>
+    <t>INTOG X STAR</t>
+  </si>
+  <si>
+    <t>INTOG Z STAR</t>
+  </si>
+  <si>
+    <t>KAKLU A/Z STAR</t>
+  </si>
+  <si>
+    <t>KAKLU V STAR</t>
+  </si>
+  <si>
+    <t>KAKLU X STAR</t>
+  </si>
+  <si>
+    <t>PAMMY V STAR (AGROS trans)</t>
+  </si>
+  <si>
+    <t>PAMMY V STAR (MARGO trans)</t>
+  </si>
+  <si>
+    <t>RAYNA A/Z STAR (ERITH FF)</t>
+  </si>
+  <si>
+    <t>RAYNA A/Z STAR (KLAVA FF)</t>
+  </si>
+  <si>
+    <t>RAYNA V STAR (ERITH FF)</t>
+  </si>
+  <si>
+    <t>RAYNA V STAR (KLAVA FF)</t>
+  </si>
+  <si>
+    <t>SURGN STAR (KAKLU FF)</t>
+  </si>
+  <si>
+    <t>DRINA DCT IAF</t>
+  </si>
+  <si>
+    <t>AGROS DCT IAF</t>
+  </si>
+  <si>
+    <t>ATNAR DCT IAF</t>
+  </si>
+  <si>
+    <t>KAKLU DCT 5nm Final</t>
+  </si>
+  <si>
+    <t>KLAVA DCT IAF/5nm Final</t>
+  </si>
+  <si>
+    <t>MARGO DCT IAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last edit 19th May 2025 on DAP 182 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1163,6 +1136,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1270,7 +1251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1316,6 +1297,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1328,6 +1312,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1670,13 +1655,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1915,11 +1900,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -2029,12 +2014,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2203,11 +2188,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2308,12 +2293,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2368,16 +2353,16 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="24" t="s">
         <v>290</v>
       </c>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -2392,14 +2377,14 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -2414,14 +2399,14 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -2436,14 +2421,14 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -2458,14 +2443,14 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -2480,14 +2465,14 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -2574,11 +2559,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2687,30 +2672,30 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
-  <dimension ref="A2:M51"/>
+  <dimension ref="A2:J55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="9.5703125" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" customWidth="1"/>
     <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>300</v>
@@ -2726,18 +2711,20 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5" t="s">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2746,7 +2733,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
@@ -2762,87 +2749,84 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="C8" s="6"/>
+      <c r="B8" s="28" t="s">
+        <v>348</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+      <c r="E8" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>333</v>
-      </c>
+      <c r="A9" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="J9" s="21"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="J10" t="s">
-        <v>334</v>
-      </c>
+      <c r="A10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
@@ -2852,16 +2836,13 @@
       <c r="F11" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J11" t="s">
-        <v>335</v>
-      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
@@ -2871,16 +2852,13 @@
       <c r="F12" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J12" t="s">
-        <v>336</v>
-      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
@@ -2890,16 +2868,13 @@
       <c r="F13" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J13" t="s">
-        <v>337</v>
-      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
@@ -2909,29 +2884,21 @@
       <c r="F14" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J14" t="s">
-        <v>338</v>
-      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
         <v>0</v>
-      </c>
-      <c r="J15" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -2939,25 +2906,23 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
@@ -2969,174 +2934,147 @@
       <c r="F17" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J17" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>0</v>
-      </c>
+        <v>327</v>
+      </c>
+      <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F18" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J18" t="s">
-        <v>340</v>
-      </c>
-      <c r="M18" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>0</v>
-      </c>
+        <v>328</v>
+      </c>
+      <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F19" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J19" t="s">
-        <v>341</v>
-      </c>
-      <c r="M19" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="J20" t="s">
-        <v>342</v>
-      </c>
-      <c r="M20" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="B22" s="28" t="s">
+        <v>346</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="M21" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="M22" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>316</v>
+        <v>333</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F25" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>317</v>
+        <v>334</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
@@ -3149,12 +3087,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>318</v>
+        <v>335</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
@@ -3167,103 +3105,109 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="B31" s="28" t="s">
+        <v>349</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5" t="s">
+      <c r="B32" s="28" t="s">
+        <v>350</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5" t="s">
+      <c r="A33" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>351</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3272,100 +3216,199 @@
         <v>3</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
+      <c r="F34" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="22" t="s">
+      <c r="A39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="11" t="s">
+      <c r="B43" s="22"/>
+      <c r="C43" s="22"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B44" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C44" s="6">
         <v>14.8</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C45" s="6">
         <v>15.8</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="3"/>
+      <c r="B46" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="C42" s="6">
+      <c r="C46" s="6">
         <v>6.5</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C47" s="6">
         <v>9.4</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C48" s="6">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="12" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B50" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="C46" s="7">
+      <c r="C50" s="7">
         <v>14.2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="12"/>
-      <c r="B47" s="4" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="12"/>
+      <c r="B51" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="C47" s="7">
+      <c r="C51" s="7">
         <v>18.7</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>266</v>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A39:C39"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3382,16 +3425,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3442,16 +3485,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3478,14 +3521,14 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -3592,11 +3635,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -3689,12 +3732,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3809,11 +3852,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -3884,12 +3927,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4004,11 +4047,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4082,14 +4125,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4550,11 +4593,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4687,12 +4730,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4805,11 +4848,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4919,12 +4962,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5023,11 +5066,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5146,14 +5189,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5554,11 +5597,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5673,12 +5716,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -6159,7 +6202,7 @@
         <v>20</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>349</v>
+        <v>302</v>
       </c>
       <c r="C37" s="5">
         <v>71.2</v>
@@ -6173,7 +6216,7 @@
         <v>20</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>350</v>
+        <v>303</v>
       </c>
       <c r="C38" s="5">
         <v>67.2</v>
@@ -6185,7 +6228,7 @@
         <v>20</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>351</v>
+        <v>304</v>
       </c>
       <c r="C39" s="5">
         <v>67.599999999999994</v>
@@ -6267,7 +6310,7 @@
         <v>20</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>352</v>
+        <v>305</v>
       </c>
       <c r="C45" s="5">
         <v>65.8</v>
@@ -6281,7 +6324,7 @@
         <v>20</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>353</v>
+        <v>306</v>
       </c>
       <c r="C46" s="5">
         <v>76.8</v>
@@ -6295,7 +6338,7 @@
         <v>20</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>354</v>
+        <v>307</v>
       </c>
       <c r="C47" s="5">
         <v>62</v>
@@ -6309,7 +6352,7 @@
         <v>20</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>357</v>
+        <v>310</v>
       </c>
       <c r="C48" s="5">
         <v>80.400000000000006</v>
@@ -6323,7 +6366,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>356</v>
+        <v>309</v>
       </c>
       <c r="C49" s="5">
         <v>91.4</v>
@@ -6337,7 +6380,7 @@
         <v>20</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>355</v>
+        <v>308</v>
       </c>
       <c r="C50" s="5">
         <v>76.599999999999994</v>
@@ -6351,7 +6394,7 @@
         <v>20</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>359</v>
+        <v>312</v>
       </c>
       <c r="C51" s="5">
         <v>35</v>
@@ -6365,7 +6408,7 @@
         <v>20</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>360</v>
+        <v>313</v>
       </c>
       <c r="C52" s="5">
         <v>46</v>
@@ -6379,7 +6422,7 @@
         <v>20</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>361</v>
+        <v>314</v>
       </c>
       <c r="C53" s="5">
         <v>31.2</v>
@@ -6487,7 +6530,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>358</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalise YPAD flow structure (finally)
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207067C8-6C1E-499F-B6FB-16E4C58DA700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8921C3-14B8-4D5B-9725-F4CE3041EAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="5" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="355">
   <si>
     <t>-</t>
   </si>
@@ -1054,24 +1054,12 @@
     <t>GULFS V STAR (ATNAR FF)</t>
   </si>
   <si>
-    <t>INTOG V STAR</t>
-  </si>
-  <si>
-    <t>INTOG X STAR</t>
-  </si>
-  <si>
     <t>INTOG Z STAR</t>
   </si>
   <si>
     <t>KAKLU A/Z STAR</t>
   </si>
   <si>
-    <t>KAKLU V STAR</t>
-  </si>
-  <si>
-    <t>KAKLU X STAR</t>
-  </si>
-  <si>
     <t>PAMMY V STAR (AGROS trans)</t>
   </si>
   <si>
@@ -1093,25 +1081,43 @@
     <t>SURGN STAR (KAKLU FF)</t>
   </si>
   <si>
-    <t>DRINA DCT IAF</t>
-  </si>
-  <si>
     <t>AGROS DCT IAF</t>
   </si>
   <si>
     <t>ATNAR DCT IAF</t>
   </si>
   <si>
-    <t>KAKLU DCT 5nm Final</t>
-  </si>
-  <si>
-    <t>KLAVA DCT IAF/5nm Final</t>
-  </si>
-  <si>
     <t>MARGO DCT IAF</t>
   </si>
   <si>
-    <t xml:space="preserve">Last edit 19th May 2025 on DAP 182 </t>
+    <t xml:space="preserve">Last edit 20th May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>INTOG V/X STAR</t>
+  </si>
+  <si>
+    <t>KAKLU V/X STAR</t>
+  </si>
+  <si>
+    <t>ELROX DCT IAF</t>
+  </si>
+  <si>
+    <t>Circuit Join (DRINA FF)</t>
+  </si>
+  <si>
+    <t>Circuit Join (KLAVA FF)</t>
+  </si>
+  <si>
+    <t>Circuit Join (MARGO FF)</t>
+  </si>
+  <si>
+    <t>Circuit Join (AGROS FF)</t>
+  </si>
+  <si>
+    <t>Circuit Join (ATNAR FF)</t>
+  </si>
+  <si>
+    <t>Circuit Join (ELROX FF)</t>
   </si>
 </sst>
 </file>
@@ -1297,6 +1303,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1312,7 +1319,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1655,13 +1661,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1900,11 +1906,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -2014,12 +2020,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2188,11 +2194,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2293,12 +2299,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2353,16 +2359,16 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="25" t="s">
         <v>290</v>
       </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -2377,14 +2383,14 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
+      <c r="M7" s="25"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -2399,14 +2405,14 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="24"/>
-      <c r="M8" s="24"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="25"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -2421,14 +2427,14 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
-      <c r="L9" s="24"/>
-      <c r="M9" s="24"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
+      <c r="M9" s="25"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -2443,14 +2449,14 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -2465,14 +2471,14 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -2559,11 +2565,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2672,7 +2678,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
-  <dimension ref="A2:J55"/>
+  <dimension ref="A2:J56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -2683,14 +2689,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2714,8 +2720,8 @@
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>347</v>
+      <c r="B4" s="23" t="s">
+        <v>342</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>0</v>
@@ -2724,32 +2730,26 @@
       <c r="E4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
@@ -2765,34 +2765,32 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>348</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6" t="s">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2800,12 +2798,16 @@
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="C9" s="6"/>
+      <c r="B9" s="23" t="s">
+        <v>343</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
+      <c r="E9" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="F9" s="6"/>
       <c r="J9" s="21"/>
     </row>
@@ -2813,8 +2815,8 @@
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>319</v>
+      <c r="B10" s="23" t="s">
+        <v>353</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -2822,43 +2824,35 @@
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="A11" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="A12" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
@@ -2874,7 +2868,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
@@ -2890,7 +2884,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
@@ -2906,7 +2900,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
@@ -2922,15 +2916,13 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
         <v>0</v>
       </c>
@@ -2940,15 +2932,13 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
         <v>0</v>
       </c>
@@ -2958,7 +2948,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
@@ -2976,15 +2966,15 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>0</v>
-      </c>
+        <v>327</v>
+      </c>
+      <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E20" s="5"/>
+      <c r="E20" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F20" s="5" t="s">
         <v>0</v>
       </c>
@@ -2994,46 +2984,52 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="28" t="s">
-        <v>346</v>
-      </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6" t="s">
+      <c r="C23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3041,83 +3037,63 @@
       <c r="A24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>332</v>
+      <c r="B24" s="23" t="s">
+        <v>349</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="F24" s="6"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F25" s="5" t="s">
+      <c r="A25" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="A26" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>348</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="A27" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>354</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5" t="s">
+      <c r="A28" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3126,7 +3102,7 @@
         <v>20</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
@@ -3144,7 +3120,7 @@
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
@@ -3158,38 +3134,36 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="28" t="s">
-        <v>349</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6" t="s">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>350</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6" t="s">
+      <c r="A32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3197,81 +3171,67 @@
       <c r="A33" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="28" t="s">
-        <v>351</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="B33" s="23" t="s">
+        <v>350</v>
+      </c>
+      <c r="C33" s="6"/>
       <c r="D33" s="6"/>
-      <c r="E33" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="3" t="s">
-        <v>339</v>
-      </c>
-      <c r="C34" s="6"/>
+      <c r="B34" s="23" t="s">
+        <v>344</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="E34" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F34" s="6"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>340</v>
+      <c r="B35" s="23" t="s">
+        <v>351</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
-      <c r="F35" s="6" t="s">
-        <v>0</v>
-      </c>
+      <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5" t="s">
+      <c r="A36" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5" t="s">
+      <c r="A37" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3280,7 +3240,7 @@
         <v>20</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>0</v>
@@ -3298,7 +3258,7 @@
         <v>20</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>0</v>
@@ -3312,99 +3272,135 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="22" t="s">
+      <c r="B42" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="11" t="s">
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B46" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C46" s="6">
         <v>14.8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C45" s="6">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C46" s="6">
-        <v>6.5</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C47" s="6">
-        <v>9.4</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C48" s="6">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C49" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="C48" s="6">
+      <c r="C50" s="6">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="12" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B52" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="C50" s="7">
+      <c r="C52" s="7">
         <v>14.2</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="12"/>
-      <c r="B51" s="4" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="12"/>
+      <c r="B53" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C53" s="7">
         <v>18.7</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>352</v>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -3425,16 +3421,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3485,16 +3481,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="24" t="s">
+      <c r="J4" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="24"/>
-      <c r="Q4" s="24"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3521,14 +3517,14 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="24"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="24"/>
-      <c r="M5" s="24"/>
-      <c r="N5" s="24"/>
-      <c r="O5" s="24"/>
-      <c r="P5" s="24"/>
-      <c r="Q5" s="24"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="25"/>
+      <c r="O5" s="25"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -3635,11 +3631,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -3732,12 +3728,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3852,11 +3848,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -3927,12 +3923,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4047,11 +4043,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4125,14 +4121,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4593,11 +4589,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4730,12 +4726,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4848,11 +4844,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4962,12 +4958,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5066,11 +5062,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5189,14 +5185,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5597,11 +5593,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5716,12 +5712,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
Add YPAD flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8921C3-14B8-4D5B-9725-F4CE3041EAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55EB8D43-B4D4-40E1-8FFB-99C5AACE3EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="360">
   <si>
     <t>-</t>
   </si>
@@ -1009,12 +1009,6 @@
     <t>ATNAR W STAR</t>
   </si>
   <si>
-    <t xml:space="preserve">ATPIP STAR (INTOG FF) </t>
-  </si>
-  <si>
-    <t>BEVSO STAR</t>
-  </si>
-  <si>
     <t>BUGSU A/Z STAR (AGROS trans)</t>
   </si>
   <si>
@@ -1078,53 +1072,74 @@
     <t>RAYNA V STAR (KLAVA FF)</t>
   </si>
   <si>
-    <t>SURGN STAR (KAKLU FF)</t>
-  </si>
-  <si>
-    <t>AGROS DCT IAF</t>
-  </si>
-  <si>
-    <t>ATNAR DCT IAF</t>
-  </si>
-  <si>
-    <t>MARGO DCT IAF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last edit 20th May 2025 on DAP 182 </t>
-  </si>
-  <si>
     <t>INTOG V/X STAR</t>
   </si>
   <si>
     <t>KAKLU V/X STAR</t>
   </si>
   <si>
-    <t>ELROX DCT IAF</t>
-  </si>
-  <si>
-    <t>Circuit Join (DRINA FF)</t>
-  </si>
-  <si>
-    <t>Circuit Join (KLAVA FF)</t>
-  </si>
-  <si>
-    <t>Circuit Join (MARGO FF)</t>
-  </si>
-  <si>
-    <t>Circuit Join (AGROS FF)</t>
-  </si>
-  <si>
-    <t>Circuit Join (ATNAR FF)</t>
-  </si>
-  <si>
-    <t>Circuit Join (ELROX FF)</t>
+    <t xml:space="preserve">Last edit 21st May 2025 on DAP 182 </t>
+  </si>
+  <si>
+    <t>SURGN STAR - IAP (KAKLU FF)</t>
+  </si>
+  <si>
+    <t>SURGN STAR - Circuit Join (KAKLU FF)</t>
+  </si>
+  <si>
+    <t>BEVSO STAR - Circuit Join</t>
+  </si>
+  <si>
+    <t>BEVSO STAR - IAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATPIP STAR - Circuit Join (INTOG FF) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATPIP STAR - IAP (INTOG FF) </t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (AGROS FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (ATNAR FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (DRINA FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (ELROX FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (KLAVA FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Circuit Join (MARGO FF)</t>
+  </si>
+  <si>
+    <t>No STAR - AGROS DCT IAF</t>
+  </si>
+  <si>
+    <t>No STAR - ATNAR DCT IAF</t>
+  </si>
+  <si>
+    <t>No STAR - ELROX DCT IAF</t>
+  </si>
+  <si>
+    <t>No STAR - MARGO DCT IAF</t>
+  </si>
+  <si>
+    <t>RNP (All - PADEK, PADEL, PADEN)</t>
+  </si>
+  <si>
+    <t>RNP (All - PADWQ, PADWP, PADWO)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1146,16 +1161,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1189,6 +1196,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1257,7 +1270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1303,10 +1316,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1319,6 +1328,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1661,13 +1676,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1906,11 +1921,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -2020,12 +2035,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2194,11 +2209,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2299,12 +2314,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2359,16 +2374,16 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="23" t="s">
         <v>290</v>
       </c>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -2383,14 +2398,14 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -2405,14 +2420,14 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-      <c r="M8" s="25"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -2427,14 +2442,14 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -2449,14 +2464,14 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="25"/>
-      <c r="M10" s="25"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -2471,14 +2486,14 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -2565,11 +2580,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2678,25 +2693,25 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
-  <dimension ref="A2:J56"/>
+  <dimension ref="A2:J61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.7109375" customWidth="1"/>
     <col min="3" max="4" width="9.5703125" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" customWidth="1"/>
     <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2717,135 +2732,185 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>342</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6"/>
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" s="5">
+        <v>51.8</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>73.2</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>352</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C5" s="5">
+        <v>49</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>62</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="C6" s="5"/>
+        <v>317</v>
+      </c>
+      <c r="C6" s="5">
+        <v>48.8</v>
+      </c>
       <c r="D6" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F6" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5" t="s">
-        <v>0</v>
+      <c r="A7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C7" s="6">
+        <v>55</v>
+      </c>
+      <c r="D7" s="6">
+        <v>53</v>
+      </c>
+      <c r="E7" s="6">
+        <v>57.1</v>
+      </c>
+      <c r="F7" s="6">
+        <v>50.2</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>0</v>
+      <c r="A8" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="6">
+        <v>73.7</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6">
+        <v>52.9</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="23" t="s">
-        <v>343</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6"/>
+      <c r="B9" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C9" s="6">
+        <v>54</v>
+      </c>
+      <c r="D9" s="6">
+        <v>56</v>
+      </c>
+      <c r="E9" s="6">
+        <v>50</v>
+      </c>
+      <c r="F9" s="6">
+        <v>55</v>
+      </c>
       <c r="J9" s="21"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>353</v>
-      </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="B10" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C10" s="6">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="D10" s="6">
+        <v>64.7</v>
+      </c>
+      <c r="E10" s="6">
+        <v>50.3</v>
+      </c>
+      <c r="F10" s="6">
+        <v>68.7</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="C11" s="5">
+        <v>62.8</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>70.2</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="C12" s="5">
+        <v>67.8</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>75.2</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -2854,11 +2919,15 @@
       <c r="B13" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C13" s="5"/>
+      <c r="C13" s="5">
+        <v>57.8</v>
+      </c>
       <c r="D13" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E13" s="5"/>
+      <c r="E13" s="5">
+        <v>65.2</v>
+      </c>
       <c r="F13" s="5" t="s">
         <v>0</v>
       </c>
@@ -2870,11 +2939,15 @@
       <c r="B14" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="C14" s="5"/>
+      <c r="C14" s="5">
+        <v>59</v>
+      </c>
       <c r="D14" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="5"/>
+      <c r="E14" s="5">
+        <v>58</v>
+      </c>
       <c r="F14" s="5" t="s">
         <v>0</v>
       </c>
@@ -2886,11 +2959,15 @@
       <c r="B15" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="C15" s="5"/>
+      <c r="C15" s="5">
+        <v>64</v>
+      </c>
       <c r="D15" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="5"/>
+      <c r="E15" s="5">
+        <v>63</v>
+      </c>
       <c r="F15" s="5" t="s">
         <v>0</v>
       </c>
@@ -2902,11 +2979,15 @@
       <c r="B16" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="C16" s="5"/>
+      <c r="C16" s="5">
+        <v>54</v>
+      </c>
       <c r="D16" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5">
+        <v>53</v>
+      </c>
       <c r="F16" s="5" t="s">
         <v>0</v>
       </c>
@@ -2918,11 +2999,15 @@
       <c r="B17" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="C17" s="5"/>
+      <c r="C17" s="5">
+        <v>58.8</v>
+      </c>
       <c r="D17" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E17" s="5"/>
+      <c r="E17" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F17" s="5" t="s">
         <v>0</v>
       </c>
@@ -2934,11 +3019,15 @@
       <c r="B18" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="C18" s="5"/>
+      <c r="C18" s="5">
+        <v>63.8</v>
+      </c>
       <c r="D18" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="F18" s="5" t="s">
         <v>0</v>
       </c>
@@ -2950,7 +3039,9 @@
       <c r="B19" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="C19" s="5"/>
+      <c r="C19" s="5">
+        <v>53.8</v>
+      </c>
       <c r="D19" s="5" t="s">
         <v>0</v>
       </c>
@@ -2968,12 +3059,14 @@
       <c r="B20" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C20" s="5"/>
+      <c r="C20" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D20" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>0</v>
+      <c r="E20" s="5">
+        <v>59.2</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>0</v>
@@ -2986,132 +3079,176 @@
       <c r="B21" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="C21" s="5"/>
+      <c r="C21" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D21" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>0</v>
+      <c r="E21" s="5">
+        <v>55</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="s">
+      <c r="A22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5" t="s">
+      <c r="C22" s="6">
+        <v>37</v>
+      </c>
+      <c r="D22" s="6">
+        <v>40</v>
+      </c>
+      <c r="E22" s="6">
+        <v>46</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="2" t="s">
+      <c r="A23" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5" t="s">
+      <c r="C23" s="6">
+        <v>47</v>
+      </c>
+      <c r="D23" s="6">
+        <v>45</v>
+      </c>
+      <c r="E23" s="6">
+        <v>50</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>349</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C24" s="5">
+        <v>57</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="3" t="s">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6" t="s">
+      <c r="C25" s="5">
+        <v>58.8</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>348</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C26" s="5">
+        <v>67.8</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5">
+        <v>47.2</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>354</v>
-      </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
+      <c r="A27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C27" s="5">
+        <v>64</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
+        <v>333</v>
+      </c>
+      <c r="C28" s="6">
+        <v>51</v>
+      </c>
+      <c r="D28" s="6">
+        <v>45</v>
+      </c>
+      <c r="E28" s="6">
+        <v>47</v>
+      </c>
       <c r="F28" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>346</v>
-      </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5" t="s">
+      <c r="A29" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C29" s="6">
+        <v>46</v>
+      </c>
+      <c r="D29" s="6">
+        <v>40</v>
+      </c>
+      <c r="E29" s="6">
+        <v>42</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -3120,14 +3257,16 @@
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="C30" s="5"/>
+        <v>335</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D30" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>0</v>
+      <c r="E30" s="5">
+        <v>53.2</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>0</v>
@@ -3138,13 +3277,17 @@
         <v>20</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="C31" s="5"/>
+        <v>336</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D31" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E31" s="5"/>
+      <c r="E31" s="5">
+        <v>53.2</v>
+      </c>
       <c r="F31" s="5" t="s">
         <v>0</v>
       </c>
@@ -3154,258 +3297,401 @@
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="C32" s="5"/>
+        <v>337</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D32" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>0</v>
+      <c r="E32" s="5">
+        <v>50</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>350</v>
-      </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
+      <c r="A33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5">
+        <v>50</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="23" t="s">
-        <v>344</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F34" s="6"/>
+      <c r="B34" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="C34" s="6">
+        <v>48.5</v>
+      </c>
+      <c r="D34" s="6">
+        <v>48.5</v>
+      </c>
+      <c r="E34" s="6">
+        <v>45</v>
+      </c>
+      <c r="F34" s="6">
+        <v>46.7</v>
+      </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B35" s="23" t="s">
-        <v>351</v>
-      </c>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
+      <c r="B35" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="6">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" s="6">
+        <v>51.5</v>
+      </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6" t="s">
-        <v>0</v>
+      <c r="B36" s="30" t="s">
+        <v>348</v>
+      </c>
+      <c r="C36" s="6">
+        <v>50</v>
+      </c>
+      <c r="D36" s="6">
+        <v>44.4</v>
+      </c>
+      <c r="E36" s="6">
+        <v>50.8</v>
+      </c>
+      <c r="F36" s="6">
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6" t="s">
-        <v>0</v>
+      <c r="B37" s="30" t="s">
+        <v>349</v>
+      </c>
+      <c r="C37" s="6">
+        <v>47.4</v>
+      </c>
+      <c r="D37" s="6">
+        <v>45</v>
+      </c>
+      <c r="E37" s="6">
+        <v>55</v>
+      </c>
+      <c r="F37" s="6">
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5" t="s">
-        <v>0</v>
+      <c r="A38" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>350</v>
+      </c>
+      <c r="C38" s="6">
+        <v>51.6</v>
+      </c>
+      <c r="D38" s="6">
+        <v>49</v>
+      </c>
+      <c r="E38" s="6">
+        <v>50</v>
+      </c>
+      <c r="F38" s="6">
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5" t="s">
-        <v>0</v>
+      <c r="A39" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39" s="30" t="s">
+        <v>351</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F39" s="6">
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5" t="s">
-        <v>0</v>
+      <c r="A40" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40" s="30" t="s">
+        <v>352</v>
+      </c>
+      <c r="C40" s="6">
+        <v>56</v>
+      </c>
+      <c r="D40" s="6">
+        <v>46</v>
+      </c>
+      <c r="E40" s="6">
+        <v>46</v>
+      </c>
+      <c r="F40" s="6">
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5" t="s">
-        <v>0</v>
+      <c r="A41" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B41" s="30" t="s">
+        <v>353</v>
+      </c>
+      <c r="C41" s="6">
+        <v>46</v>
+      </c>
+      <c r="D41" s="6">
+        <v>40</v>
+      </c>
+      <c r="E41" s="6">
+        <v>46</v>
+      </c>
+      <c r="F41" s="6">
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
+      <c r="B42" s="30" t="s">
+        <v>354</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D42" s="6">
+        <v>44.8</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F42" s="6">
+        <v>78.099999999999994</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B43" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="6">
+        <v>45.6</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6">
+        <v>77.8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B44" s="30" t="s">
+        <v>356</v>
+      </c>
+      <c r="C44" s="6">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="D44" s="6">
+        <v>42.8</v>
+      </c>
+      <c r="E44" s="6">
+        <v>69.2</v>
+      </c>
+      <c r="F44" s="6">
+        <v>60.2</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B45" s="30" t="s">
+        <v>357</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D45" s="6">
+        <v>41</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F45" s="6">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="11" t="s">
+      <c r="B47" s="25"/>
+      <c r="C47" s="26"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B48" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="C46" s="6">
+      <c r="C48" s="6">
         <v>14.8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C47" s="6">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C48" s="6">
-        <v>6.5</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C49" s="6">
-        <v>9.4</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C50" s="6">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C51" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="C50" s="6">
+      <c r="C52" s="6">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="12" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B54" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="C52" s="7">
+      <c r="C54" s="7">
         <v>14.2</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="12"/>
-      <c r="B53" s="4" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="12"/>
+      <c r="B55" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="C53" s="7">
+      <c r="C55" s="7">
         <v>18.7</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>345</v>
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="C57" s="5">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B59" s="28" t="s">
+        <v>359</v>
+      </c>
+      <c r="C59" s="29">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>341</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A47:C47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3421,16 +3707,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3481,16 +3767,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="25"/>
-      <c r="N4" s="25"/>
-      <c r="O4" s="25"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="25"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3517,14 +3803,14 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
-      <c r="O5" s="25"/>
-      <c r="P5" s="25"/>
-      <c r="Q5" s="25"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -3631,11 +3917,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -3728,12 +4014,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3848,11 +4134,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -3923,12 +4209,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4043,11 +4329,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4121,14 +4407,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4589,11 +4875,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4726,12 +5012,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4844,11 +5130,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -4958,12 +5244,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5062,11 +5348,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5185,14 +5471,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5593,11 +5879,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5712,12 +5998,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
Add new YMML data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55EB8D43-B4D4-40E1-8FFB-99C5AACE3EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE02067-7911-4922-9A1C-AAC175C8CA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="11" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="12" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="YBTL" sheetId="18" r:id="rId10"/>
     <sheet name="YWLM" sheetId="19" r:id="rId11"/>
     <sheet name="YPAD" sheetId="20" r:id="rId12"/>
+    <sheet name="YMML" sheetId="21" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="376">
   <si>
     <t>-</t>
   </si>
@@ -1133,6 +1134,54 @@
   </si>
   <si>
     <t>RNP (All - PADWQ, PADWP, PADWO)</t>
+  </si>
+  <si>
+    <t>Data is incomplete as the SOPs data currently uses historical data.</t>
+  </si>
+  <si>
+    <t>RWY 09</t>
+  </si>
+  <si>
+    <t>RWY 16</t>
+  </si>
+  <si>
+    <t>RWY 27</t>
+  </si>
+  <si>
+    <t>RWY 34</t>
+  </si>
+  <si>
+    <t>No STAR - Vectors to IAF (MENOG FF)</t>
+  </si>
+  <si>
+    <t>Runway 09</t>
+  </si>
+  <si>
+    <t>Runway 27</t>
+  </si>
+  <si>
+    <t>Runway 34</t>
+  </si>
+  <si>
+    <t>Runway 16</t>
+  </si>
+  <si>
+    <t>GUPUG</t>
+  </si>
+  <si>
+    <t>BELTA</t>
+  </si>
+  <si>
+    <t>VISAS</t>
+  </si>
+  <si>
+    <t>AKDEL</t>
+  </si>
+  <si>
+    <t>PORTS A STAR (LATTA FF)</t>
+  </si>
+  <si>
+    <t>PORTS A STAR (EKKAS FF)</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1313,6 +1362,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1328,12 +1382,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1676,13 +1724,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1921,11 +1969,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -2035,12 +2083,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2209,11 +2257,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2314,12 +2362,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2374,16 +2422,16 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="26" t="s">
         <v>290</v>
       </c>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -2398,14 +2446,14 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -2420,14 +2468,14 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -2442,14 +2490,14 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="23"/>
-      <c r="M9" s="23"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -2464,14 +2512,14 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -2486,14 +2534,14 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -2580,11 +2628,11 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -2704,14 +2752,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3376,7 +3424,7 @@
       <c r="A36" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="3" t="s">
         <v>348</v>
       </c>
       <c r="C36" s="6">
@@ -3396,7 +3444,7 @@
       <c r="A37" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="3" t="s">
         <v>349</v>
       </c>
       <c r="C37" s="6">
@@ -3416,7 +3464,7 @@
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B38" s="30" t="s">
+      <c r="B38" s="3" t="s">
         <v>350</v>
       </c>
       <c r="C38" s="6">
@@ -3436,7 +3484,7 @@
       <c r="A39" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B39" s="30" t="s">
+      <c r="B39" s="3" t="s">
         <v>351</v>
       </c>
       <c r="C39" s="6" t="s">
@@ -3456,7 +3504,7 @@
       <c r="A40" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B40" s="30" t="s">
+      <c r="B40" s="3" t="s">
         <v>352</v>
       </c>
       <c r="C40" s="6">
@@ -3476,7 +3524,7 @@
       <c r="A41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B41" s="30" t="s">
+      <c r="B41" s="3" t="s">
         <v>353</v>
       </c>
       <c r="C41" s="6">
@@ -3496,7 +3544,7 @@
       <c r="A42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="30" t="s">
+      <c r="B42" s="3" t="s">
         <v>354</v>
       </c>
       <c r="C42" s="6" t="s">
@@ -3516,7 +3564,7 @@
       <c r="A43" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B43" s="30" t="s">
+      <c r="B43" s="3" t="s">
         <v>355</v>
       </c>
       <c r="C43" s="6" t="s">
@@ -3536,7 +3584,7 @@
       <c r="A44" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="3" t="s">
         <v>356</v>
       </c>
       <c r="C44" s="6">
@@ -3556,7 +3604,7 @@
       <c r="A45" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B45" s="30" t="s">
+      <c r="B45" s="3" t="s">
         <v>357</v>
       </c>
       <c r="C45" s="6" t="s">
@@ -3573,11 +3621,11 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="24" t="s">
+      <c r="A47" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="29"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
@@ -3673,13 +3721,13 @@
       <c r="C58" s="1"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="27" t="s">
+      <c r="A59" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B59" s="28" t="s">
+      <c r="B59" s="23" t="s">
         <v>359</v>
       </c>
-      <c r="C59" s="29">
+      <c r="C59" s="24">
         <v>14.3</v>
       </c>
     </row>
@@ -3692,6 +3740,176 @@
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A47:C47"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB965F8-E493-4C2F-8F83-E7C5A76D760C}">
+  <dimension ref="A2:I42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C4" s="5">
+        <v>55.7</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C5" s="5">
+        <v>59.7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C6" s="5">
+        <v>40</v>
+      </c>
+      <c r="D6" s="5">
+        <v>64</v>
+      </c>
+      <c r="E6" s="5">
+        <v>42.7</v>
+      </c>
+      <c r="F6" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="C29" s="8">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C30" s="8">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="C31" s="8">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="C32" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>266</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3707,16 +3925,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -3767,16 +3985,16 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3803,14 +4021,14 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="26"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -3917,11 +4135,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
@@ -4014,12 +4232,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4134,11 +4352,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4209,12 +4427,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4329,11 +4547,11 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
@@ -4407,14 +4625,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -4875,11 +5093,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5012,12 +5230,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5130,11 +5348,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5244,12 +5462,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5348,11 +5566,11 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5471,14 +5689,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -5879,11 +6097,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="26"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
@@ -5998,12 +6216,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
Add YPPH OLMAM feeder fix
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE02067-7911-4922-9A1C-AAC175C8CA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9E1CAA-1253-4AE4-93E5-447A966EAFC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="12" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="7" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="377">
   <si>
     <t>-</t>
   </si>
@@ -1182,6 +1182,9 @@
   </si>
   <si>
     <t>PORTS A STAR (EKKAS FF)</t>
+  </si>
+  <si>
+    <t>No STAR - Vectors to IAF (OLMAM FF)</t>
   </si>
 </sst>
 </file>
@@ -1367,12 +1370,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1381,6 +1378,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1717,22 +1720,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
   <dimension ref="A2:E42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1747,7 +1750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1764,7 +1767,7 @@
         <v>68.099999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1781,7 +1784,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1798,7 +1801,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1815,7 +1818,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1832,7 +1835,7 @@
         <v>57.5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>64.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -1866,7 +1869,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -1883,7 +1886,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1900,7 +1903,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1917,7 +1920,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1934,7 +1937,7 @@
         <v>43.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1951,7 +1954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1968,14 +1971,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
@@ -1986,7 +1989,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1995,7 +1998,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -2004,7 +2007,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -2013,12 +2016,12 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="12" t="s">
         <v>26</v>
       </c>
@@ -2029,7 +2032,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>22</v>
@@ -2038,7 +2041,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>23</v>
@@ -2047,7 +2050,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>24</v>
@@ -2056,7 +2059,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2073,24 +2076,24 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2102,7 +2105,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2116,7 +2119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2130,7 +2133,7 @@
         <v>41.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2144,7 +2147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2158,7 +2161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2172,7 +2175,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2186,7 +2189,7 @@
         <v>44.9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2200,7 +2203,7 @@
         <v>52.5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2214,7 +2217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2228,7 +2231,7 @@
         <v>63.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2242,7 +2245,7 @@
         <v>53.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2256,14 +2259,14 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>247</v>
       </c>
@@ -2274,7 +2277,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>250</v>
@@ -2283,7 +2286,7 @@
         <v>19.3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>251</v>
@@ -2292,7 +2295,7 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>252</v>
@@ -2301,12 +2304,12 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12" t="s">
         <v>248</v>
       </c>
@@ -2317,7 +2320,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
         <v>253</v>
@@ -2326,7 +2329,7 @@
         <v>19.899999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>254</v>
@@ -2335,7 +2338,7 @@
         <v>24.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>266</v>
       </c>
@@ -2352,24 +2355,24 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49864E6F-5D2D-438C-A891-0771B0E2C7F9}">
   <dimension ref="A2:M42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2381,7 +2384,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2395,7 +2398,7 @@
         <v>24.1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2409,7 +2412,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2422,18 +2425,18 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="29"/>
+      <c r="M6" s="29"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2446,16 +2449,16 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+      <c r="L7" s="29"/>
+      <c r="M7" s="29"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -2468,16 +2471,16 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="M8" s="26"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+      <c r="L8" s="29"/>
+      <c r="M8" s="29"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -2490,16 +2493,16 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="26"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -2512,16 +2515,16 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="29"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2534,16 +2537,16 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="29"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2557,7 +2560,7 @@
         <v>65.900000000000006</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2571,7 +2574,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2585,7 +2588,7 @@
         <v>43.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -2599,7 +2602,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -2613,7 +2616,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -2627,14 +2630,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>54</v>
       </c>
@@ -2645,7 +2648,7 @@
         <v>12.7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>268</v>
@@ -2654,7 +2657,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>269</v>
@@ -2663,7 +2666,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>286</v>
@@ -2672,12 +2675,12 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12" t="s">
         <v>57</v>
       </c>
@@ -2688,7 +2691,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
         <v>271</v>
@@ -2697,7 +2700,7 @@
         <v>20.9</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>275</v>
@@ -2706,7 +2709,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>272</v>
@@ -2715,7 +2718,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>273</v>
@@ -2724,7 +2727,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>266</v>
       </c>
@@ -2742,26 +2745,26 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
   <dimension ref="A2:J61"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="37.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -2779,7 +2782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2799,7 +2802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2819,7 +2822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -2839,7 +2842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -2859,7 +2862,7 @@
         <v>50.2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -2879,7 +2882,7 @@
         <v>52.9</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
@@ -2900,7 +2903,7 @@
       </c>
       <c r="J9" s="21"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
@@ -2920,7 +2923,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2940,7 +2943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -2960,7 +2963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2980,7 +2983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3000,7 +3003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -3020,7 +3023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -3040,7 +3043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -3060,7 +3063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -3080,7 +3083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -3100,7 +3103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -3120,7 +3123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3140,7 +3143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
@@ -3160,7 +3163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="3" t="s">
         <v>3</v>
       </c>
@@ -3180,7 +3183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -3200,7 +3203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -3220,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -3240,7 +3243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -3260,7 +3263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
@@ -3280,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>3</v>
       </c>
@@ -3300,7 +3303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -3320,7 +3323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -3340,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -3360,7 +3363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -3380,7 +3383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34" s="3" t="s">
         <v>3</v>
       </c>
@@ -3400,7 +3403,7 @@
         <v>46.7</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
         <v>3</v>
       </c>
@@ -3420,7 +3423,7 @@
         <v>51.5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
         <v>3</v>
       </c>
@@ -3440,7 +3443,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>3</v>
       </c>
@@ -3460,7 +3463,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
@@ -3480,7 +3483,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>3</v>
       </c>
@@ -3500,7 +3503,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>3</v>
       </c>
@@ -3520,7 +3523,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
         <v>3</v>
       </c>
@@ -3540,7 +3543,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
         <v>3</v>
       </c>
@@ -3560,7 +3563,7 @@
         <v>78.099999999999994</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>3</v>
       </c>
@@ -3580,7 +3583,7 @@
         <v>77.8</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" s="3" t="s">
         <v>3</v>
       </c>
@@ -3600,7 +3603,7 @@
         <v>60.2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" s="3" t="s">
         <v>3</v>
       </c>
@@ -3620,14 +3623,14 @@
         <v>72.8</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="27" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="28"/>
-      <c r="C47" s="29"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B47" s="26"/>
+      <c r="C47" s="27"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48" s="11" t="s">
         <v>291</v>
       </c>
@@ -3638,7 +3641,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A49" s="3"/>
       <c r="B49" s="3" t="s">
         <v>294</v>
@@ -3647,7 +3650,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A50" s="3"/>
       <c r="B50" s="3" t="s">
         <v>295</v>
@@ -3656,7 +3659,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A51" s="3"/>
       <c r="B51" s="3" t="s">
         <v>296</v>
@@ -3665,7 +3668,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
         <v>297</v>
@@ -3674,12 +3677,12 @@
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A54" s="12" t="s">
         <v>292</v>
       </c>
@@ -3690,7 +3693,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A55" s="12"/>
       <c r="B55" s="4" t="s">
         <v>299</v>
@@ -3699,12 +3702,12 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A57" s="16" t="s">
         <v>57</v>
       </c>
@@ -3715,12 +3718,12 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A59" s="22" t="s">
         <v>54</v>
       </c>
@@ -3731,7 +3734,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>341</v>
       </c>
@@ -3748,26 +3751,26 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB965F8-E493-4C2F-8F83-E7C5A76D760C}">
   <dimension ref="A2:I42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="33.85546875" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="33.84375" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -3785,7 +3788,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3805,7 +3808,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3825,7 +3828,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -3845,19 +3848,19 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="I9" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="9" t="s">
         <v>366</v>
       </c>
@@ -3868,7 +3871,7 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="9" t="s">
         <v>369</v>
       </c>
@@ -3879,7 +3882,7 @@
         <v>11.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="9" t="s">
         <v>367</v>
       </c>
@@ -3890,7 +3893,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="9" t="s">
         <v>368</v>
       </c>
@@ -3901,7 +3904,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>266</v>
       </c>
@@ -3918,25 +3921,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3960,7 +3963,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -3985,18 +3988,18 @@
       <c r="H4" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="26" t="s">
+      <c r="J4" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="26"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4021,16 +4024,16 @@
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-      <c r="Q5" s="26"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4056,7 +4059,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4082,7 +4085,7 @@
         <v>65.7</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4108,7 +4111,7 @@
         <v>79.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4134,14 +4137,14 @@
         <v>81.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -4152,7 +4155,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="9" t="s">
         <v>36</v>
       </c>
@@ -4163,7 +4166,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9" t="s">
         <v>37</v>
       </c>
@@ -4174,7 +4177,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -4185,7 +4188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="9" t="s">
         <v>39</v>
       </c>
@@ -4196,7 +4199,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
@@ -4207,7 +4210,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4225,21 +4228,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4251,7 +4254,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4273,7 +4276,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4295,7 +4298,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4309,7 +4312,7 @@
         <v>39.700000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4323,7 +4326,7 @@
         <v>67.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4337,7 +4340,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4351,14 +4354,14 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -4369,7 +4372,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>56</v>
@@ -4378,12 +4381,12 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>57</v>
       </c>
@@ -4394,7 +4397,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>59</v>
@@ -4403,7 +4406,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4420,21 +4423,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>72</v>
@@ -4446,7 +4449,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4468,7 +4471,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4490,7 +4493,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4504,7 +4507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4518,7 +4521,7 @@
         <v>88.6</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4532,7 +4535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4546,14 +4549,14 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A19" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
         <v>66</v>
       </c>
@@ -4564,7 +4567,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>69</v>
@@ -4573,12 +4576,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
         <v>67</v>
       </c>
@@ -4589,7 +4592,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>71</v>
@@ -4598,7 +4601,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4615,26 +4618,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4652,7 +4655,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4672,7 +4675,7 @@
         <v>98.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4692,7 +4695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4712,7 +4715,7 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4732,7 +4735,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4752,7 +4755,7 @@
         <v>93.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4772,7 +4775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4792,7 +4795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -4812,7 +4815,7 @@
         <v>92.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -4832,7 +4835,7 @@
         <v>88.4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4852,7 +4855,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4872,7 +4875,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -4892,7 +4895,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -4912,7 +4915,7 @@
         <v>41.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -4932,7 +4935,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -4952,7 +4955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -4972,7 +4975,7 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4992,7 +4995,7 @@
         <v>45.4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -5012,7 +5015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -5032,7 +5035,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -5052,7 +5055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -5072,7 +5075,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -5092,14 +5095,14 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>103</v>
       </c>
@@ -5110,7 +5113,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>108</v>
@@ -5119,12 +5122,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>104</v>
       </c>
@@ -5135,7 +5138,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
         <v>119</v>
@@ -5144,7 +5147,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
         <v>110</v>
@@ -5153,12 +5156,12 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="9"/>
       <c r="B35" s="1"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14" t="s">
         <v>105</v>
       </c>
@@ -5169,7 +5172,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
         <v>112</v>
@@ -5178,12 +5181,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="9"/>
       <c r="B38" s="1"/>
       <c r="C38" s="8"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" s="16" t="s">
         <v>106</v>
       </c>
@@ -5194,7 +5197,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>114</v>
@@ -5203,7 +5206,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5220,24 +5223,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -5249,7 +5252,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -5263,7 +5266,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5277,7 +5280,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -5291,7 +5294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5305,7 +5308,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5319,7 +5322,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -5333,7 +5336,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -5347,14 +5350,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>123</v>
       </c>
@@ -5365,7 +5368,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>126</v>
@@ -5374,7 +5377,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>127</v>
@@ -5383,7 +5386,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>128</v>
@@ -5392,7 +5395,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>129</v>
@@ -5401,12 +5404,12 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>124</v>
       </c>
@@ -5417,7 +5420,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>131</v>
@@ -5426,7 +5429,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>139</v>
@@ -5435,7 +5438,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5452,24 +5455,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5481,7 +5484,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -5495,7 +5498,7 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5509,7 +5512,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -5523,7 +5526,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5537,7 +5540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5551,7 +5554,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -5565,14 +5568,14 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>140</v>
       </c>
@@ -5583,7 +5586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>143</v>
@@ -5592,7 +5595,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>144</v>
@@ -5601,7 +5604,7 @@
         <v>19.100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>145</v>
@@ -5610,7 +5613,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>146</v>
@@ -5619,12 +5622,12 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="12" t="s">
         <v>141</v>
       </c>
@@ -5635,7 +5638,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>148</v>
@@ -5644,7 +5647,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>145</v>
@@ -5653,7 +5656,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>144</v>
@@ -5662,7 +5665,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5679,26 +5682,26 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5716,7 +5719,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -5736,7 +5739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -5756,7 +5759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -5776,7 +5779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5796,7 +5799,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -5816,7 +5819,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -5836,7 +5839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -5856,7 +5859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -5876,7 +5879,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -5896,7 +5899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>2</v>
       </c>
@@ -5916,7 +5919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -5936,7 +5939,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -5956,7 +5959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -5976,7 +5979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -5996,7 +5999,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -6016,7 +6019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -6036,7 +6039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -6056,7 +6059,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -6076,7 +6079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -6096,14 +6099,34 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C23" s="5">
+        <v>35</v>
+      </c>
+      <c r="D23" s="5">
+        <v>40</v>
+      </c>
+      <c r="E23" s="5">
+        <v>56</v>
+      </c>
+      <c r="F23" s="5">
+        <v>59.4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="11" t="s">
         <v>160</v>
       </c>
@@ -6114,7 +6137,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>164</v>
@@ -6123,12 +6146,12 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="12" t="s">
         <v>161</v>
       </c>
@@ -6139,12 +6162,12 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="9"/>
       <c r="B33" s="1"/>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="14" t="s">
         <v>162</v>
       </c>
@@ -6155,7 +6178,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>172</v>
@@ -6164,7 +6187,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>173</v>
@@ -6173,12 +6196,12 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="9"/>
       <c r="B37" s="1"/>
       <c r="C37" s="8"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="16" t="s">
         <v>163</v>
       </c>
@@ -6189,7 +6212,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -6206,24 +6229,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
   <dimension ref="A2:D70"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" customWidth="1"/>
+    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="3" max="4" width="9.53515625" customWidth="1"/>
+    <col min="5" max="5" width="9.3828125" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -6235,7 +6258,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -6249,7 +6272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6263,7 +6286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -6277,7 +6300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -6291,7 +6314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -6305,7 +6328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -6319,7 +6342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -6333,7 +6356,7 @@
         <v>97.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -6347,7 +6370,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6361,7 +6384,7 @@
         <v>50.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -6375,7 +6398,7 @@
         <v>56.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6389,7 +6412,7 @@
         <v>104.9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -6403,7 +6426,7 @@
         <v>94.9</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -6417,7 +6440,7 @@
         <v>113.9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -6431,7 +6454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -6445,7 +6468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -6459,7 +6482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -6473,7 +6496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -6487,7 +6510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -6501,7 +6524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -6515,7 +6538,7 @@
         <v>109.9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -6529,7 +6552,7 @@
         <v>105.9</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -6543,7 +6566,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -6557,7 +6580,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -6571,7 +6594,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -6585,7 +6608,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -6599,7 +6622,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -6613,7 +6636,7 @@
         <v>81.900000000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -6627,7 +6650,7 @@
         <v>77.900000000000006</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -6641,7 +6664,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -6655,7 +6678,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -6669,7 +6692,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -6683,7 +6706,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -6697,7 +6720,7 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -6711,7 +6734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -6723,7 +6746,7 @@
       </c>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -6735,7 +6758,7 @@
       </c>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -6749,7 +6772,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -6763,7 +6786,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -6777,7 +6800,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -6791,7 +6814,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -6805,7 +6828,7 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
@@ -6819,7 +6842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
@@ -6833,7 +6856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -6847,7 +6870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
@@ -6861,7 +6884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -6875,7 +6898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -6889,7 +6912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="2" t="s">
         <v>20</v>
       </c>
@@ -6903,7 +6926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="2" t="s">
         <v>20</v>
       </c>
@@ -6917,7 +6940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
         <v>20</v>
       </c>
@@ -6931,14 +6954,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B56" s="19"/>
       <c r="C56" s="20"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A57" s="11" t="s">
         <v>192</v>
       </c>
@@ -6949,7 +6972,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>198</v>
@@ -6958,7 +6981,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A59" s="3"/>
       <c r="B59" s="3" t="s">
         <v>199</v>
@@ -6967,7 +6990,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="3"/>
       <c r="B60" s="3" t="s">
         <v>195</v>
@@ -6976,7 +6999,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="3"/>
       <c r="B61" s="3" t="s">
         <v>197</v>
@@ -6985,12 +7008,12 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="12" t="s">
         <v>193</v>
       </c>
@@ -7001,7 +7024,7 @@
         <v>22.9</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="12"/>
       <c r="B64" s="4" t="s">
         <v>201</v>
@@ -7010,7 +7033,7 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A65" s="12"/>
       <c r="B65" s="4" t="s">
         <v>200</v>
@@ -7019,7 +7042,7 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A66" s="12"/>
       <c r="B66" s="4" t="s">
         <v>202</v>
@@ -7028,7 +7051,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>311</v>
       </c>

</xml_diff>

<commit_message>
Replace YSSY ODALE STAR with AKMIR STAR
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\GitHub\image-source-files\flow-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9E1CAA-1253-4AE4-93E5-447A966EAFC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6708F3B4-6412-4E69-BDD4-D9CF33C4DA1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="7" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="378">
   <si>
     <t>-</t>
   </si>
@@ -782,9 +782,6 @@
     <t>MEPIL (YAKKA FF)</t>
   </si>
   <si>
-    <t>ODALE (WELSH FF)</t>
-  </si>
-  <si>
     <t>ANUPA A/X (SUDAG FF)</t>
   </si>
   <si>
@@ -1185,6 +1182,12 @@
   </si>
   <si>
     <t>No STAR - Vectors to IAF (OLMAM FF)</t>
+  </si>
+  <si>
+    <t>Last edit 1st May 2026 on DAP 187</t>
+  </si>
+  <si>
+    <t>AKMIR</t>
   </si>
 </sst>
 </file>
@@ -1370,6 +1373,12 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1378,12 +1387,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1720,22 +1723,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6375F09E-4F8C-4C4B-B3AA-29BB7C841182}">
   <dimension ref="A2:E42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -1750,7 +1753,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1767,7 +1770,7 @@
         <v>68.099999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1784,7 +1787,7 @@
         <v>67.099999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1801,7 +1804,7 @@
         <v>59.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1818,7 +1821,7 @@
         <v>64.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1835,7 +1838,7 @@
         <v>57.5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -1852,7 +1855,7 @@
         <v>64.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -1869,7 +1872,7 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -1886,7 +1889,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1903,7 +1906,7 @@
         <v>55.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1920,7 +1923,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -1937,7 +1940,7 @@
         <v>43.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -1954,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1971,14 +1974,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="28" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>21</v>
       </c>
@@ -1989,7 +1992,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1998,7 +2001,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -2007,7 +2010,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -2016,12 +2019,12 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>26</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="4" t="s">
         <v>22</v>
@@ -2041,7 +2044,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
         <v>23</v>
@@ -2050,7 +2053,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4" t="s">
         <v>24</v>
@@ -2059,7 +2062,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -2076,41 +2079,41 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C4" s="5">
         <v>72.5</v>
@@ -2119,12 +2122,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>0</v>
@@ -2133,12 +2136,12 @@
         <v>41.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C6" s="5">
         <v>58.2</v>
@@ -2147,12 +2150,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C7" s="5">
         <v>51.5</v>
@@ -2161,12 +2164,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -2175,12 +2178,12 @@
         <v>53.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C9" s="5">
         <v>43.5</v>
@@ -2189,12 +2192,12 @@
         <v>44.9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -2203,12 +2206,12 @@
         <v>52.5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C11" s="5">
         <v>38.5</v>
@@ -2217,12 +2220,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -2231,12 +2234,12 @@
         <v>63.5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C13" s="5">
         <v>38.5</v>
@@ -2245,12 +2248,12 @@
         <v>53.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -2259,59 +2262,59 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C29" s="6">
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C30" s="6">
         <v>19.3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C31" s="6">
         <v>21.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C32" s="6">
         <v>19.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>142</v>
@@ -2320,27 +2323,27 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C35" s="7">
         <v>19.899999999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C36" s="7">
         <v>24.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2355,24 +2358,24 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49864E6F-5D2D-438C-A891-0771B0E2C7F9}">
   <dimension ref="A2:M42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -2384,12 +2387,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C4" s="5">
         <v>63.5</v>
@@ -2398,12 +2401,12 @@
         <v>24.1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C5" s="5">
         <v>48.5</v>
@@ -2412,12 +2415,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>0</v>
@@ -2425,23 +2428,23 @@
       <c r="D6" s="5">
         <v>27.5</v>
       </c>
-      <c r="F6" s="29" t="s">
-        <v>290</v>
-      </c>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F6" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>0</v>
@@ -2449,21 +2452,21 @@
       <c r="D7" s="5">
         <v>28.5</v>
       </c>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
-      <c r="K7" s="29"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="29"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -2471,21 +2474,21 @@
       <c r="D8" s="5">
         <v>32.5</v>
       </c>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -2493,21 +2496,21 @@
       <c r="D9" s="5">
         <v>28</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
-      <c r="K9" s="29"/>
-      <c r="L9" s="29"/>
-      <c r="M9" s="29"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -2515,21 +2518,21 @@
       <c r="D10" s="5">
         <v>29</v>
       </c>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="29"/>
-      <c r="L10" s="29"/>
-      <c r="M10" s="29"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>0</v>
@@ -2537,21 +2540,21 @@
       <c r="D11" s="5">
         <v>33</v>
       </c>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
-      <c r="M11" s="29"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C12" s="5">
         <v>31.5</v>
@@ -2560,12 +2563,12 @@
         <v>65.900000000000006</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C13" s="5">
         <v>41.7</v>
@@ -2574,12 +2577,12 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C14" s="5">
         <v>28.6</v>
@@ -2588,12 +2591,12 @@
         <v>43.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C15" s="5">
         <v>28.5</v>
@@ -2602,12 +2605,12 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C16" s="5">
         <v>44.5</v>
@@ -2616,12 +2619,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C17" s="5">
         <v>34.5</v>
@@ -2630,106 +2633,106 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>54</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C29" s="6">
         <v>12.7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C30" s="6">
         <v>16.5</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C31" s="6">
         <v>16.5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C32" s="6">
         <v>9.6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>57</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C34" s="7">
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C35" s="7">
         <v>20.9</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C36" s="7">
         <v>14.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C37" s="7">
         <v>14.8</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C38" s="7">
         <v>9.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2745,49 +2748,49 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
   <dimension ref="A2:J61"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="37.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="37.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>53</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C4" s="5">
         <v>51.8</v>
@@ -2802,12 +2805,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C5" s="5">
         <v>49</v>
@@ -2822,12 +2825,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C6" s="5">
         <v>48.8</v>
@@ -2842,12 +2845,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C7" s="6">
         <v>55</v>
@@ -2862,12 +2865,12 @@
         <v>50.2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>0</v>
@@ -2882,12 +2885,12 @@
         <v>52.9</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C9" s="6">
         <v>54</v>
@@ -2903,12 +2906,12 @@
       </c>
       <c r="J9" s="21"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C10" s="6">
         <v>76.900000000000006</v>
@@ -2923,12 +2926,12 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C11" s="5">
         <v>62.8</v>
@@ -2943,12 +2946,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C12" s="5">
         <v>67.8</v>
@@ -2963,12 +2966,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C13" s="5">
         <v>57.8</v>
@@ -2983,12 +2986,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C14" s="5">
         <v>59</v>
@@ -3003,12 +3006,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C15" s="5">
         <v>64</v>
@@ -3023,12 +3026,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C16" s="5">
         <v>54</v>
@@ -3043,12 +3046,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C17" s="5">
         <v>58.8</v>
@@ -3063,12 +3066,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C18" s="5">
         <v>63.8</v>
@@ -3083,12 +3086,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C19" s="5">
         <v>53.8</v>
@@ -3103,12 +3106,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>0</v>
@@ -3123,12 +3126,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>0</v>
@@ -3143,12 +3146,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C22" s="6">
         <v>37</v>
@@ -3163,12 +3166,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C23" s="6">
         <v>47</v>
@@ -3183,12 +3186,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C24" s="5">
         <v>57</v>
@@ -3203,12 +3206,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C25" s="5">
         <v>58.8</v>
@@ -3223,12 +3226,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C26" s="5">
         <v>67.8</v>
@@ -3243,12 +3246,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C27" s="5">
         <v>64</v>
@@ -3263,12 +3266,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C28" s="6">
         <v>51</v>
@@ -3283,12 +3286,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C29" s="6">
         <v>46</v>
@@ -3303,12 +3306,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>0</v>
@@ -3323,12 +3326,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>0</v>
@@ -3343,12 +3346,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -3363,12 +3366,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>0</v>
@@ -3383,12 +3386,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C34" s="6">
         <v>48.5</v>
@@ -3403,12 +3406,12 @@
         <v>46.7</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>0</v>
@@ -3423,12 +3426,12 @@
         <v>51.5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C36" s="6">
         <v>50</v>
@@ -3443,12 +3446,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C37" s="6">
         <v>47.4</v>
@@ -3463,12 +3466,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C38" s="6">
         <v>51.6</v>
@@ -3483,12 +3486,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>0</v>
@@ -3503,12 +3506,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C40" s="6">
         <v>56</v>
@@ -3523,12 +3526,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C41" s="6">
         <v>46</v>
@@ -3543,12 +3546,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>0</v>
@@ -3563,12 +3566,12 @@
         <v>78.099999999999994</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>0</v>
@@ -3583,12 +3586,12 @@
         <v>77.8</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C44" s="6">
         <v>35.799999999999997</v>
@@ -3603,12 +3606,12 @@
         <v>60.2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>0</v>
@@ -3623,120 +3626,120 @@
         <v>72.8</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A47" s="25" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="26"/>
-      <c r="C47" s="27"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B47" s="28"/>
+      <c r="C47" s="29"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C48" s="6">
         <v>14.8</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C49" s="6">
         <v>15.8</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C50" s="6">
         <v>6.5</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C51" s="6">
         <v>9.4</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C52" s="6">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C54" s="7">
         <v>14.2</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="12"/>
       <c r="B55" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C55" s="7">
         <v>18.7</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>57</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C57" s="5">
         <v>18.5</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="22" t="s">
         <v>54</v>
       </c>
       <c r="B59" s="23" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C59" s="24">
         <v>14.3</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -3751,49 +3754,49 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB965F8-E493-4C2F-8F83-E7C5A76D760C}">
   <dimension ref="A2:I42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="33.84375" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C4" s="5">
         <v>55.7</v>
@@ -3808,12 +3811,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C5" s="5">
         <v>59.7</v>
@@ -3828,12 +3831,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C6" s="5">
         <v>40</v>
@@ -3848,65 +3851,65 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C29" s="8">
         <v>10.7</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C30" s="8">
         <v>11.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C31" s="8">
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C32" s="8">
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3921,25 +3924,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738FA743-E210-4ACA-8A16-41DC9AE22AF2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -3963,188 +3966,188 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C4" s="5">
+        <v>67</v>
+      </c>
+      <c r="D4" s="5">
+        <v>105.4</v>
+      </c>
+      <c r="E4" s="5">
+        <v>91.6</v>
+      </c>
+      <c r="F4" s="5">
+        <v>96.9</v>
+      </c>
+      <c r="G4" s="5">
+        <v>93.9</v>
+      </c>
+      <c r="H4" s="5">
+        <v>104.7</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C5" s="5">
         <v>64.099999999999994</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D5" s="5">
         <v>43.8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E5" s="5">
         <v>42.3</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F5" s="5">
         <v>61.4</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G5" s="5">
         <v>78.099999999999994</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H5" s="5">
         <v>78.2</v>
       </c>
-      <c r="J4" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="26"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="C6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5">
         <v>42.4</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="29"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="29"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="F6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C7" s="5">
         <v>67.2</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D7" s="5">
         <v>47.1</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E7" s="5">
         <v>45.7</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F7" s="5">
         <v>62.7</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G7" s="5">
         <v>81.3</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H7" s="5">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C8" s="5">
         <v>69.2</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D8" s="5">
         <v>73.599999999999994</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E8" s="5">
         <v>77.3</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F8" s="5">
         <v>46.5</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G8" s="5">
         <v>80.599999999999994</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H8" s="5">
         <v>65.7</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C9" s="5">
         <v>42.6</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D9" s="5">
         <v>79.599999999999994</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E9" s="5">
         <v>67.3</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F9" s="5">
         <v>70.099999999999994</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G9" s="5">
         <v>63.9</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H9" s="5">
         <v>79.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="C9" s="5">
-        <v>44</v>
-      </c>
-      <c r="D9" s="5">
-        <v>82.4</v>
-      </c>
-      <c r="E9" s="5">
-        <v>68.599999999999994</v>
-      </c>
-      <c r="F9" s="5">
-        <v>73.900000000000006</v>
-      </c>
-      <c r="G9" s="5">
-        <v>70.900000000000006</v>
-      </c>
-      <c r="H9" s="5">
-        <v>81.7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="28" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -4155,7 +4158,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>36</v>
       </c>
@@ -4166,7 +4169,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>37</v>
       </c>
@@ -4177,7 +4180,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -4188,7 +4191,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>39</v>
       </c>
@@ -4199,7 +4202,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>40</v>
       </c>
@@ -4210,9 +4213,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>376</v>
       </c>
     </row>
   </sheetData>
@@ -4228,21 +4231,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4254,7 +4257,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4276,7 +4279,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4298,7 +4301,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4312,7 +4315,7 @@
         <v>39.700000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4326,7 +4329,7 @@
         <v>67.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4340,7 +4343,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4354,14 +4357,14 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="28" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>54</v>
       </c>
@@ -4372,7 +4375,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>56</v>
@@ -4381,12 +4384,12 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>57</v>
       </c>
@@ -4397,7 +4400,7 @@
         <v>10.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>59</v>
@@ -4406,7 +4409,7 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4423,21 +4426,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>72</v>
@@ -4449,7 +4452,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4471,7 +4474,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4493,7 +4496,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4507,7 +4510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4521,7 +4524,7 @@
         <v>88.6</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4535,7 +4538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4549,14 +4552,14 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="28" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>66</v>
       </c>
@@ -4567,7 +4570,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
         <v>69</v>
@@ -4576,12 +4579,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="1"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>67</v>
       </c>
@@ -4592,7 +4595,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
         <v>71</v>
@@ -4601,7 +4604,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -4618,26 +4621,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -4655,7 +4658,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -4675,7 +4678,7 @@
         <v>98.4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4695,7 +4698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -4715,7 +4718,7 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -4735,7 +4738,7 @@
         <v>70.3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -4755,7 +4758,7 @@
         <v>93.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -4775,7 +4778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -4795,7 +4798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -4815,7 +4818,7 @@
         <v>92.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -4835,7 +4838,7 @@
         <v>88.4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4855,7 +4858,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4875,7 +4878,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -4895,7 +4898,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -4915,7 +4918,7 @@
         <v>41.9</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -4935,7 +4938,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -4955,7 +4958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -4975,7 +4978,7 @@
         <v>45.3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -4995,7 +4998,7 @@
         <v>45.4</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -5015,7 +5018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -5035,7 +5038,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -5055,7 +5058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -5075,7 +5078,7 @@
         <v>62.4</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -5095,14 +5098,14 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>103</v>
       </c>
@@ -5113,7 +5116,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>108</v>
@@ -5122,12 +5125,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>104</v>
       </c>
@@ -5138,7 +5141,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
         <v>119</v>
@@ -5147,7 +5150,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
         <v>110</v>
@@ -5156,12 +5159,12 @@
         <v>11.7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="B35" s="1"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>105</v>
       </c>
@@ -5172,7 +5175,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
         <v>112</v>
@@ -5181,12 +5184,12 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
       <c r="B38" s="1"/>
       <c r="C38" s="8"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>106</v>
       </c>
@@ -5197,7 +5200,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
         <v>114</v>
@@ -5206,7 +5209,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5223,24 +5226,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>120</v>
@@ -5252,7 +5255,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -5266,7 +5269,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5280,7 +5283,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -5294,7 +5297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5308,7 +5311,7 @@
         <v>44.3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5322,7 +5325,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -5336,7 +5339,7 @@
         <v>68.7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -5350,14 +5353,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>123</v>
       </c>
@@ -5368,7 +5371,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>126</v>
@@ -5377,7 +5380,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>127</v>
@@ -5386,7 +5389,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>128</v>
@@ -5395,7 +5398,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>129</v>
@@ -5404,12 +5407,12 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>124</v>
       </c>
@@ -5420,7 +5423,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>131</v>
@@ -5429,7 +5432,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>139</v>
@@ -5438,7 +5441,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5455,24 +5458,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5484,12 +5487,12 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C4" s="5">
         <v>48.4</v>
@@ -5498,7 +5501,7 @@
         <v>82.4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5512,7 +5515,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -5526,7 +5529,7 @@
         <v>26.4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -5540,7 +5543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5554,7 +5557,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -5568,14 +5571,14 @@
         <v>65.400000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>140</v>
       </c>
@@ -5586,7 +5589,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>143</v>
@@ -5595,7 +5598,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
         <v>144</v>
@@ -5604,7 +5607,7 @@
         <v>19.100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
         <v>145</v>
@@ -5613,7 +5616,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
         <v>146</v>
@@ -5622,12 +5625,12 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>141</v>
       </c>
@@ -5638,7 +5641,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
         <v>148</v>
@@ -5647,7 +5650,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
         <v>145</v>
@@ -5656,7 +5659,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
         <v>144</v>
@@ -5665,7 +5668,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -5682,26 +5685,26 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -5719,7 +5722,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -5739,7 +5742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -5759,7 +5762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -5779,12 +5782,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C7" s="5">
         <v>74</v>
@@ -5799,7 +5802,7 @@
         <v>77.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -5819,7 +5822,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -5839,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>2</v>
       </c>
@@ -5859,7 +5862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -5879,7 +5882,7 @@
         <v>57.4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -5899,7 +5902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>2</v>
       </c>
@@ -5919,7 +5922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -5939,7 +5942,7 @@
         <v>53.4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -5959,7 +5962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -5979,7 +5982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -5999,7 +6002,7 @@
         <v>35.4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -6019,7 +6022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -6039,7 +6042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -6059,7 +6062,7 @@
         <v>49.1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -6079,7 +6082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -6099,12 +6102,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C23" s="5">
         <v>35</v>
@@ -6119,14 +6122,14 @@
         <v>59.4</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="25" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>160</v>
       </c>
@@ -6137,7 +6140,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
         <v>164</v>
@@ -6146,12 +6149,12 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>161</v>
       </c>
@@ -6162,12 +6165,12 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
       <c r="B33" s="1"/>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>162</v>
       </c>
@@ -6178,7 +6181,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>172</v>
@@ -6187,7 +6190,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>173</v>
@@ -6196,12 +6199,12 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="1"/>
       <c r="C37" s="8"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>163</v>
       </c>
@@ -6212,7 +6215,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -6229,24 +6232,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
   <dimension ref="A2:D70"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" customWidth="1"/>
-    <col min="2" max="2" width="22.69140625" customWidth="1"/>
-    <col min="3" max="4" width="9.53515625" customWidth="1"/>
-    <col min="5" max="5" width="9.3828125" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2" s="25" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="27"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
         <v>1</v>
@@ -6258,7 +6261,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -6272,7 +6275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6286,7 +6289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -6300,7 +6303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -6314,7 +6317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -6328,7 +6331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -6342,7 +6345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -6356,7 +6359,7 @@
         <v>97.9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -6370,7 +6373,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6384,7 +6387,7 @@
         <v>50.9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -6398,7 +6401,7 @@
         <v>56.9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6412,7 +6415,7 @@
         <v>104.9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -6426,7 +6429,7 @@
         <v>94.9</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -6440,7 +6443,7 @@
         <v>113.9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -6454,7 +6457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -6468,7 +6471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -6482,7 +6485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -6496,7 +6499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -6510,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -6524,7 +6527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -6538,7 +6541,7 @@
         <v>109.9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -6552,7 +6555,7 @@
         <v>105.9</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
@@ -6566,7 +6569,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -6580,7 +6583,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -6594,7 +6597,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>20</v>
       </c>
@@ -6608,7 +6611,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -6622,7 +6625,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -6636,7 +6639,7 @@
         <v>81.900000000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
@@ -6650,7 +6653,7 @@
         <v>77.900000000000006</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>20</v>
       </c>
@@ -6664,7 +6667,7 @@
         <v>84.9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -6678,7 +6681,7 @@
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
@@ -6692,7 +6695,7 @@
         <v>105.1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>20</v>
       </c>
@@ -6706,7 +6709,7 @@
         <v>101.1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -6720,12 +6723,12 @@
         <v>97.1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C37" s="5">
         <v>71.2</v>
@@ -6734,31 +6737,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C38" s="5">
         <v>67.2</v>
       </c>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C39" s="5">
         <v>67.599999999999994</v>
       </c>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>20</v>
       </c>
@@ -6772,7 +6775,7 @@
         <v>88.3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -6786,7 +6789,7 @@
         <v>56.3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
@@ -6800,7 +6803,7 @@
         <v>54.3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>20</v>
       </c>
@@ -6814,7 +6817,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -6828,12 +6831,12 @@
         <v>103.3</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C45" s="5">
         <v>65.8</v>
@@ -6842,12 +6845,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C46" s="5">
         <v>76.8</v>
@@ -6856,12 +6859,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C47" s="5">
         <v>62</v>
@@ -6870,12 +6873,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C48" s="5">
         <v>80.400000000000006</v>
@@ -6884,12 +6887,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C49" s="5">
         <v>91.4</v>
@@ -6898,12 +6901,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C50" s="5">
         <v>76.599999999999994</v>
@@ -6912,12 +6915,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C51" s="5">
         <v>35</v>
@@ -6926,12 +6929,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C52" s="5">
         <v>46</v>
@@ -6940,12 +6943,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C53" s="5">
         <v>31.2</v>
@@ -6954,14 +6957,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="18" t="s">
         <v>28</v>
       </c>
       <c r="B56" s="19"/>
       <c r="C56" s="20"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
         <v>192</v>
       </c>
@@ -6972,7 +6975,7 @@
         <v>17.7</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
         <v>198</v>
@@ -6981,7 +6984,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3" t="s">
         <v>199</v>
@@ -6990,7 +6993,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3" t="s">
         <v>195</v>
@@ -6999,7 +7002,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3" t="s">
         <v>197</v>
@@ -7008,12 +7011,12 @@
         <v>21.2</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
         <v>193</v>
       </c>
@@ -7024,7 +7027,7 @@
         <v>22.9</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="12"/>
       <c r="B64" s="4" t="s">
         <v>201</v>
@@ -7033,7 +7036,7 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="12"/>
       <c r="B65" s="4" t="s">
         <v>200</v>
@@ -7042,7 +7045,7 @@
         <v>32.1</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="12"/>
       <c r="B66" s="4" t="s">
         <v>202</v>
@@ -7051,9 +7054,9 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add YSSY AKMIR STAR
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6708F3B4-6412-4E69-BDD4-D9CF33C4DA1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8A2E7F-002D-42CD-A1FB-7CDE2F4EC0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -3974,22 +3974,22 @@
         <v>377</v>
       </c>
       <c r="C4" s="5">
-        <v>67</v>
+        <v>55.9</v>
       </c>
       <c r="D4" s="5">
-        <v>105.4</v>
+        <v>94</v>
       </c>
       <c r="E4" s="5">
-        <v>91.6</v>
+        <v>79.900000000000006</v>
       </c>
       <c r="F4" s="5">
-        <v>96.9</v>
+        <v>83</v>
       </c>
       <c r="G4" s="5">
+        <v>82.4</v>
+      </c>
+      <c r="H4" s="5">
         <v>93.9</v>
-      </c>
-      <c r="H4" s="5">
-        <v>104.7</v>
       </c>
       <c r="J4" s="26" t="s">
         <v>52</v>
@@ -4140,6 +4140,11 @@
         <v>79.5</v>
       </c>
     </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+    </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>28</v>
@@ -4225,6 +4230,7 @@
     <mergeCell ref="J4:Q5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add YSWS flow data
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8A2E7F-002D-42CD-A1FB-7CDE2F4EC0A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF38C0F-95E5-4555-8AB9-044254C85A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="32670" windowHeight="20985" activeTab="2" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
     <sheet name="YSSY" sheetId="10" r:id="rId2"/>
-    <sheet name="YMHB" sheetId="11" r:id="rId3"/>
-    <sheet name="YMLT" sheetId="12" r:id="rId4"/>
-    <sheet name="YBBN" sheetId="13" r:id="rId5"/>
-    <sheet name="YBCG" sheetId="14" r:id="rId6"/>
-    <sheet name="YPDN" sheetId="15" r:id="rId7"/>
-    <sheet name="YPPH" sheetId="16" r:id="rId8"/>
-    <sheet name="YBCS" sheetId="17" r:id="rId9"/>
-    <sheet name="YBTL" sheetId="18" r:id="rId10"/>
-    <sheet name="YWLM" sheetId="19" r:id="rId11"/>
-    <sheet name="YPAD" sheetId="20" r:id="rId12"/>
-    <sheet name="YMML" sheetId="21" r:id="rId13"/>
+    <sheet name="YSWS" sheetId="22" r:id="rId3"/>
+    <sheet name="YMHB" sheetId="11" r:id="rId4"/>
+    <sheet name="YMLT" sheetId="12" r:id="rId5"/>
+    <sheet name="YBBN" sheetId="13" r:id="rId6"/>
+    <sheet name="YBCG" sheetId="14" r:id="rId7"/>
+    <sheet name="YPDN" sheetId="15" r:id="rId8"/>
+    <sheet name="YPPH" sheetId="16" r:id="rId9"/>
+    <sheet name="YBCS" sheetId="17" r:id="rId10"/>
+    <sheet name="YBTL" sheetId="18" r:id="rId11"/>
+    <sheet name="YWLM" sheetId="19" r:id="rId12"/>
+    <sheet name="YPAD" sheetId="20" r:id="rId13"/>
+    <sheet name="YMML" sheetId="21" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="FFs">#REF!</definedName>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="395">
   <si>
     <t>-</t>
   </si>
@@ -1188,6 +1189,57 @@
   </si>
   <si>
     <t>AKMIR</t>
+  </si>
+  <si>
+    <t>ENROK (ILS)</t>
+  </si>
+  <si>
+    <t>PIBIX (RNP X)</t>
+  </si>
+  <si>
+    <t>PIBIX (ILS/RNP Z)</t>
+  </si>
+  <si>
+    <t>NUGSO (RNP X)</t>
+  </si>
+  <si>
+    <t>GUSDO (ILS/RNP Z)</t>
+  </si>
+  <si>
+    <t>NUGSO (ILS/RNP Z)</t>
+  </si>
+  <si>
+    <t>BIKUS A</t>
+  </si>
+  <si>
+    <t>REVKI A</t>
+  </si>
+  <si>
+    <t>REVKI N</t>
+  </si>
+  <si>
+    <t>UNTAV B</t>
+  </si>
+  <si>
+    <t>UNTAV N</t>
+  </si>
+  <si>
+    <t>UNTAV Q</t>
+  </si>
+  <si>
+    <t>GODUK N</t>
+  </si>
+  <si>
+    <t>UNTAV A</t>
+  </si>
+  <si>
+    <t>All aircraft assumed to be tracking via the ILS</t>
+  </si>
+  <si>
+    <t>Both REVKI STARs can be presented as a single option, for obvious reasons</t>
+  </si>
+  <si>
+    <t>RIKNI N (MARLN FF)</t>
   </si>
 </sst>
 </file>
@@ -2077,6 +2129,845 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
+  <dimension ref="A2:D70"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="5">
+        <v>58.1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C5" s="5">
+        <v>51.1</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="5">
+        <v>52.1</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C7" s="5">
+        <v>52.1</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C8" s="5">
+        <v>61.1</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C9" s="5">
+        <v>57.1</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5">
+        <v>97.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5">
+        <v>48.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <v>50.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>94.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5">
+        <v>113.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C17" s="5">
+        <v>63</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C18" s="5">
+        <v>55</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C19" s="5">
+        <v>51</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C20" s="5">
+        <v>58</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C21" s="5">
+        <v>66</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C22" s="5">
+        <v>51</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <v>109.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <v>105.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <v>101.9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5">
+        <v>81.900000000000006</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5">
+        <v>77.900000000000006</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5">
+        <v>84.9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5">
+        <v>73.900000000000006</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5">
+        <v>105.1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5">
+        <v>101.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5">
+        <v>97.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C37" s="5">
+        <v>71.2</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C38" s="5">
+        <v>67.2</v>
+      </c>
+      <c r="D38" s="5"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C39" s="5">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="D39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D40" s="5">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5">
+        <v>56.3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D42" s="5">
+        <v>54.3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="5">
+        <v>85.3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D44" s="5">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C45" s="5">
+        <v>65.8</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C46" s="5">
+        <v>76.8</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C47" s="5">
+        <v>62</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="C48" s="5">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C49" s="5">
+        <v>91.4</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C50" s="5">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C51" s="5">
+        <v>35</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C53" s="5">
+        <v>31.2</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B56" s="19"/>
+      <c r="C56" s="20"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C57" s="6">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="3"/>
+      <c r="B58" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C58" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C59" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C60" s="6">
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C61" s="6">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C63" s="7">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="12"/>
+      <c r="B64" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C64" s="7">
+        <v>18.899999999999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="12"/>
+      <c r="B65" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C65" s="7">
+        <v>32.1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="12"/>
+      <c r="B66" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C66" s="7">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>310</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B423E42B-58C3-4048-B6AA-4A2777AA66C2}">
   <dimension ref="A2:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2355,7 +3246,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49864E6F-5D2D-438C-A891-0771B0E2C7F9}">
   <dimension ref="A2:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2745,7 +3636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
   <dimension ref="A2:J61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3751,7 +4642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB965F8-E493-4C2F-8F83-E7C5A76D760C}">
   <dimension ref="A2:I42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4235,6 +5126,284 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F113EEA-A593-4575-858C-D276517D9617}">
+  <dimension ref="A2:Q42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C4" s="5">
+        <v>90.5</v>
+      </c>
+      <c r="D4" s="5">
+        <v>84</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>393</v>
+      </c>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C5" s="5">
+        <v>41.7</v>
+      </c>
+      <c r="D5" s="5">
+        <v>61</v>
+      </c>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="26"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="C6" s="5">
+        <v>41.7</v>
+      </c>
+      <c r="D6" s="5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="C7" s="5">
+        <v>103.7</v>
+      </c>
+      <c r="D7" s="5">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C8" s="5">
+        <v>80.5</v>
+      </c>
+      <c r="D8" s="5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C9" s="5">
+        <v>70.5</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J9" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" s="5">
+        <v>74.7</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="26"/>
+      <c r="P10" s="26"/>
+      <c r="Q10" s="26"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C11" s="5">
+        <v>77.7</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C20" s="6">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="11"/>
+      <c r="B21" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C21" s="6">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="11"/>
+      <c r="B22" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C22" s="6">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="8"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="C24" s="7">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="C25" s="7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="12"/>
+      <c r="B26" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C26" s="7">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>376</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="J4:Q5"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="J9:Q10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF2F9C14-24DD-4346-BD0F-4973CA74E2F8}">
   <dimension ref="A2:Q42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4429,7 +5598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBAE287-0B90-4E49-92A2-65E7CB2082F2}">
   <dimension ref="A2:Q42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4624,7 +5793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356EE3A2-5767-4B87-B203-C715848F2C44}">
   <dimension ref="A2:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5229,7 +6398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FA1FB4-B707-4F2A-8FE0-62699825C7A5}">
   <dimension ref="A2:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5461,7 +6630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D573D47-E01B-4687-B4AA-3BC4439FCCB5}">
   <dimension ref="A2:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5688,7 +6857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640AF1F2-4AB1-40AD-84F9-7D254EF129F1}">
   <dimension ref="A2:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6233,843 +7402,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CC78CC-1C97-417D-A9DE-26F33EC1DEB1}">
-  <dimension ref="A2:D70"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="C4" s="5">
-        <v>58.1</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C5" s="5">
-        <v>51.1</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="C6" s="5">
-        <v>52.1</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C7" s="5">
-        <v>52.1</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C8" s="5">
-        <v>61.1</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C9" s="5">
-        <v>57.1</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5">
-        <v>97.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5">
-        <v>48.9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D12" s="5">
-        <v>50.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5">
-        <v>56.9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5">
-        <v>104.9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5">
-        <v>94.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5">
-        <v>113.9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C17" s="5">
-        <v>63</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="C18" s="5">
-        <v>55</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C19" s="5">
-        <v>51</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="C20" s="5">
-        <v>58</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="5">
-        <v>66</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="C22" s="5">
-        <v>51</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="5">
-        <v>109.9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D24" s="5">
-        <v>105.9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D25" s="5">
-        <v>101.9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="5">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D28" s="5">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D29" s="5">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D30" s="5">
-        <v>81.900000000000006</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="5">
-        <v>77.900000000000006</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" s="5">
-        <v>84.9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D33" s="5">
-        <v>73.900000000000006</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" s="5">
-        <v>105.1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D35" s="5">
-        <v>101.1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D36" s="5">
-        <v>97.1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="C37" s="5">
-        <v>71.2</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="C38" s="5">
-        <v>67.2</v>
-      </c>
-      <c r="D38" s="5"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="C39" s="5">
-        <v>67.599999999999994</v>
-      </c>
-      <c r="D39" s="5"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D40" s="5">
-        <v>88.3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D41" s="5">
-        <v>56.3</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D42" s="5">
-        <v>54.3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D43" s="5">
-        <v>85.3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D44" s="5">
-        <v>103.3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C45" s="5">
-        <v>65.8</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="C46" s="5">
-        <v>76.8</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C47" s="5">
-        <v>62</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="C48" s="5">
-        <v>80.400000000000006</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C49" s="5">
-        <v>91.4</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C50" s="5">
-        <v>76.599999999999994</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C51" s="5">
-        <v>35</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="C52" s="5">
-        <v>46</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="C53" s="5">
-        <v>31.2</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B56" s="19"/>
-      <c r="C56" s="20"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="C57" s="6">
-        <v>17.7</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C58" s="6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="C59" s="6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="C60" s="6">
-        <v>20.399999999999999</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="C61" s="6">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C63" s="7">
-        <v>22.9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="12"/>
-      <c r="B64" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C64" s="7">
-        <v>18.899999999999999</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="12"/>
-      <c r="B65" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C65" s="7">
-        <v>32.1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="12"/>
-      <c r="B66" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="C66" s="7">
-        <v>25.3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>310</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Change YSSY RIVET FF to ENLAD
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF38C0F-95E5-4555-8AB9-044254C85A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA30EA16-BA98-4A71-B99B-AC52DC2B2B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="32670" windowHeight="20985" activeTab="2" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="396">
   <si>
     <t>-</t>
   </si>
@@ -150,9 +150,6 @@
     <t>MARLN</t>
   </si>
   <si>
-    <t>RIVET</t>
-  </si>
-  <si>
     <t>BOREE A</t>
   </si>
   <si>
@@ -1240,6 +1237,12 @@
   </si>
   <si>
     <t>RIKNI N (MARLN FF)</t>
+  </si>
+  <si>
+    <t>Last edit 4th May 2026 on DAP 187</t>
+  </si>
+  <si>
+    <t>RIVET (ENLAD FF)</t>
   </si>
 </sst>
 </file>
@@ -2116,7 +2119,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2154,10 +2157,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2165,7 +2168,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C4" s="5">
         <v>58.1</v>
@@ -2179,7 +2182,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C5" s="5">
         <v>51.1</v>
@@ -2193,7 +2196,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C6" s="5">
         <v>52.1</v>
@@ -2207,7 +2210,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C7" s="5">
         <v>52.1</v>
@@ -2221,7 +2224,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C8" s="5">
         <v>61.1</v>
@@ -2235,7 +2238,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C9" s="5">
         <v>57.1</v>
@@ -2249,7 +2252,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -2263,7 +2266,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>0</v>
@@ -2277,7 +2280,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -2291,7 +2294,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>0</v>
@@ -2305,7 +2308,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -2319,7 +2322,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>0</v>
@@ -2333,7 +2336,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>0</v>
@@ -2347,7 +2350,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C17" s="5">
         <v>63</v>
@@ -2361,7 +2364,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C18" s="5">
         <v>55</v>
@@ -2375,7 +2378,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C19" s="5">
         <v>51</v>
@@ -2389,7 +2392,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C20" s="5">
         <v>58</v>
@@ -2403,7 +2406,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C21" s="5">
         <v>66</v>
@@ -2417,7 +2420,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C22" s="5">
         <v>51</v>
@@ -2431,7 +2434,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>0</v>
@@ -2445,7 +2448,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>0</v>
@@ -2459,7 +2462,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>0</v>
@@ -2473,7 +2476,7 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>0</v>
@@ -2487,7 +2490,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>0</v>
@@ -2501,7 +2504,7 @@
         <v>20</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>0</v>
@@ -2515,7 +2518,7 @@
         <v>20</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>0</v>
@@ -2529,7 +2532,7 @@
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>0</v>
@@ -2543,7 +2546,7 @@
         <v>20</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>0</v>
@@ -2557,7 +2560,7 @@
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -2571,7 +2574,7 @@
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>0</v>
@@ -2585,7 +2588,7 @@
         <v>20</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>0</v>
@@ -2599,7 +2602,7 @@
         <v>20</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>0</v>
@@ -2613,7 +2616,7 @@
         <v>20</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>0</v>
@@ -2627,7 +2630,7 @@
         <v>20</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C37" s="5">
         <v>71.2</v>
@@ -2641,7 +2644,7 @@
         <v>20</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C38" s="5">
         <v>67.2</v>
@@ -2653,7 +2656,7 @@
         <v>20</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C39" s="5">
         <v>67.599999999999994</v>
@@ -2665,7 +2668,7 @@
         <v>20</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>0</v>
@@ -2679,7 +2682,7 @@
         <v>20</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>0</v>
@@ -2693,7 +2696,7 @@
         <v>20</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>0</v>
@@ -2707,7 +2710,7 @@
         <v>20</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>0</v>
@@ -2721,7 +2724,7 @@
         <v>20</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>0</v>
@@ -2735,7 +2738,7 @@
         <v>20</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C45" s="5">
         <v>65.8</v>
@@ -2749,7 +2752,7 @@
         <v>20</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C46" s="5">
         <v>76.8</v>
@@ -2763,7 +2766,7 @@
         <v>20</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C47" s="5">
         <v>62</v>
@@ -2777,7 +2780,7 @@
         <v>20</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C48" s="5">
         <v>80.400000000000006</v>
@@ -2791,7 +2794,7 @@
         <v>20</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C49" s="5">
         <v>91.4</v>
@@ -2805,7 +2808,7 @@
         <v>20</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C50" s="5">
         <v>76.599999999999994</v>
@@ -2819,7 +2822,7 @@
         <v>20</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C51" s="5">
         <v>35</v>
@@ -2833,7 +2836,7 @@
         <v>20</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C52" s="5">
         <v>46</v>
@@ -2847,7 +2850,7 @@
         <v>20</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C53" s="5">
         <v>31.2</v>
@@ -2865,10 +2868,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C57" s="6">
         <v>17.7</v>
@@ -2877,7 +2880,7 @@
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C58" s="6">
         <v>20</v>
@@ -2886,7 +2889,7 @@
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C59" s="6">
         <v>20</v>
@@ -2895,7 +2898,7 @@
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C60" s="6">
         <v>20.399999999999999</v>
@@ -2904,7 +2907,7 @@
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C61" s="6">
         <v>21.2</v>
@@ -2917,10 +2920,10 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>194</v>
       </c>
       <c r="C63" s="7">
         <v>22.9</v>
@@ -2929,7 +2932,7 @@
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="12"/>
       <c r="B64" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C64" s="7">
         <v>18.899999999999999</v>
@@ -2938,7 +2941,7 @@
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="12"/>
       <c r="B65" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C65" s="7">
         <v>32.1</v>
@@ -2947,7 +2950,7 @@
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="12"/>
       <c r="B66" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C66" s="7">
         <v>25.3</v>
@@ -2955,7 +2958,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -2993,10 +2996,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>244</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3004,7 +3007,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C4" s="5">
         <v>72.5</v>
@@ -3018,7 +3021,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>0</v>
@@ -3032,7 +3035,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C6" s="5">
         <v>58.2</v>
@@ -3046,7 +3049,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C7" s="5">
         <v>51.5</v>
@@ -3060,7 +3063,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -3074,7 +3077,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C9" s="5">
         <v>43.5</v>
@@ -3088,7 +3091,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -3102,7 +3105,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" s="5">
         <v>38.5</v>
@@ -3116,7 +3119,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -3130,7 +3133,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C13" s="5">
         <v>38.5</v>
@@ -3144,7 +3147,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -3162,10 +3165,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C29" s="6">
         <v>13.5</v>
@@ -3174,7 +3177,7 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C30" s="6">
         <v>19.3</v>
@@ -3183,7 +3186,7 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C31" s="6">
         <v>21.5</v>
@@ -3192,7 +3195,7 @@
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C32" s="6">
         <v>19.5</v>
@@ -3205,10 +3208,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C34" s="7">
         <v>15.5</v>
@@ -3217,7 +3220,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C35" s="7">
         <v>19.899999999999999</v>
@@ -3226,7 +3229,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C36" s="7">
         <v>24.5</v>
@@ -3234,7 +3237,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -3272,7 +3275,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -3283,7 +3286,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C4" s="5">
         <v>63.5</v>
@@ -3297,7 +3300,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C5" s="5">
         <v>48.5</v>
@@ -3311,7 +3314,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>0</v>
@@ -3320,7 +3323,7 @@
         <v>27.5</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G6" s="26"/>
       <c r="H6" s="26"/>
@@ -3335,7 +3338,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>0</v>
@@ -3357,7 +3360,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -3379,7 +3382,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -3401,7 +3404,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -3423,7 +3426,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>0</v>
@@ -3445,7 +3448,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C12" s="5">
         <v>31.5</v>
@@ -3459,7 +3462,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C13" s="5">
         <v>41.7</v>
@@ -3473,7 +3476,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C14" s="5">
         <v>28.6</v>
@@ -3487,7 +3490,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C15" s="5">
         <v>28.5</v>
@@ -3501,7 +3504,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C16" s="5">
         <v>44.5</v>
@@ -3515,7 +3518,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C17" s="5">
         <v>34.5</v>
@@ -3533,10 +3536,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C29" s="6">
         <v>12.7</v>
@@ -3545,7 +3548,7 @@
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C30" s="6">
         <v>16.5</v>
@@ -3554,7 +3557,7 @@
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C31" s="6">
         <v>16.5</v>
@@ -3563,7 +3566,7 @@
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C32" s="6">
         <v>9.6</v>
@@ -3576,10 +3579,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C34" s="7">
         <v>21</v>
@@ -3588,7 +3591,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C35" s="7">
         <v>20.9</v>
@@ -3597,7 +3600,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C36" s="7">
         <v>14.1</v>
@@ -3606,7 +3609,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C37" s="7">
         <v>14.8</v>
@@ -3615,7 +3618,7 @@
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C38" s="7">
         <v>9.5</v>
@@ -3623,7 +3626,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -3661,16 +3664,16 @@
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>299</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>300</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>5</v>
@@ -3681,7 +3684,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C4" s="5">
         <v>51.8</v>
@@ -3701,7 +3704,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C5" s="5">
         <v>49</v>
@@ -3721,7 +3724,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C6" s="5">
         <v>48.8</v>
@@ -3741,7 +3744,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C7" s="6">
         <v>55</v>
@@ -3761,7 +3764,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>0</v>
@@ -3781,7 +3784,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C9" s="6">
         <v>54</v>
@@ -3802,7 +3805,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C10" s="6">
         <v>76.900000000000006</v>
@@ -3822,7 +3825,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C11" s="5">
         <v>62.8</v>
@@ -3842,7 +3845,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C12" s="5">
         <v>67.8</v>
@@ -3862,7 +3865,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C13" s="5">
         <v>57.8</v>
@@ -3882,7 +3885,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C14" s="5">
         <v>59</v>
@@ -3902,7 +3905,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C15" s="5">
         <v>64</v>
@@ -3922,7 +3925,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C16" s="5">
         <v>54</v>
@@ -3942,7 +3945,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C17" s="5">
         <v>58.8</v>
@@ -3962,7 +3965,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C18" s="5">
         <v>63.8</v>
@@ -3982,7 +3985,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C19" s="5">
         <v>53.8</v>
@@ -4002,7 +4005,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>0</v>
@@ -4022,7 +4025,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>0</v>
@@ -4042,7 +4045,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C22" s="6">
         <v>37</v>
@@ -4062,7 +4065,7 @@
         <v>3</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C23" s="6">
         <v>47</v>
@@ -4082,7 +4085,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C24" s="5">
         <v>57</v>
@@ -4102,7 +4105,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C25" s="5">
         <v>58.8</v>
@@ -4122,7 +4125,7 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C26" s="5">
         <v>67.8</v>
@@ -4142,7 +4145,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C27" s="5">
         <v>64</v>
@@ -4162,7 +4165,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C28" s="6">
         <v>51</v>
@@ -4182,7 +4185,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C29" s="6">
         <v>46</v>
@@ -4202,7 +4205,7 @@
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>0</v>
@@ -4222,7 +4225,7 @@
         <v>20</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>0</v>
@@ -4242,7 +4245,7 @@
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -4262,7 +4265,7 @@
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>0</v>
@@ -4282,7 +4285,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C34" s="6">
         <v>48.5</v>
@@ -4302,7 +4305,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>0</v>
@@ -4322,7 +4325,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C36" s="6">
         <v>50</v>
@@ -4342,7 +4345,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C37" s="6">
         <v>47.4</v>
@@ -4362,7 +4365,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C38" s="6">
         <v>51.6</v>
@@ -4382,7 +4385,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>0</v>
@@ -4402,7 +4405,7 @@
         <v>3</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C40" s="6">
         <v>56</v>
@@ -4422,7 +4425,7 @@
         <v>3</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C41" s="6">
         <v>46</v>
@@ -4442,7 +4445,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>0</v>
@@ -4462,7 +4465,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>0</v>
@@ -4482,7 +4485,7 @@
         <v>3</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C44" s="6">
         <v>35.799999999999997</v>
@@ -4502,7 +4505,7 @@
         <v>3</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>0</v>
@@ -4526,10 +4529,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C48" s="6">
         <v>14.8</v>
@@ -4538,7 +4541,7 @@
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C49" s="6">
         <v>15.8</v>
@@ -4547,7 +4550,7 @@
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C50" s="6">
         <v>6.5</v>
@@ -4556,7 +4559,7 @@
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C51" s="6">
         <v>9.4</v>
@@ -4565,7 +4568,7 @@
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C52" s="6">
         <v>9.8000000000000007</v>
@@ -4578,10 +4581,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C54" s="7">
         <v>14.2</v>
@@ -4590,7 +4593,7 @@
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="12"/>
       <c r="B55" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C55" s="7">
         <v>18.7</v>
@@ -4603,10 +4606,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C57" s="5">
         <v>18.5</v>
@@ -4619,10 +4622,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B59" s="23" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C59" s="24">
         <v>14.3</v>
@@ -4630,7 +4633,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -4667,19 +4670,19 @@
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>362</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4687,7 +4690,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C4" s="5">
         <v>55.7</v>
@@ -4707,7 +4710,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C5" s="5">
         <v>59.7</v>
@@ -4727,7 +4730,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C6" s="5">
         <v>40</v>
@@ -4744,7 +4747,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -4756,10 +4759,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C29" s="8">
         <v>10.7</v>
@@ -4767,10 +4770,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C30" s="8">
         <v>11.8</v>
@@ -4778,10 +4781,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C31" s="8">
         <v>8.6999999999999993</v>
@@ -4789,10 +4792,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C32" s="8">
         <v>9</v>
@@ -4800,7 +4803,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -4839,22 +4842,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>50</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -4862,7 +4865,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C4" s="5">
         <v>55.9</v>
@@ -4883,7 +4886,7 @@
         <v>93.9</v>
       </c>
       <c r="J4" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K4" s="26"/>
       <c r="L4" s="26"/>
@@ -4898,7 +4901,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C5" s="5">
         <v>64.099999999999994</v>
@@ -4932,7 +4935,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>0</v>
@@ -4958,7 +4961,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C7" s="5">
         <v>67.2</v>
@@ -5010,25 +5013,25 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>395</v>
       </c>
       <c r="C9" s="5">
-        <v>42.6</v>
+        <v>55.4</v>
       </c>
       <c r="D9" s="5">
-        <v>79.599999999999994</v>
+        <v>92.4</v>
       </c>
       <c r="E9" s="5">
-        <v>67.3</v>
+        <v>80.099999999999994</v>
       </c>
       <c r="F9" s="5">
-        <v>70.099999999999994</v>
+        <v>82.9</v>
       </c>
       <c r="G9" s="5">
-        <v>63.9</v>
+        <v>76.7</v>
       </c>
       <c r="H9" s="5">
-        <v>79.5</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -5045,10 +5048,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" s="8">
         <v>9.9</v>
@@ -5056,10 +5059,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="8">
         <v>11.4</v>
@@ -5067,10 +5070,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="8">
         <v>14.5</v>
@@ -5078,10 +5081,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C23" s="8">
         <v>10</v>
@@ -5089,10 +5092,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C24" s="8">
         <v>12.9</v>
@@ -5100,10 +5103,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C25" s="8">
         <v>13</v>
@@ -5111,7 +5114,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -5148,10 +5151,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>299</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -5159,7 +5162,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C4" s="5">
         <v>90.5</v>
@@ -5168,7 +5171,7 @@
         <v>84</v>
       </c>
       <c r="J4" s="26" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="K4" s="26"/>
       <c r="L4" s="26"/>
@@ -5183,7 +5186,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C5" s="5">
         <v>41.7</v>
@@ -5205,7 +5208,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C6" s="5">
         <v>41.7</v>
@@ -5219,7 +5222,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C7" s="5">
         <v>103.7</v>
@@ -5233,7 +5236,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C8" s="5">
         <v>80.5</v>
@@ -5247,7 +5250,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C9" s="5">
         <v>70.5</v>
@@ -5256,7 +5259,7 @@
         <v>0</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
@@ -5271,7 +5274,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C10" s="5">
         <v>74.7</v>
@@ -5293,7 +5296,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C11" s="5">
         <v>77.7</v>
@@ -5307,7 +5310,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -5325,10 +5328,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C20" s="6">
         <v>13.7</v>
@@ -5337,7 +5340,7 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C21" s="6">
         <v>30.5</v>
@@ -5346,7 +5349,7 @@
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="B22" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C22" s="6">
         <v>22.3</v>
@@ -5359,10 +5362,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C24" s="7">
         <v>9.1999999999999993</v>
@@ -5371,7 +5374,7 @@
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
       <c r="B25" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C25" s="7">
         <v>15</v>
@@ -5380,7 +5383,7 @@
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C26" s="7">
         <v>13.4</v>
@@ -5388,7 +5391,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -5426,7 +5429,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -5437,7 +5440,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C4" s="5">
         <v>46.9</v>
@@ -5459,7 +5462,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="5">
         <v>36</v>
@@ -5481,7 +5484,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="5">
         <v>35.9</v>
@@ -5495,7 +5498,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" s="5">
         <v>45.9</v>
@@ -5509,7 +5512,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>0</v>
@@ -5523,7 +5526,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -5541,10 +5544,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="C20" s="6">
         <v>16.899999999999999</v>
@@ -5553,7 +5556,7 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C21" s="6">
         <v>14.9</v>
@@ -5566,10 +5569,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>58</v>
       </c>
       <c r="C23" s="7">
         <v>10.4</v>
@@ -5578,7 +5581,7 @@
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C24" s="7">
         <v>11.7</v>
@@ -5586,7 +5589,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -5618,13 +5621,13 @@
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -5632,7 +5635,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C4" s="5">
         <v>43.3</v>
@@ -5654,7 +5657,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>0</v>
@@ -5676,7 +5679,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" s="5">
         <v>65</v>
@@ -5690,7 +5693,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>0</v>
@@ -5704,7 +5707,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C8" s="5">
         <v>64.8</v>
@@ -5718,7 +5721,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -5736,10 +5739,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C20" s="6">
         <v>15</v>
@@ -5748,7 +5751,7 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C21" s="6">
         <v>17</v>
@@ -5761,10 +5764,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C23" s="7">
         <v>18.2</v>
@@ -5773,7 +5776,7 @@
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" s="7">
         <v>17.2</v>
@@ -5781,7 +5784,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -5821,16 +5824,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>83</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -5838,7 +5841,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" s="5">
         <v>55.5</v>
@@ -5858,7 +5861,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>0</v>
@@ -5878,7 +5881,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C6" s="5">
         <v>44.5</v>
@@ -5898,7 +5901,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>0</v>
@@ -5918,7 +5921,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C8" s="5">
         <v>58.5</v>
@@ -5938,7 +5941,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -5958,7 +5961,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
@@ -5978,7 +5981,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>0</v>
@@ -5998,7 +6001,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -6018,7 +6021,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>0</v>
@@ -6038,7 +6041,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>0</v>
@@ -6058,7 +6061,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C15" s="5">
         <v>70.5</v>
@@ -6078,7 +6081,7 @@
         <v>20</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C16" s="5">
         <v>51.3</v>
@@ -6098,7 +6101,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C17" s="5">
         <v>64.5</v>
@@ -6118,7 +6121,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>0</v>
@@ -6138,7 +6141,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C19" s="5">
         <v>51.5</v>
@@ -6158,7 +6161,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C20" s="5">
         <v>81.5</v>
@@ -6178,7 +6181,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>0</v>
@@ -6198,7 +6201,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C22" s="5">
         <v>65.5</v>
@@ -6218,7 +6221,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>0</v>
@@ -6238,7 +6241,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C24" s="5">
         <v>59.5</v>
@@ -6258,7 +6261,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C25" s="5">
         <v>44.3</v>
@@ -6282,10 +6285,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C29" s="6">
         <v>14.5</v>
@@ -6294,7 +6297,7 @@
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C30" s="6">
         <v>14.5</v>
@@ -6307,10 +6310,10 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="7">
         <v>9.5</v>
@@ -6319,7 +6322,7 @@
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C33" s="7">
         <v>9.6</v>
@@ -6328,7 +6331,7 @@
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C34" s="7">
         <v>11.7</v>
@@ -6341,10 +6344,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C36" s="17">
         <v>12.8</v>
@@ -6353,7 +6356,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C37" s="17">
         <v>14.5</v>
@@ -6366,10 +6369,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C39" s="5">
         <v>11.3</v>
@@ -6378,7 +6381,7 @@
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C40" s="5">
         <v>11.4</v>
@@ -6386,7 +6389,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -6421,13 +6424,13 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -6435,7 +6438,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C4" s="5">
         <v>66.8</v>
@@ -6449,7 +6452,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C5" s="5">
         <v>58.4</v>
@@ -6463,7 +6466,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C6" s="5">
         <v>59.7</v>
@@ -6477,7 +6480,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C7" s="5">
         <v>55.8</v>
@@ -6491,7 +6494,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8" s="5">
         <v>49.7</v>
@@ -6505,7 +6508,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>0</v>
@@ -6519,7 +6522,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C10" s="5">
         <v>47.4</v>
@@ -6537,10 +6540,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" s="6">
         <v>13.5</v>
@@ -6549,7 +6552,7 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C30" s="6">
         <v>14.8</v>
@@ -6558,7 +6561,7 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C31" s="6">
         <v>14.7</v>
@@ -6567,7 +6570,7 @@
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" s="6">
         <v>10</v>
@@ -6576,7 +6579,7 @@
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C33" s="6">
         <v>9.4</v>
@@ -6589,10 +6592,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C35" s="7">
         <v>15.3</v>
@@ -6601,7 +6604,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C36" s="7">
         <v>15</v>
@@ -6610,7 +6613,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C37" s="7">
         <v>10.5</v>
@@ -6618,7 +6621,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -6656,10 +6659,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>150</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -6667,7 +6670,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C4" s="5">
         <v>48.4</v>
@@ -6681,7 +6684,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" s="5">
         <v>75.400000000000006</v>
@@ -6695,7 +6698,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C6" s="5">
         <v>55.4</v>
@@ -6709,7 +6712,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C7" s="5">
         <v>45.4</v>
@@ -6723,7 +6726,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C8" s="5">
         <v>67.400000000000006</v>
@@ -6737,7 +6740,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C9" s="5">
         <v>58.9</v>
@@ -6755,10 +6758,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C29" s="6">
         <v>15</v>
@@ -6767,7 +6770,7 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C30" s="6">
         <v>9.4</v>
@@ -6776,7 +6779,7 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C31" s="6">
         <v>19.100000000000001</v>
@@ -6785,7 +6788,7 @@
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C32" s="6">
         <v>20.399999999999999</v>
@@ -6794,7 +6797,7 @@
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C33" s="6">
         <v>18.899999999999999</v>
@@ -6807,10 +6810,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C35" s="7">
         <v>15.3</v>
@@ -6819,7 +6822,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C36" s="7">
         <v>9.4</v>
@@ -6828,7 +6831,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C37" s="7">
         <v>20.399999999999999</v>
@@ -6837,7 +6840,7 @@
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C38" s="7">
         <v>20.7</v>
@@ -6845,7 +6848,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -6885,16 +6888,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -6902,7 +6905,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C4" s="6">
         <v>47</v>
@@ -6922,7 +6925,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C5" s="6">
         <v>40</v>
@@ -6942,7 +6945,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C6" s="6">
         <v>38.299999999999997</v>
@@ -6962,7 +6965,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C7" s="5">
         <v>74</v>
@@ -6982,7 +6985,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C8" s="7">
         <v>78.599999999999994</v>
@@ -7002,7 +7005,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C9" s="7">
         <v>66</v>
@@ -7022,7 +7025,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C10" s="7">
         <v>64.3</v>
@@ -7042,7 +7045,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C11" s="7">
         <v>65</v>
@@ -7062,7 +7065,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C12" s="7">
         <v>55</v>
@@ -7082,7 +7085,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C13" s="7">
         <v>53.3</v>
@@ -7102,7 +7105,7 @@
         <v>3</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C14" s="6">
         <v>70</v>
@@ -7122,7 +7125,7 @@
         <v>3</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C15" s="6">
         <v>58</v>
@@ -7142,7 +7145,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C16" s="6">
         <v>56.3</v>
@@ -7162,7 +7165,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C17" s="6">
         <v>79</v>
@@ -7182,7 +7185,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C18" s="6">
         <v>66</v>
@@ -7202,7 +7205,7 @@
         <v>3</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C19" s="6">
         <v>64.3</v>
@@ -7222,7 +7225,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C20" s="5">
         <v>43</v>
@@ -7242,7 +7245,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C21" s="5">
         <v>40</v>
@@ -7262,7 +7265,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C22" s="5">
         <v>38.299999999999997</v>
@@ -7282,7 +7285,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C23" s="5">
         <v>35</v>
@@ -7306,10 +7309,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C29" s="6">
         <v>10</v>
@@ -7318,7 +7321,7 @@
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C30" s="6">
         <v>12.3</v>
@@ -7331,10 +7334,10 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C32" s="7">
         <v>9.1999999999999993</v>
@@ -7347,10 +7350,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C34" s="17">
         <v>8.1</v>
@@ -7359,7 +7362,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C35" s="17">
         <v>16.3</v>
@@ -7368,7 +7371,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C36" s="17">
         <v>13.1</v>
@@ -7381,10 +7384,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C38" s="5">
         <v>8.4</v>
@@ -7392,7 +7395,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ELROX6A/V STARs to YPAD
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA30EA16-BA98-4A71-B99B-AC52DC2B2B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9536665B-7940-45D1-B53D-BDE0944F00B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="12" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="398">
   <si>
     <t>-</t>
   </si>
@@ -1074,9 +1074,6 @@
     <t>KAKLU V/X STAR</t>
   </si>
   <si>
-    <t xml:space="preserve">Last edit 21st May 2025 on DAP 182 </t>
-  </si>
-  <si>
     <t>SURGN STAR - IAP (KAKLU FF)</t>
   </si>
   <si>
@@ -1243,6 +1240,15 @@
   </si>
   <si>
     <t>RIVET (ENLAD FF)</t>
+  </si>
+  <si>
+    <t>ELROX A STAR</t>
+  </si>
+  <si>
+    <t>ELROX Z STAR</t>
+  </si>
+  <si>
+    <t>Last edit 03rd Aug 2026 on DAP 188</t>
   </si>
 </sst>
 </file>
@@ -1380,7 +1386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1441,6 +1447,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3641,7 +3653,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB7F36C5-51BD-40E7-89E4-2CA7A521DEBF}">
-  <dimension ref="A2:J61"/>
+  <dimension ref="A2:J63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -3744,7 +3756,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C7" s="6">
         <v>55</v>
@@ -3764,7 +3776,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>0</v>
@@ -3784,7 +3796,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C9" s="6">
         <v>54</v>
@@ -3805,7 +3817,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C10" s="6">
         <v>76.900000000000006</v>
@@ -4041,22 +4053,22 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="C22" s="6">
-        <v>37</v>
-      </c>
-      <c r="D22" s="6">
-        <v>40</v>
-      </c>
-      <c r="E22" s="6">
-        <v>46</v>
-      </c>
-      <c r="F22" s="6" t="s">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="30">
+        <v>70.2</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>0</v>
       </c>
     </row>
@@ -4065,16 +4077,16 @@
         <v>3</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C23" s="6">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D23" s="6">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E23" s="6">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>0</v>
@@ -4085,38 +4097,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="C24" s="5">
-        <v>57</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="C24" s="30">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="D24" s="30">
+        <v>43.3</v>
+      </c>
+      <c r="E24" s="30">
+        <v>70.2</v>
+      </c>
+      <c r="F24" s="31" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="C25" s="5">
-        <v>58.8</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F25" s="5" t="s">
+      <c r="A25" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C25" s="6">
+        <v>47</v>
+      </c>
+      <c r="D25" s="6">
+        <v>45</v>
+      </c>
+      <c r="E25" s="6">
+        <v>50</v>
+      </c>
+      <c r="F25" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -4125,16 +4137,16 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="C26" s="5">
-        <v>67.8</v>
+        <v>57</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E26" s="5">
-        <v>47.2</v>
+      <c r="E26" s="5" t="s">
+        <v>0</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>0</v>
@@ -4145,98 +4157,98 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C27" s="5">
+        <v>58.8</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C28" s="5">
+        <v>67.8</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5">
+        <v>47.2</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C29" s="5">
         <v>64</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="D29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B30" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C30" s="6">
         <v>51</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D30" s="6">
         <v>45</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E30" s="6">
         <v>47</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="F30" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B31" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C31" s="6">
         <v>46</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D31" s="6">
         <v>40</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E31" s="6">
         <v>42</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E30" s="5">
-        <v>53.2</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E31" s="5">
-        <v>53.2</v>
-      </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -4245,7 +4257,7 @@
         <v>20</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>0</v>
@@ -4254,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="5">
-        <v>50</v>
+        <v>53.2</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>0</v>
@@ -4265,59 +4277,59 @@
         <v>20</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5">
+        <v>53.2</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5">
+        <v>50</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="E33" s="5">
+      <c r="C35" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5">
         <v>50</v>
       </c>
-      <c r="F33" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="C34" s="6">
-        <v>48.5</v>
-      </c>
-      <c r="D34" s="6">
-        <v>48.5</v>
-      </c>
-      <c r="E34" s="6">
-        <v>45</v>
-      </c>
-      <c r="F34" s="6">
-        <v>46.7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D35" s="6">
-        <v>65.900000000000006</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F35" s="6">
-        <v>51.5</v>
+      <c r="F35" s="5" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -4325,19 +4337,19 @@
         <v>3</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="C36" s="6">
-        <v>50</v>
+        <v>48.5</v>
       </c>
       <c r="D36" s="6">
-        <v>44.4</v>
+        <v>48.5</v>
       </c>
       <c r="E36" s="6">
-        <v>50.8</v>
+        <v>45</v>
       </c>
       <c r="F36" s="6">
-        <v>49</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -4345,19 +4357,19 @@
         <v>3</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="C37" s="6">
-        <v>47.4</v>
+        <v>339</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="D37" s="6">
-        <v>45</v>
-      </c>
-      <c r="E37" s="6">
-        <v>55</v>
+        <v>65.900000000000006</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="F37" s="6">
-        <v>49</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -4365,19 +4377,19 @@
         <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C38" s="6">
-        <v>51.6</v>
+        <v>50</v>
       </c>
       <c r="D38" s="6">
+        <v>44.4</v>
+      </c>
+      <c r="E38" s="6">
+        <v>50.8</v>
+      </c>
+      <c r="F38" s="6">
         <v>49</v>
-      </c>
-      <c r="E38" s="6">
-        <v>50</v>
-      </c>
-      <c r="F38" s="6">
-        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -4385,19 +4397,19 @@
         <v>3</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>0</v>
+        <v>346</v>
+      </c>
+      <c r="C39" s="6">
+        <v>47.4</v>
+      </c>
+      <c r="D39" s="6">
+        <v>45</v>
+      </c>
+      <c r="E39" s="6">
+        <v>55</v>
       </c>
       <c r="F39" s="6">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -4405,19 +4417,19 @@
         <v>3</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C40" s="6">
-        <v>56</v>
+        <v>51.6</v>
       </c>
       <c r="D40" s="6">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E40" s="6">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F40" s="6">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -4425,19 +4437,19 @@
         <v>3</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="C41" s="6">
-        <v>46</v>
-      </c>
-      <c r="D41" s="6">
-        <v>40</v>
-      </c>
-      <c r="E41" s="6">
-        <v>46</v>
+        <v>348</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="F41" s="6">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -4445,19 +4457,19 @@
         <v>3</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>0</v>
+        <v>349</v>
+      </c>
+      <c r="C42" s="6">
+        <v>56</v>
       </c>
       <c r="D42" s="6">
-        <v>44.8</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>0</v>
+        <v>46</v>
+      </c>
+      <c r="E42" s="6">
+        <v>46</v>
       </c>
       <c r="F42" s="6">
-        <v>78.099999999999994</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -4465,19 +4477,19 @@
         <v>3</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>353</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>0</v>
+        <v>350</v>
+      </c>
+      <c r="C43" s="6">
+        <v>46</v>
       </c>
       <c r="D43" s="6">
-        <v>45.6</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>0</v>
+        <v>40</v>
+      </c>
+      <c r="E43" s="6">
+        <v>46</v>
       </c>
       <c r="F43" s="6">
-        <v>77.8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -4485,19 +4497,19 @@
         <v>3</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="C44" s="6">
-        <v>35.799999999999997</v>
+        <v>351</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="D44" s="6">
-        <v>42.8</v>
-      </c>
-      <c r="E44" s="6">
-        <v>69.2</v>
+        <v>44.8</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="F44" s="6">
-        <v>60.2</v>
+        <v>78.099999999999994</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -4505,114 +4517,138 @@
         <v>3</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>0</v>
       </c>
       <c r="D45" s="6">
+        <v>45.6</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F45" s="6">
+        <v>77.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="C46" s="6">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="D46" s="6">
+        <v>42.8</v>
+      </c>
+      <c r="E46" s="6">
+        <v>69.2</v>
+      </c>
+      <c r="F46" s="6">
+        <v>60.2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D47" s="6">
         <v>41</v>
       </c>
-      <c r="E45" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F45" s="6">
+      <c r="E47" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F47" s="6">
         <v>72.8</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="27" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="28"/>
-      <c r="C47" s="29"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="11" t="s">
+      <c r="B49" s="28"/>
+      <c r="C49" s="29"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B50" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="C48" s="6">
+      <c r="C50" s="6">
         <v>14.8</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="C49" s="6">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="C50" s="6">
-        <v>6.5</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C51" s="6">
-        <v>9.4</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C52" s="6">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C53" s="6">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="3"/>
+      <c r="B54" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="C52" s="6">
+      <c r="C54" s="6">
         <v>9.8000000000000007</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="12" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B56" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="C54" s="7">
+      <c r="C56" s="7">
         <v>14.2</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="12"/>
-      <c r="B55" s="4" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="12"/>
+      <c r="B57" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="C55" s="7">
+      <c r="C57" s="7">
         <v>18.7</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="C57" s="5">
-        <v>18.5</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -4621,27 +4657,44 @@
       <c r="C58" s="1"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="22" t="s">
+      <c r="A59" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C59" s="5">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="1"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="B59" s="23" t="s">
-        <v>357</v>
-      </c>
-      <c r="C59" s="24">
+      <c r="B61" s="23" t="s">
+        <v>356</v>
+      </c>
+      <c r="C61" s="24">
         <v>14.3</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>339</v>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>397</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A49:C49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4673,16 +4726,16 @@
         <v>119</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>361</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4690,7 +4743,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C4" s="5">
         <v>55.7</v>
@@ -4710,7 +4763,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C5" s="5">
         <v>59.7</v>
@@ -4730,7 +4783,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C6" s="5">
         <v>40</v>
@@ -4747,7 +4800,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -4759,10 +4812,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C29" s="8">
         <v>10.7</v>
@@ -4770,10 +4823,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C30" s="8">
         <v>11.8</v>
@@ -4781,10 +4834,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C31" s="8">
         <v>8.6999999999999993</v>
@@ -4792,10 +4845,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C32" s="8">
         <v>9</v>
@@ -4865,7 +4918,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C4" s="5">
         <v>55.9</v>
@@ -5013,7 +5066,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C9" s="5">
         <v>55.4</v>
@@ -5114,7 +5167,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -5162,7 +5215,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C4" s="5">
         <v>90.5</v>
@@ -5171,7 +5224,7 @@
         <v>84</v>
       </c>
       <c r="J4" s="26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="K4" s="26"/>
       <c r="L4" s="26"/>
@@ -5186,7 +5239,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C5" s="5">
         <v>41.7</v>
@@ -5208,7 +5261,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C6" s="5">
         <v>41.7</v>
@@ -5222,7 +5275,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C7" s="5">
         <v>103.7</v>
@@ -5236,7 +5289,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C8" s="5">
         <v>80.5</v>
@@ -5250,7 +5303,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C9" s="5">
         <v>70.5</v>
@@ -5259,7 +5312,7 @@
         <v>0</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
@@ -5274,7 +5327,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C10" s="5">
         <v>74.7</v>
@@ -5296,7 +5349,7 @@
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C11" s="5">
         <v>77.7</v>
@@ -5310,7 +5363,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>0</v>
@@ -5331,7 +5384,7 @@
         <v>289</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C20" s="6">
         <v>13.7</v>
@@ -5340,7 +5393,7 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C21" s="6">
         <v>30.5</v>
@@ -5349,7 +5402,7 @@
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="B22" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C22" s="6">
         <v>22.3</v>
@@ -5365,7 +5418,7 @@
         <v>290</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C24" s="7">
         <v>9.1999999999999993</v>
@@ -5374,7 +5427,7 @@
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
       <c r="B25" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C25" s="7">
         <v>15</v>
@@ -5383,7 +5436,7 @@
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C26" s="7">
         <v>13.4</v>
@@ -5391,7 +5444,7 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -7285,7 +7338,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C23" s="5">
         <v>35</v>

</xml_diff>

<commit_message>
Finish adding ELROX STAR to YPAD
</commit_message>
<xml_diff>
--- a/flow-data/Flow Distances.xlsx
+++ b/flow-data/Flow Distances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Documents\GitHub\image-source-files\flow-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9536665B-7940-45D1-B53D-BDE0944F00B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB3E831-0E87-4B46-B6BB-5A5F323C1607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="12" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="12" xr2:uid="{929881EF-ACD6-4EB1-B094-42C9C0A4B466}"/>
   </bookViews>
   <sheets>
     <sheet name="YSCB" sheetId="9" r:id="rId1"/>
@@ -1386,7 +1386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1447,9 +1447,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4108,7 +4105,7 @@
       <c r="E24" s="30">
         <v>70.2</v>
       </c>
-      <c r="F24" s="31" t="s">
+      <c r="F24" s="30" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>